<commit_message>
Update organization roster with CSV-based personnel data
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1E0EAD2-8DB5-425D-A23F-BD0F99137BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{7379B17E-867F-4EBC-A110-47B53CC5822D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="376">
   <si>
     <t>order</t>
   </si>
@@ -1262,6 +1262,33 @@
   <dxfs count="26">
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -1357,111 +1384,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -1509,6 +1431,44 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
         <name val="Segoe UI"/>
         <family val="2"/>
         <scheme val="none"/>
@@ -1654,6 +1614,46 @@
         <scheme val="none"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1668,35 +1668,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:W71" headerRowDxfId="7" dataDxfId="8" totalsRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:W71" headerRowDxfId="25" dataDxfId="24" totalsRowDxfId="23">
   <tableColumns count="23">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="24"/>
-    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="22"/>
-    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="21">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="20"/>
+    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="18">
       <calculatedColumnFormula>IF(D2="","",LEFT(TRIM(D2),1)&amp;".")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="20"/>
-    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="19">
+    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="17"/>
+    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="16">
       <calculatedColumnFormula>TRIM(_xlfn.TEXTJOIN(" ",TRUE,C2,IF(E2&lt;&gt;"",IF(RIGHT(E2,1)=".",E2,E2&amp;"."),D2),B2,F2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="18"/>
-    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="17"/>
-    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="16"/>
-    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="5"/>
-    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="12"/>
-    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="0"/>
-    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="1"/>
-    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="15"/>
+    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="14"/>
+    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="13"/>
+    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="12"/>
+    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="11"/>
+    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="7"/>
+    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="6"/>
+    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="5"/>
+    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="4"/>
     <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="3"/>
-    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="11"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="10"/>
+    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1863,13 +1863,14 @@
     <col min="7" max="7" width="30.3984375" style="4" customWidth="1"/>
     <col min="8" max="8" width="23.5" style="4" customWidth="1"/>
     <col min="9" max="9" width="25.3984375" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="12" width="28" style="4" customWidth="1"/>
-    <col min="13" max="13" width="22.09765625" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31" style="4" customWidth="1"/>
+    <col min="11" max="12" width="28" style="4" customWidth="1"/>
+    <col min="13" max="13" width="32.8984375" style="4" customWidth="1"/>
     <col min="14" max="14" width="26.69921875" style="4" customWidth="1"/>
     <col min="15" max="15" width="20.09765625" style="4" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="45.19921875" style="7" customWidth="1"/>
     <col min="17" max="21" width="24.19921875" style="7" customWidth="1"/>
-    <col min="22" max="22" width="33.8984375" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="36.69921875" style="4" customWidth="1"/>
     <col min="23" max="23" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
     <col min="24" max="16384" width="8.796875" style="4"/>
   </cols>
@@ -2036,7 +2037,9 @@
         <v>17</v>
       </c>
       <c r="P3" s="6"/>
-      <c r="Q3" s="6"/>
+      <c r="Q3" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R3" s="6"/>
       <c r="S3" s="6"/>
       <c r="T3" s="6"/>
@@ -2136,7 +2139,9 @@
         <v>17</v>
       </c>
       <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
+      <c r="Q5" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R5" s="6"/>
       <c r="S5" s="6"/>
       <c r="T5" s="6"/>
@@ -2186,7 +2191,9 @@
         <v>14</v>
       </c>
       <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
+      <c r="Q6" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R6" s="6"/>
       <c r="S6" s="6"/>
       <c r="T6" s="6"/>
@@ -2236,7 +2243,9 @@
         <v>14</v>
       </c>
       <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
+      <c r="Q7" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R7" s="6"/>
       <c r="S7" s="6"/>
       <c r="T7" s="6"/>
@@ -2388,7 +2397,9 @@
         <v>14</v>
       </c>
       <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
+      <c r="Q10" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R10" s="6"/>
       <c r="S10" s="6"/>
       <c r="T10" s="6"/>
@@ -2438,7 +2449,9 @@
         <v>17</v>
       </c>
       <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
+      <c r="Q11" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R11" s="6"/>
       <c r="S11" s="6"/>
       <c r="T11" s="6"/>
@@ -2488,7 +2501,9 @@
         <v>17</v>
       </c>
       <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
+      <c r="Q12" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R12" s="6"/>
       <c r="S12" s="6"/>
       <c r="T12" s="6"/>
@@ -2588,7 +2603,9 @@
         <v>17</v>
       </c>
       <c r="P14" s="6"/>
-      <c r="Q14" s="6"/>
+      <c r="Q14" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R14" s="6"/>
       <c r="S14" s="6"/>
       <c r="T14" s="6"/>
@@ -2638,7 +2655,9 @@
         <v>14</v>
       </c>
       <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
+      <c r="Q15" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R15" s="6"/>
       <c r="S15" s="6"/>
       <c r="T15" s="6"/>
@@ -2686,7 +2705,9 @@
         <v>17</v>
       </c>
       <c r="P16" s="6"/>
-      <c r="Q16" s="6"/>
+      <c r="Q16" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R16" s="6"/>
       <c r="S16" s="6"/>
       <c r="T16" s="6"/>
@@ -2836,7 +2857,9 @@
         <v>14</v>
       </c>
       <c r="P19" s="6"/>
-      <c r="Q19" s="6"/>
+      <c r="Q19" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R19" s="6"/>
       <c r="S19" s="6"/>
       <c r="T19" s="6"/>
@@ -2938,7 +2961,9 @@
         <v>17</v>
       </c>
       <c r="P21" s="6"/>
-      <c r="Q21" s="6"/>
+      <c r="Q21" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R21" s="6"/>
       <c r="S21" s="6"/>
       <c r="T21" s="6"/>
@@ -2988,7 +3013,9 @@
         <v>17</v>
       </c>
       <c r="P22" s="6"/>
-      <c r="Q22" s="6"/>
+      <c r="Q22" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
       <c r="T22" s="6"/>
@@ -3038,7 +3065,9 @@
         <v>7</v>
       </c>
       <c r="P23" s="6"/>
-      <c r="Q23" s="6"/>
+      <c r="Q23" s="6" t="s">
+        <v>367</v>
+      </c>
       <c r="R23" s="6"/>
       <c r="S23" s="6"/>
       <c r="T23" s="6"/>
@@ -3088,7 +3117,9 @@
         <v>17</v>
       </c>
       <c r="P24" s="6"/>
-      <c r="Q24" s="6"/>
+      <c r="Q24" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R24" s="6"/>
       <c r="S24" s="6"/>
       <c r="T24" s="6"/>
@@ -3138,7 +3169,9 @@
         <v>17</v>
       </c>
       <c r="P25" s="6"/>
-      <c r="Q25" s="6"/>
+      <c r="Q25" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R25" s="6"/>
       <c r="S25" s="6"/>
       <c r="T25" s="6"/>
@@ -3188,7 +3221,9 @@
         <v>17</v>
       </c>
       <c r="P26" s="6"/>
-      <c r="Q26" s="6"/>
+      <c r="Q26" s="6" t="s">
+        <v>367</v>
+      </c>
       <c r="R26" s="6"/>
       <c r="S26" s="6"/>
       <c r="T26" s="6"/>
@@ -3236,7 +3271,9 @@
         <v>17</v>
       </c>
       <c r="P27" s="6"/>
-      <c r="Q27" s="6"/>
+      <c r="Q27" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R27" s="6"/>
       <c r="S27" s="6"/>
       <c r="T27" s="6"/>
@@ -3286,7 +3323,9 @@
         <v>17</v>
       </c>
       <c r="P28" s="6"/>
-      <c r="Q28" s="6"/>
+      <c r="Q28" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R28" s="6"/>
       <c r="S28" s="6"/>
       <c r="T28" s="6"/>
@@ -3338,7 +3377,9 @@
         <v>14</v>
       </c>
       <c r="P29" s="6"/>
-      <c r="Q29" s="6"/>
+      <c r="Q29" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R29" s="6"/>
       <c r="S29" s="6"/>
       <c r="T29" s="6"/>
@@ -3388,7 +3429,9 @@
         <v>17</v>
       </c>
       <c r="P30" s="6"/>
-      <c r="Q30" s="6"/>
+      <c r="Q30" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R30" s="6"/>
       <c r="S30" s="6"/>
       <c r="T30" s="6"/>
@@ -3438,7 +3481,9 @@
         <v>17</v>
       </c>
       <c r="P31" s="6"/>
-      <c r="Q31" s="6"/>
+      <c r="Q31" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R31" s="6"/>
       <c r="S31" s="6"/>
       <c r="T31" s="6"/>
@@ -3488,7 +3533,9 @@
         <v>14</v>
       </c>
       <c r="P32" s="6"/>
-      <c r="Q32" s="6"/>
+      <c r="Q32" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R32" s="6"/>
       <c r="S32" s="6"/>
       <c r="T32" s="6"/>
@@ -3538,7 +3585,9 @@
         <v>17</v>
       </c>
       <c r="P33" s="6"/>
-      <c r="Q33" s="6"/>
+      <c r="Q33" s="6" t="s">
+        <v>370</v>
+      </c>
       <c r="R33" s="6"/>
       <c r="S33" s="6"/>
       <c r="T33" s="6"/>
@@ -3588,7 +3637,9 @@
         <v>17</v>
       </c>
       <c r="P34" s="6"/>
-      <c r="Q34" s="6"/>
+      <c r="Q34" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R34" s="6"/>
       <c r="S34" s="6"/>
       <c r="T34" s="6"/>
@@ -3638,7 +3689,9 @@
         <v>17</v>
       </c>
       <c r="P35" s="6"/>
-      <c r="Q35" s="6"/>
+      <c r="Q35" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R35" s="6"/>
       <c r="S35" s="6"/>
       <c r="T35" s="6"/>
@@ -3688,7 +3741,9 @@
         <v>17</v>
       </c>
       <c r="P36" s="6"/>
-      <c r="Q36" s="6"/>
+      <c r="Q36" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R36" s="6"/>
       <c r="S36" s="6"/>
       <c r="T36" s="6"/>
@@ -3738,7 +3793,9 @@
         <v>17</v>
       </c>
       <c r="P37" s="6"/>
-      <c r="Q37" s="6"/>
+      <c r="Q37" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R37" s="6"/>
       <c r="S37" s="6"/>
       <c r="T37" s="6"/>
@@ -3788,7 +3845,9 @@
         <v>17</v>
       </c>
       <c r="P38" s="6"/>
-      <c r="Q38" s="6"/>
+      <c r="Q38" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R38" s="6"/>
       <c r="S38" s="6"/>
       <c r="T38" s="6"/>
@@ -3838,7 +3897,9 @@
         <v>17</v>
       </c>
       <c r="P39" s="6"/>
-      <c r="Q39" s="6"/>
+      <c r="Q39" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R39" s="6"/>
       <c r="S39" s="6"/>
       <c r="T39" s="6"/>
@@ -3888,7 +3949,9 @@
         <v>17</v>
       </c>
       <c r="P40" s="6"/>
-      <c r="Q40" s="6"/>
+      <c r="Q40" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R40" s="6"/>
       <c r="S40" s="6"/>
       <c r="T40" s="6"/>
@@ -3938,7 +4001,9 @@
         <v>17</v>
       </c>
       <c r="P41" s="6"/>
-      <c r="Q41" s="6"/>
+      <c r="Q41" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R41" s="6"/>
       <c r="S41" s="6"/>
       <c r="T41" s="6"/>
@@ -3986,7 +4051,9 @@
         <v>17</v>
       </c>
       <c r="P42" s="6"/>
-      <c r="Q42" s="6"/>
+      <c r="Q42" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R42" s="6"/>
       <c r="S42" s="6"/>
       <c r="T42" s="6"/>
@@ -4036,7 +4103,9 @@
         <v>14</v>
       </c>
       <c r="P43" s="6"/>
-      <c r="Q43" s="6"/>
+      <c r="Q43" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R43" s="6"/>
       <c r="S43" s="6"/>
       <c r="T43" s="6"/>
@@ -4049,7 +4118,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:23" ht="33.6">
+    <row r="44" spans="1:23">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -4072,7 +4141,7 @@
         <v>Richie Ryan C. Mabunay</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>12</v>
+        <v>250</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>291</v>
@@ -4094,7 +4163,9 @@
       <c r="P44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q44" s="6"/>
+      <c r="Q44" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R44" s="6"/>
       <c r="S44" s="6"/>
       <c r="T44" s="6"/>
@@ -4144,7 +4215,9 @@
         <v>17</v>
       </c>
       <c r="P45" s="6"/>
-      <c r="Q45" s="6"/>
+      <c r="Q45" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R45" s="6"/>
       <c r="S45" s="6"/>
       <c r="T45" s="6"/>
@@ -4194,7 +4267,9 @@
         <v>17</v>
       </c>
       <c r="P46" s="6"/>
-      <c r="Q46" s="6"/>
+      <c r="Q46" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R46" s="6"/>
       <c r="S46" s="6"/>
       <c r="T46" s="6"/>
@@ -4244,7 +4319,9 @@
         <v>17</v>
       </c>
       <c r="P47" s="6"/>
-      <c r="Q47" s="6"/>
+      <c r="Q47" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R47" s="6"/>
       <c r="S47" s="6"/>
       <c r="T47" s="6"/>
@@ -4294,7 +4371,9 @@
         <v>17</v>
       </c>
       <c r="P48" s="6"/>
-      <c r="Q48" s="6"/>
+      <c r="Q48" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R48" s="6"/>
       <c r="S48" s="6"/>
       <c r="T48" s="6"/>
@@ -4344,7 +4423,9 @@
         <v>17</v>
       </c>
       <c r="P49" s="6"/>
-      <c r="Q49" s="6"/>
+      <c r="Q49" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R49" s="6"/>
       <c r="S49" s="6"/>
       <c r="T49" s="6"/>
@@ -4394,7 +4475,9 @@
         <v>17</v>
       </c>
       <c r="P50" s="6"/>
-      <c r="Q50" s="6"/>
+      <c r="Q50" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R50" s="6"/>
       <c r="S50" s="6"/>
       <c r="T50" s="6"/>
@@ -4444,7 +4527,9 @@
         <v>17</v>
       </c>
       <c r="P51" s="6"/>
-      <c r="Q51" s="6"/>
+      <c r="Q51" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R51" s="6"/>
       <c r="S51" s="6"/>
       <c r="T51" s="6"/>
@@ -4494,7 +4579,9 @@
         <v>14</v>
       </c>
       <c r="P52" s="6"/>
-      <c r="Q52" s="6"/>
+      <c r="Q52" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
       <c r="T52" s="6"/>
@@ -4544,7 +4631,9 @@
         <v>17</v>
       </c>
       <c r="P53" s="6"/>
-      <c r="Q53" s="6"/>
+      <c r="Q53" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R53" s="6"/>
       <c r="S53" s="6"/>
       <c r="T53" s="6"/>
@@ -4594,7 +4683,9 @@
         <v>17</v>
       </c>
       <c r="P54" s="6"/>
-      <c r="Q54" s="6"/>
+      <c r="Q54" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R54" s="6"/>
       <c r="S54" s="6"/>
       <c r="T54" s="6"/>
@@ -4644,7 +4735,9 @@
         <v>17</v>
       </c>
       <c r="P55" s="6"/>
-      <c r="Q55" s="6"/>
+      <c r="Q55" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R55" s="6"/>
       <c r="S55" s="6"/>
       <c r="T55" s="6"/>
@@ -4694,7 +4787,9 @@
         <v>17</v>
       </c>
       <c r="P56" s="6"/>
-      <c r="Q56" s="6"/>
+      <c r="Q56" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R56" s="6"/>
       <c r="S56" s="6"/>
       <c r="T56" s="6"/>
@@ -4744,7 +4839,9 @@
         <v>17</v>
       </c>
       <c r="P57" s="6"/>
-      <c r="Q57" s="6"/>
+      <c r="Q57" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R57" s="6"/>
       <c r="S57" s="6"/>
       <c r="T57" s="6"/>
@@ -4794,7 +4891,9 @@
         <v>17</v>
       </c>
       <c r="P58" s="6"/>
-      <c r="Q58" s="6"/>
+      <c r="Q58" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R58" s="6"/>
       <c r="S58" s="6"/>
       <c r="T58" s="6"/>
@@ -4844,7 +4943,9 @@
         <v>17</v>
       </c>
       <c r="P59" s="6"/>
-      <c r="Q59" s="6"/>
+      <c r="Q59" s="6" t="s">
+        <v>370</v>
+      </c>
       <c r="R59" s="6"/>
       <c r="S59" s="6"/>
       <c r="T59" s="6"/>
@@ -4894,7 +4995,9 @@
         <v>17</v>
       </c>
       <c r="P60" s="6"/>
-      <c r="Q60" s="6"/>
+      <c r="Q60" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R60" s="6"/>
       <c r="S60" s="6"/>
       <c r="T60" s="6"/>
@@ -4944,7 +5047,9 @@
         <v>17</v>
       </c>
       <c r="P61" s="6"/>
-      <c r="Q61" s="6"/>
+      <c r="Q61" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R61" s="6"/>
       <c r="S61" s="6"/>
       <c r="T61" s="6"/>
@@ -4957,7 +5062,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="33.6">
+    <row r="62" spans="1:23">
       <c r="A62" s="5">
         <v>61</v>
       </c>
@@ -4994,13 +5099,15 @@
         <v>17</v>
       </c>
       <c r="P62" s="6"/>
-      <c r="Q62" s="6"/>
+      <c r="Q62" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R62" s="6"/>
       <c r="S62" s="6"/>
       <c r="T62" s="6"/>
       <c r="U62" s="6"/>
       <c r="V62" s="5" t="str">
-        <f t="shared" si="2"/>
+        <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C62&amp;" "&amp;B62)," ","-"))&amp;".jpg"</f>
         <v>/personnel/bella-arquine-samontañez.jpg</v>
       </c>
       <c r="W62" s="6" t="s">
@@ -5044,7 +5151,9 @@
         <v>14</v>
       </c>
       <c r="P63" s="6"/>
-      <c r="Q63" s="6"/>
+      <c r="Q63" s="6" t="s">
+        <v>371</v>
+      </c>
       <c r="R63" s="6"/>
       <c r="S63" s="6"/>
       <c r="T63" s="6"/>
@@ -5094,7 +5203,9 @@
         <v>17</v>
       </c>
       <c r="P64" s="6"/>
-      <c r="Q64" s="6"/>
+      <c r="Q64" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="R64" s="6"/>
       <c r="S64" s="6"/>
       <c r="T64" s="6"/>
@@ -5146,7 +5257,9 @@
         <v>7</v>
       </c>
       <c r="P65" s="6"/>
-      <c r="Q65" s="6"/>
+      <c r="Q65" s="6" t="s">
+        <v>274</v>
+      </c>
       <c r="R65" s="6"/>
       <c r="S65" s="6"/>
       <c r="T65" s="6"/>
@@ -5196,7 +5309,9 @@
         <v>14</v>
       </c>
       <c r="P66" s="6"/>
-      <c r="Q66" s="6"/>
+      <c r="Q66" s="6" t="s">
+        <v>372</v>
+      </c>
       <c r="R66" s="6"/>
       <c r="S66" s="6"/>
       <c r="T66" s="6"/>
@@ -5246,7 +5361,9 @@
         <v>374</v>
       </c>
       <c r="P67" s="6"/>
-      <c r="Q67" s="6"/>
+      <c r="Q67" s="6" t="s">
+        <v>373</v>
+      </c>
       <c r="R67" s="6"/>
       <c r="S67" s="6"/>
       <c r="T67" s="6"/>
@@ -5259,7 +5376,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="33.6">
+    <row r="68" spans="1:23">
       <c r="A68" s="5">
         <v>67</v>
       </c>
@@ -5296,7 +5413,9 @@
         <v>374</v>
       </c>
       <c r="P68" s="6"/>
-      <c r="Q68" s="6"/>
+      <c r="Q68" s="6" t="s">
+        <v>373</v>
+      </c>
       <c r="R68" s="6"/>
       <c r="S68" s="6"/>
       <c r="T68" s="6"/>
@@ -5346,7 +5465,9 @@
         <v>374</v>
       </c>
       <c r="P69" s="6"/>
-      <c r="Q69" s="6"/>
+      <c r="Q69" s="6" t="s">
+        <v>373</v>
+      </c>
       <c r="R69" s="6"/>
       <c r="S69" s="6"/>
       <c r="T69" s="6"/>
@@ -5396,7 +5517,9 @@
         <v>374</v>
       </c>
       <c r="P70" s="6"/>
-      <c r="Q70" s="6"/>
+      <c r="Q70" s="6" t="s">
+        <v>373</v>
+      </c>
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
       <c r="T70" s="6"/>

</xml_diff>

<commit_message>
Update organization roster with CSV-based personnel data v3
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A37C7BDA-DA1C-4B71-ABE9-1240B01A5A10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A22A98-65F6-4E30-9B68-709C7B3757D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="21315" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personnel" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="395">
   <si>
     <t>order</t>
   </si>
@@ -1214,6 +1214,12 @@
   </si>
   <si>
     <t>Computer Systems Servicing / Filipino</t>
+  </si>
+  <si>
+    <t>7th Grade Level Chairpersons</t>
+  </si>
+  <si>
+    <t>8th Grade Level Chairpersons</t>
   </si>
 </sst>
 </file>
@@ -1320,47 +1326,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="26">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1588,6 +1553,47 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1741,22 +1747,22 @@
     <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="16">
       <calculatedColumnFormula>TRIM(_xlfn.TEXTJOIN(" ",TRUE,C2,IF(E2&lt;&gt;"",IF(RIGHT(E2,1)=".",E2,E2&amp;"."),D2),B2,F2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="0"/>
-    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="1"/>
-    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="15"/>
-    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="14"/>
-    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="10"/>
-    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="9"/>
-    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="8"/>
-    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="7"/>
-    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="6"/>
-    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="15"/>
+    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="14"/>
+    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="13"/>
+    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="12"/>
+    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="11"/>
+    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="7"/>
+    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="6"/>
+    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="5"/>
+    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="4"/>
+    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="3"/>
+    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2050,7 +2056,9 @@
       <c r="Q2" s="6"/>
       <c r="R2" s="6"/>
       <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
+      <c r="T2" s="6">
+        <v>2</v>
+      </c>
       <c r="U2" s="6"/>
       <c r="V2" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C2&amp;" "&amp;B2)," ","-"))&amp;".jpg"</f>
@@ -2760,7 +2768,9 @@
       </c>
       <c r="R15" s="6"/>
       <c r="S15" s="6"/>
-      <c r="T15" s="6"/>
+      <c r="T15" s="6">
+        <v>1</v>
+      </c>
       <c r="U15" s="6"/>
       <c r="V15" s="5" t="str">
         <f t="shared" si="2"/>
@@ -3026,7 +3036,9 @@
       <c r="Q20" s="6"/>
       <c r="R20" s="6"/>
       <c r="S20" s="6"/>
-      <c r="T20" s="6"/>
+      <c r="T20" s="6">
+        <v>3</v>
+      </c>
       <c r="U20" s="6"/>
       <c r="V20" s="5" t="str">
         <f t="shared" si="2"/>
@@ -3732,7 +3744,7 @@
         <v>244</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>367</v>
+        <v>394</v>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="5"/>
@@ -3752,7 +3764,9 @@
       </c>
       <c r="R33" s="6"/>
       <c r="S33" s="6"/>
-      <c r="T33" s="6"/>
+      <c r="T33" s="6">
+        <v>4</v>
+      </c>
       <c r="U33" s="6"/>
       <c r="V33" s="5" t="str">
         <f t="shared" si="2"/>
@@ -5176,7 +5190,7 @@
         <v>12</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>367</v>
+        <v>393</v>
       </c>
       <c r="J59" s="5"/>
       <c r="K59" s="5"/>
@@ -5196,7 +5210,9 @@
       </c>
       <c r="R59" s="6"/>
       <c r="S59" s="6"/>
-      <c r="T59" s="6"/>
+      <c r="T59" s="6">
+        <v>5</v>
+      </c>
       <c r="U59" s="6"/>
       <c r="V59" s="5" t="str">
         <f t="shared" si="2"/>

</xml_diff>

<commit_message>
Update organization personnel card designation format
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4A22A98-65F6-4E30-9B68-709C7B3757D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB6C8804-AD6D-4FAF-9623-3DB465BD80B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="21315" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personnel" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="421">
   <si>
     <t>order</t>
   </si>
@@ -1180,9 +1180,6 @@
     <t>SDRRM Coordinator</t>
   </si>
   <si>
-    <t>LIS/ICT/EBEIS Coordinator</t>
-  </si>
-  <si>
     <t>SSLG Coordinator</t>
   </si>
   <si>
@@ -1220,6 +1217,87 @@
   </si>
   <si>
     <t>8th Grade Level Chairpersons</t>
+  </si>
+  <si>
+    <t>Subject Teacher</t>
+  </si>
+  <si>
+    <t>LIS/ICT/EBEIS Coordinator/SMIS Manager</t>
+  </si>
+  <si>
+    <t>advisoryGradeLevel</t>
+  </si>
+  <si>
+    <t>advisorySection</t>
+  </si>
+  <si>
+    <t>Swan</t>
+  </si>
+  <si>
+    <t>Jade</t>
+  </si>
+  <si>
+    <t>Maple</t>
+  </si>
+  <si>
+    <t>Ruby</t>
+  </si>
+  <si>
+    <t>Raven</t>
+  </si>
+  <si>
+    <t>Carrion</t>
+  </si>
+  <si>
+    <t>Olive</t>
+  </si>
+  <si>
+    <t>Emerald</t>
+  </si>
+  <si>
+    <t>Periwinkle</t>
+  </si>
+  <si>
+    <t>Cypress</t>
+  </si>
+  <si>
+    <t>Amethyst</t>
+  </si>
+  <si>
+    <t>Falcon</t>
+  </si>
+  <si>
+    <t>Dove</t>
+  </si>
+  <si>
+    <t>Rose</t>
+  </si>
+  <si>
+    <t>Diamond</t>
+  </si>
+  <si>
+    <t>Aspen</t>
+  </si>
+  <si>
+    <t>Hyacinth</t>
+  </si>
+  <si>
+    <t>Canary</t>
+  </si>
+  <si>
+    <t>Stargazer</t>
+  </si>
+  <si>
+    <t>Sapphire</t>
+  </si>
+  <si>
+    <t>Eagle</t>
+  </si>
+  <si>
+    <t>Elm</t>
+  </si>
+  <si>
+    <t>Hazel</t>
   </si>
 </sst>
 </file>
@@ -1325,7 +1403,45 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="28">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1734,35 +1850,37 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:W71" headerRowDxfId="25" dataDxfId="24" totalsRowDxfId="23">
-  <tableColumns count="23">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="21"/>
-    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="20"/>
-    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="19"/>
-    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:Y71" headerRowDxfId="27" dataDxfId="26" totalsRowDxfId="25">
+  <tableColumns count="25">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="23"/>
+    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="22"/>
+    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="21"/>
+    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="20">
       <calculatedColumnFormula>IF(D2="","",LEFT(TRIM(D2),1)&amp;".")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="17"/>
-    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="16">
+    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="19"/>
+    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="18">
       <calculatedColumnFormula>TRIM(_xlfn.TEXTJOIN(" ",TRUE,C2,IF(E2&lt;&gt;"",IF(RIGHT(E2,1)=".",E2,E2&amp;"."),D2),B2,F2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="7"/>
-    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="6"/>
-    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="5"/>
-    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="3"/>
-    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="17"/>
+    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="16"/>
+    <tableColumn id="24" xr3:uid="{9E70E31F-1B17-4E67-A99E-4037A94153C1}" name="advisoryGradeLevel" dataDxfId="1"/>
+    <tableColumn id="25" xr3:uid="{82F63A8C-E0AF-4172-B1EB-CC758DA39858}" name="advisorySection" dataDxfId="0"/>
+    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="15"/>
+    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="14"/>
+    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="13"/>
+    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="9"/>
+    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="8"/>
+    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="7"/>
+    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="5"/>
+    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1917,7 +2035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W71"/>
+  <dimension ref="A1:Y71"/>
   <sheetFormatPr defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="5.59765625" style="4" bestFit="1" customWidth="1"/>
@@ -1928,20 +2046,22 @@
     <col min="6" max="6" width="5.796875" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30.3984375" style="4" customWidth="1"/>
     <col min="8" max="8" width="23.5" style="4" customWidth="1"/>
-    <col min="9" max="9" width="27.69921875" style="11" customWidth="1"/>
-    <col min="10" max="10" width="31" style="4" customWidth="1"/>
-    <col min="11" max="12" width="28" style="4" customWidth="1"/>
-    <col min="13" max="13" width="32.8984375" style="4" customWidth="1"/>
-    <col min="14" max="14" width="26.69921875" style="4" customWidth="1"/>
-    <col min="15" max="15" width="20.09765625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="45.19921875" style="7" customWidth="1"/>
-    <col min="17" max="21" width="24.19921875" style="7" customWidth="1"/>
-    <col min="22" max="22" width="36.69921875" style="4" customWidth="1"/>
-    <col min="23" max="23" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="8.796875" style="4"/>
+    <col min="9" max="9" width="40.796875" style="11" customWidth="1"/>
+    <col min="10" max="10" width="19.296875" style="11" customWidth="1"/>
+    <col min="11" max="11" width="17.296875" style="11" customWidth="1"/>
+    <col min="12" max="12" width="31" style="4" customWidth="1"/>
+    <col min="13" max="14" width="28" style="4" customWidth="1"/>
+    <col min="15" max="15" width="32.8984375" style="4" customWidth="1"/>
+    <col min="16" max="16" width="26.69921875" style="4" customWidth="1"/>
+    <col min="17" max="17" width="20.09765625" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="45.19921875" style="7" customWidth="1"/>
+    <col min="19" max="23" width="24.19921875" style="7" customWidth="1"/>
+    <col min="24" max="24" width="36.69921875" style="4" customWidth="1"/>
+    <col min="25" max="25" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="26" max="16384" width="8.796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="20.399999999999999" customHeight="1">
+    <row r="1" spans="1:25" ht="20.399999999999999" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1970,49 +2090,55 @@
         <v>324</v>
       </c>
       <c r="J1" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="L1" s="8" t="s">
         <v>325</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>358</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>359</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>326</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="W1" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="X1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="Y1" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2040,35 +2166,37 @@
       <c r="I2" s="9" t="s">
         <v>327</v>
       </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
       <c r="L2" s="5"/>
       <c r="M2" s="5"/>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="Q2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="R2" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
       <c r="S2" s="6"/>
-      <c r="T2" s="6">
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6">
         <v>2</v>
       </c>
-      <c r="U2" s="6"/>
-      <c r="V2" s="5" t="str">
+      <c r="W2" s="6"/>
+      <c r="X2" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C2&amp;" "&amp;B2)," ","-"))&amp;".jpg"</f>
         <v>/personnel/paz-abad.jpg</v>
       </c>
-      <c r="W2" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23">
+      <c r="Y2" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -2094,37 +2222,43 @@
         <v>12</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J3" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>398</v>
+      </c>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
-      <c r="N3" s="6" t="s">
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="R3" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q3" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
+      <c r="S3" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T3" s="6"/>
       <c r="U3" s="6"/>
-      <c r="V3" s="5" t="str">
-        <f t="shared" ref="V3:V66" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C3&amp;" "&amp;B3)," ","-"))&amp;".jpg"</f>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="5" t="str">
+        <f t="shared" ref="X3:X66" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C3&amp;" "&amp;B3)," ","-"))&amp;".jpg"</f>
         <v>/personnel/marissa-abalo.jpg</v>
       </c>
-      <c r="W3" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23">
+      <c r="Y3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -2150,33 +2284,35 @@
         <v>12</v>
       </c>
       <c r="I4" s="10"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="Q4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="6"/>
+      <c r="R4" s="6" t="s">
+        <v>385</v>
+      </c>
       <c r="S4" s="6"/>
       <c r="T4" s="6"/>
       <c r="U4" s="6"/>
-      <c r="V4" s="5" t="str">
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+      <c r="X4" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joseph-allosada.jpg</v>
       </c>
-      <c r="W4" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23">
+      <c r="Y4" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -2202,37 +2338,43 @@
         <v>12</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>399</v>
+      </c>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O5" s="5" t="s">
+      <c r="Q5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P5" s="6" t="s">
+      <c r="R5" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q5" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
+      <c r="S5" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T5" s="6"/>
       <c r="U5" s="6"/>
-      <c r="V5" s="5" t="str">
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+      <c r="X5" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/sharon-gay-alsa.jpg</v>
       </c>
-      <c r="W5" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23">
+      <c r="Y5" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -2258,37 +2400,39 @@
         <v>12</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J6" s="5"/>
-      <c r="K6" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="5" t="s">
+      <c r="Q6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P6" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="Q6" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
+      <c r="R6" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T6" s="6"/>
       <c r="U6" s="6"/>
-      <c r="V6" s="5" t="str">
+      <c r="V6" s="6"/>
+      <c r="W6" s="6"/>
+      <c r="X6" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lonier-andrade.jpg</v>
       </c>
-      <c r="W6" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23">
+      <c r="Y6" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -2314,37 +2458,43 @@
         <v>16</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>400</v>
+      </c>
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="Q7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="6" t="s">
+      <c r="R7" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="Q7" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
+      <c r="S7" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T7" s="6"/>
       <c r="U7" s="6"/>
-      <c r="V7" s="5" t="str">
+      <c r="V7" s="6"/>
+      <c r="W7" s="6"/>
+      <c r="X7" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/allan-raul-aparicio.jpg</v>
       </c>
-      <c r="W7" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23">
+      <c r="Y7" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -2370,33 +2520,35 @@
         <v>239</v>
       </c>
       <c r="I8" s="10"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
-      <c r="N8" s="6" t="s">
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O8" s="5" t="s">
+      <c r="Q8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P8" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
+      <c r="R8" s="6" t="s">
+        <v>387</v>
+      </c>
       <c r="S8" s="6"/>
       <c r="T8" s="6"/>
       <c r="U8" s="6"/>
-      <c r="V8" s="5" t="str">
+      <c r="V8" s="6"/>
+      <c r="W8" s="6"/>
+      <c r="X8" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/niña-kristine-ayos.jpg</v>
       </c>
-      <c r="W8" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23">
+      <c r="Y8" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -2422,33 +2574,35 @@
         <v>244</v>
       </c>
       <c r="I9" s="10"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O9" s="5" t="s">
+      <c r="Q9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="6" t="s">
+      <c r="R9" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="6"/>
       <c r="S9" s="6"/>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
-      <c r="V9" s="5" t="str">
+      <c r="V9" s="6"/>
+      <c r="W9" s="6"/>
+      <c r="X9" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/glenn-barangan.jpg</v>
       </c>
-      <c r="W9" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
+      <c r="Y9" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -2474,37 +2628,43 @@
         <v>12</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>401</v>
+      </c>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O10" s="5" t="s">
+      <c r="Q10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P10" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Q10" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
+      <c r="R10" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="S10" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T10" s="6"/>
       <c r="U10" s="6"/>
-      <c r="V10" s="5" t="str">
+      <c r="V10" s="6"/>
+      <c r="W10" s="6"/>
+      <c r="X10" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jake-barcenas.jpg</v>
       </c>
-      <c r="W10" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23">
+      <c r="Y10" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -2530,35 +2690,41 @@
         <v>12</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>402</v>
+      </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
-      <c r="N11" s="6" t="s">
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
+      <c r="P11" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O11" s="5" t="s">
+      <c r="Q11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R11" s="6"/>
-      <c r="S11" s="6"/>
+      <c r="S11" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T11" s="6"/>
       <c r="U11" s="6"/>
-      <c r="V11" s="5" t="str">
+      <c r="V11" s="6"/>
+      <c r="W11" s="6"/>
+      <c r="X11" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/eljoy-barroca.jpg</v>
       </c>
-      <c r="W11" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23">
+      <c r="Y11" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -2584,37 +2750,39 @@
         <v>12</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J12" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
       <c r="M12" s="5"/>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O12" s="5" t="s">
+      <c r="Q12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R12" s="6"/>
-      <c r="S12" s="6"/>
+      <c r="S12" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T12" s="6"/>
       <c r="U12" s="6"/>
-      <c r="V12" s="5" t="str">
+      <c r="V12" s="6"/>
+      <c r="W12" s="6"/>
+      <c r="X12" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/angel-batuigas.jpg</v>
       </c>
-      <c r="W12" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23">
+      <c r="Y12" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -2640,33 +2808,35 @@
         <v>12</v>
       </c>
       <c r="I13" s="10"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
-      <c r="N13" s="6" t="s">
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O13" s="5" t="s">
+      <c r="Q13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P13" s="6" t="s">
+      <c r="R13" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
       <c r="S13" s="6"/>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
-      <c r="V13" s="5" t="str">
+      <c r="V13" s="6"/>
+      <c r="W13" s="6"/>
+      <c r="X13" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/mary-josephine-bawiga.jpg</v>
       </c>
-      <c r="W13" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23">
+      <c r="Y13" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -2692,37 +2862,43 @@
         <v>12</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>403</v>
+      </c>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
-      <c r="N14" s="6" t="s">
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
+      <c r="P14" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O14" s="5" t="s">
+      <c r="Q14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P14" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q14" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R14" s="6"/>
-      <c r="S14" s="6"/>
+      <c r="R14" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T14" s="6"/>
       <c r="U14" s="6"/>
-      <c r="V14" s="5" t="str">
+      <c r="V14" s="6"/>
+      <c r="W14" s="6"/>
+      <c r="X14" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/endrie-bohol.jpg</v>
       </c>
-      <c r="W14" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23">
+      <c r="Y14" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -2750,37 +2926,39 @@
       <c r="I15" s="10" t="s">
         <v>331</v>
       </c>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10"/>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
-      <c r="N15" s="6" t="s">
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
+      <c r="P15" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O15" s="5" t="s">
+      <c r="Q15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P15" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q15" s="6" t="s">
+      <c r="R15" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S15" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
-      <c r="T15" s="6">
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="6">
         <v>1</v>
       </c>
-      <c r="U15" s="6"/>
-      <c r="V15" s="5" t="str">
+      <c r="W15" s="6"/>
+      <c r="X15" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/maine-bongas.jpg</v>
       </c>
-      <c r="W15" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23">
+      <c r="Y15" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -2804,35 +2982,37 @@
         <v>12</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
-      <c r="N16" s="6" t="s">
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
+      <c r="P16" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O16" s="5" t="s">
+      <c r="Q16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R16" s="6"/>
-      <c r="S16" s="6"/>
+      <c r="S16" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T16" s="6"/>
       <c r="U16" s="6"/>
-      <c r="V16" s="5" t="str">
+      <c r="V16" s="6"/>
+      <c r="W16" s="6"/>
+      <c r="X16" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/ruth-briones.jpg</v>
       </c>
-      <c r="W16" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23">
+      <c r="Y16" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -2858,31 +3038,33 @@
         <v>12</v>
       </c>
       <c r="I17" s="10"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
-      <c r="N17" s="6" t="s">
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
+      <c r="P17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O17" s="5" t="s">
+      <c r="Q17" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="6"/>
       <c r="R17" s="6"/>
       <c r="S17" s="6"/>
       <c r="T17" s="6"/>
       <c r="U17" s="6"/>
-      <c r="V17" s="5" t="str">
+      <c r="V17" s="6"/>
+      <c r="W17" s="6"/>
+      <c r="X17" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/sharon-broñola.jpg</v>
       </c>
-      <c r="W17" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23">
+      <c r="Y17" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -2910,33 +3092,35 @@
       <c r="I18" s="10" t="s">
         <v>377</v>
       </c>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
-      <c r="N18" s="6" t="s">
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
+      <c r="P18" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O18" s="5" t="s">
+      <c r="Q18" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P18" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q18" s="6"/>
-      <c r="R18" s="6"/>
+      <c r="R18" s="6" t="s">
+        <v>387</v>
+      </c>
       <c r="S18" s="6"/>
       <c r="T18" s="6"/>
       <c r="U18" s="6"/>
-      <c r="V18" s="5" t="str">
+      <c r="V18" s="6"/>
+      <c r="W18" s="6"/>
+      <c r="X18" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joan-cabalda.jpg</v>
       </c>
-      <c r="W18" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23">
+      <c r="Y18" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -2962,37 +3146,39 @@
         <v>249</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>385</v>
-      </c>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
+        <v>384</v>
+      </c>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
-      <c r="N19" s="6" t="s">
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
+      <c r="P19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O19" s="5" t="s">
+      <c r="Q19" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P19" s="6" t="s">
+      <c r="R19" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="Q19" s="6" t="s">
+      <c r="S19" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R19" s="6"/>
-      <c r="S19" s="6"/>
       <c r="T19" s="6"/>
       <c r="U19" s="6"/>
-      <c r="V19" s="5" t="str">
+      <c r="V19" s="6"/>
+      <c r="W19" s="6"/>
+      <c r="X19" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/gracelyn-cabunag.jpg</v>
       </c>
-      <c r="W19" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23">
+      <c r="Y19" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -3020,35 +3206,37 @@
       <c r="I20" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
-      <c r="N20" s="6" t="s">
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O20" s="5" t="s">
+      <c r="Q20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="P20" s="6" t="s">
+      <c r="R20" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="6"/>
       <c r="S20" s="6"/>
-      <c r="T20" s="6">
+      <c r="T20" s="6"/>
+      <c r="U20" s="6"/>
+      <c r="V20" s="6">
         <v>3</v>
       </c>
-      <c r="U20" s="6"/>
-      <c r="V20" s="5" t="str">
+      <c r="W20" s="6"/>
+      <c r="X20" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/hector-cabanca.jpg</v>
       </c>
-      <c r="W20" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23">
+      <c r="Y20" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -3074,37 +3262,43 @@
         <v>16</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J21" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="K21" s="10" t="s">
+        <v>404</v>
+      </c>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
-      <c r="N21" s="6" t="s">
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O21" s="5" t="s">
+      <c r="Q21" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P21" s="6" t="s">
+      <c r="R21" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q21" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R21" s="6"/>
-      <c r="S21" s="6"/>
+      <c r="S21" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T21" s="6"/>
       <c r="U21" s="6"/>
-      <c r="V21" s="5" t="str">
+      <c r="V21" s="6"/>
+      <c r="W21" s="6"/>
+      <c r="X21" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeffrey-caberte.jpg</v>
       </c>
-      <c r="W21" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:23">
+      <c r="Y21" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -3130,35 +3324,41 @@
         <v>12</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>405</v>
+      </c>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
-      <c r="N22" s="6" t="s">
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
+      <c r="P22" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O22" s="5" t="s">
+      <c r="Q22" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P22" s="6"/>
-      <c r="Q22" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R22" s="6"/>
-      <c r="S22" s="6"/>
+      <c r="S22" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
-      <c r="V22" s="5" t="str">
+      <c r="V22" s="6"/>
+      <c r="W22" s="6"/>
+      <c r="X22" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marilou-cabriana.jpg</v>
       </c>
-      <c r="W22" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:23">
+      <c r="Y22" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -3186,35 +3386,37 @@
       <c r="I23" s="10" t="s">
         <v>364</v>
       </c>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
-      <c r="N23" s="6" t="s">
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
+      <c r="P23" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O23" s="5" t="s">
+      <c r="Q23" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P23" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q23" s="6" t="s">
+      <c r="R23" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S23" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="R23" s="6"/>
-      <c r="S23" s="6"/>
       <c r="T23" s="6"/>
       <c r="U23" s="6"/>
-      <c r="V23" s="5" t="str">
+      <c r="V23" s="6"/>
+      <c r="W23" s="6"/>
+      <c r="X23" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jasmin-cabuenas.jpg</v>
       </c>
-      <c r="W23" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23">
+      <c r="Y23" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -3240,37 +3442,39 @@
         <v>12</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
+        <v>394</v>
+      </c>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
-      <c r="N24" s="6" t="s">
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O24" s="5" t="s">
+      <c r="Q24" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P24" s="6" t="s">
+      <c r="R24" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q24" s="6" t="s">
+      <c r="S24" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R24" s="6"/>
-      <c r="S24" s="6"/>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
-      <c r="V24" s="5" t="str">
+      <c r="V24" s="6"/>
+      <c r="W24" s="6"/>
+      <c r="X24" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/elsa-calunod.jpg</v>
       </c>
-      <c r="W24" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23">
+      <c r="Y24" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -3296,37 +3500,43 @@
         <v>12</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J25" s="5"/>
-      <c r="K25" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J25" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="K25" s="10" t="s">
+        <v>406</v>
+      </c>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
-      <c r="N25" s="6" t="s">
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O25" s="5" t="s">
+      <c r="Q25" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P25" s="6" t="s">
+      <c r="R25" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="Q25" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R25" s="6"/>
-      <c r="S25" s="6"/>
+      <c r="S25" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T25" s="6"/>
       <c r="U25" s="6"/>
-      <c r="V25" s="5" t="str">
+      <c r="V25" s="6"/>
+      <c r="W25" s="6"/>
+      <c r="X25" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/leslyn-rose-camero.jpg</v>
       </c>
-      <c r="W25" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="26" spans="1:23">
+      <c r="Y25" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -3354,35 +3564,37 @@
       <c r="I26" s="10" t="s">
         <v>378</v>
       </c>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
-      <c r="N26" s="6" t="s">
+      <c r="N26" s="5"/>
+      <c r="O26" s="5"/>
+      <c r="P26" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O26" s="5" t="s">
+      <c r="Q26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P26" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q26" s="6" t="s">
+      <c r="R26" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S26" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="R26" s="6"/>
-      <c r="S26" s="6"/>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
-      <c r="V26" s="5" t="str">
+      <c r="V26" s="6"/>
+      <c r="W26" s="6"/>
+      <c r="X26" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/dawn-camille-caparida.jpg</v>
       </c>
-      <c r="W26" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:23">
+      <c r="Y26" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -3406,37 +3618,43 @@
         <v>16</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J27" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="K27" s="10" t="s">
+        <v>407</v>
+      </c>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
-      <c r="N27" s="6" t="s">
+      <c r="N27" s="5"/>
+      <c r="O27" s="5"/>
+      <c r="P27" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O27" s="5" t="s">
+      <c r="Q27" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P27" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q27" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R27" s="6"/>
-      <c r="S27" s="6"/>
+      <c r="R27" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S27" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T27" s="6"/>
       <c r="U27" s="6"/>
-      <c r="V27" s="5" t="str">
+      <c r="V27" s="6"/>
+      <c r="W27" s="6"/>
+      <c r="X27" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lourence-capa.jpg</v>
       </c>
-      <c r="W27" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23">
+      <c r="Y27" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -3462,37 +3680,43 @@
         <v>12</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J28" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="K28" s="10" t="s">
+        <v>408</v>
+      </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
-      <c r="N28" s="6" t="s">
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O28" s="5" t="s">
+      <c r="Q28" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P28" s="6" t="s">
+      <c r="R28" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="Q28" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
+      <c r="S28" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
-      <c r="V28" s="5" t="str">
+      <c r="V28" s="6"/>
+      <c r="W28" s="6"/>
+      <c r="X28" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joan-cavite.jpg</v>
       </c>
-      <c r="W28" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="29" spans="1:23">
+      <c r="Y28" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -3520,37 +3744,39 @@
         <v>270</v>
       </c>
       <c r="I29" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
-      <c r="N29" s="6" t="s">
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O29" s="5" t="s">
+      <c r="Q29" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P29" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q29" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R29" s="6"/>
-      <c r="S29" s="6"/>
+      <c r="R29" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S29" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T29" s="6"/>
       <c r="U29" s="6"/>
-      <c r="V29" s="5" t="str">
+      <c r="V29" s="6"/>
+      <c r="W29" s="6"/>
+      <c r="X29" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joseph-dagaraga.jpg</v>
       </c>
-      <c r="W29" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:23">
+      <c r="Y29" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -3578,35 +3804,37 @@
       <c r="I30" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
       <c r="L30" s="5"/>
       <c r="M30" s="5"/>
-      <c r="N30" s="6" t="s">
+      <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
+      <c r="P30" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O30" s="5" t="s">
+      <c r="Q30" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P30" s="6" t="s">
+      <c r="R30" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="Q30" s="6" t="s">
+      <c r="S30" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
-      <c r="V30" s="5" t="str">
+      <c r="V30" s="6"/>
+      <c r="W30" s="6"/>
+      <c r="X30" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carolyn-delos-reyes.jpg</v>
       </c>
-      <c r="W30" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="31" spans="1:23">
+      <c r="Y30" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -3634,35 +3862,37 @@
       <c r="I31" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
       <c r="L31" s="5"/>
       <c r="M31" s="5"/>
-      <c r="N31" s="6" t="s">
+      <c r="N31" s="5"/>
+      <c r="O31" s="5"/>
+      <c r="P31" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O31" s="5" t="s">
+      <c r="Q31" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P31" s="6" t="s">
+      <c r="R31" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q31" s="6" t="s">
+      <c r="S31" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
       <c r="T31" s="6"/>
       <c r="U31" s="6"/>
-      <c r="V31" s="5" t="str">
+      <c r="V31" s="6"/>
+      <c r="W31" s="6"/>
+      <c r="X31" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lucille-echavez.jpg</v>
       </c>
-      <c r="W31" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:23">
+      <c r="Y31" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -3690,35 +3920,37 @@
       <c r="I32" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
       <c r="L32" s="5"/>
       <c r="M32" s="5"/>
-      <c r="N32" s="6" t="s">
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+      <c r="P32" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O32" s="5" t="s">
+      <c r="Q32" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P32" s="6" t="s">
-        <v>390</v>
-      </c>
-      <c r="Q32" s="6" t="s">
+      <c r="R32" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="S32" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R32" s="6"/>
-      <c r="S32" s="6"/>
       <c r="T32" s="6"/>
       <c r="U32" s="6"/>
-      <c r="V32" s="5" t="str">
+      <c r="V32" s="6"/>
+      <c r="W32" s="6"/>
+      <c r="X32" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/benerando-erediano.jpg</v>
       </c>
-      <c r="W32" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23">
+      <c r="Y32" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:25">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -3744,39 +3976,41 @@
         <v>244</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>394</v>
-      </c>
-      <c r="J33" s="5"/>
-      <c r="K33" s="5"/>
+        <v>393</v>
+      </c>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
       <c r="L33" s="5"/>
       <c r="M33" s="5"/>
-      <c r="N33" s="6" t="s">
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O33" s="5" t="s">
+      <c r="Q33" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P33" s="6" t="s">
+      <c r="R33" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="Q33" s="6" t="s">
+      <c r="S33" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="R33" s="6"/>
-      <c r="S33" s="6"/>
-      <c r="T33" s="6">
+      <c r="T33" s="6"/>
+      <c r="U33" s="6"/>
+      <c r="V33" s="6">
         <v>4</v>
       </c>
-      <c r="U33" s="6"/>
-      <c r="V33" s="5" t="str">
+      <c r="W33" s="6"/>
+      <c r="X33" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/metchie-gay-gastanes.jpg</v>
       </c>
-      <c r="W33" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="34" spans="1:23">
+      <c r="Y33" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:25">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -3802,37 +4036,39 @@
         <v>12</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>384</v>
-      </c>
-      <c r="J34" s="5"/>
-      <c r="K34" s="5"/>
+        <v>383</v>
+      </c>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
       <c r="L34" s="5"/>
       <c r="M34" s="5"/>
-      <c r="N34" s="6" t="s">
+      <c r="N34" s="5"/>
+      <c r="O34" s="5"/>
+      <c r="P34" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O34" s="5" t="s">
+      <c r="Q34" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P34" s="6" t="s">
+      <c r="R34" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="Q34" s="6" t="s">
+      <c r="S34" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R34" s="6"/>
-      <c r="S34" s="6"/>
       <c r="T34" s="6"/>
       <c r="U34" s="6"/>
-      <c r="V34" s="5" t="str">
+      <c r="V34" s="6"/>
+      <c r="W34" s="6"/>
+      <c r="X34" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jasmin-gerodias.jpg</v>
       </c>
-      <c r="W34" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23">
+      <c r="Y34" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:25">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -3858,37 +4094,43 @@
         <v>12</v>
       </c>
       <c r="I35" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J35" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="K35" s="10" t="s">
+        <v>409</v>
+      </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
-      <c r="N35" s="6" t="s">
+      <c r="N35" s="5"/>
+      <c r="O35" s="5"/>
+      <c r="P35" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O35" s="5" t="s">
+      <c r="Q35" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P35" s="6" t="s">
+      <c r="R35" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q35" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R35" s="6"/>
-      <c r="S35" s="6"/>
+      <c r="S35" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T35" s="6"/>
       <c r="U35" s="6"/>
-      <c r="V35" s="5" t="str">
+      <c r="V35" s="6"/>
+      <c r="W35" s="6"/>
+      <c r="X35" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeralyn-gerra.jpg</v>
       </c>
-      <c r="W35" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="36" spans="1:23">
+      <c r="Y35" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" spans="1:25">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -3914,37 +4156,43 @@
         <v>241</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J36" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="K36" s="10" t="s">
+        <v>410</v>
+      </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
-      <c r="N36" s="6" t="s">
+      <c r="N36" s="5"/>
+      <c r="O36" s="5"/>
+      <c r="P36" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O36" s="5" t="s">
+      <c r="Q36" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P36" s="6" t="s">
+      <c r="R36" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="Q36" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R36" s="6"/>
-      <c r="S36" s="6"/>
+      <c r="S36" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T36" s="6"/>
       <c r="U36" s="6"/>
-      <c r="V36" s="5" t="str">
+      <c r="V36" s="6"/>
+      <c r="W36" s="6"/>
+      <c r="X36" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/genesa-goc-ong.jpg</v>
       </c>
-      <c r="W36" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="37" spans="1:23">
+      <c r="Y36" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:25">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -3972,35 +4220,37 @@
       <c r="I37" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
       <c r="L37" s="5"/>
       <c r="M37" s="5"/>
-      <c r="N37" s="6" t="s">
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O37" s="5" t="s">
+      <c r="Q37" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P37" s="6" t="s">
+      <c r="R37" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="Q37" s="6" t="s">
+      <c r="S37" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R37" s="6"/>
-      <c r="S37" s="6"/>
       <c r="T37" s="6"/>
       <c r="U37" s="6"/>
-      <c r="V37" s="5" t="str">
+      <c r="V37" s="6"/>
+      <c r="W37" s="6"/>
+      <c r="X37" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/janelou-gomez.jpg</v>
       </c>
-      <c r="W37" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="38" spans="1:23">
+      <c r="Y37" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:25">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -4026,37 +4276,43 @@
         <v>12</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J38" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="K38" s="10" t="s">
+        <v>411</v>
+      </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
-      <c r="N38" s="6" t="s">
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+      <c r="P38" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O38" s="5" t="s">
+      <c r="Q38" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P38" s="6" t="s">
+      <c r="R38" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q38" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R38" s="6"/>
-      <c r="S38" s="6"/>
+      <c r="S38" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T38" s="6"/>
       <c r="U38" s="6"/>
-      <c r="V38" s="5" t="str">
+      <c r="V38" s="6"/>
+      <c r="W38" s="6"/>
+      <c r="X38" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/junnelyn-herbito.jpg</v>
       </c>
-      <c r="W38" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="39" spans="1:23">
+      <c r="Y38" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:25">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -4082,37 +4338,43 @@
         <v>241</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J39" s="5"/>
-      <c r="K39" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J39" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="K39" s="10" t="s">
+        <v>412</v>
+      </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
-      <c r="N39" s="6" t="s">
+      <c r="N39" s="5"/>
+      <c r="O39" s="5"/>
+      <c r="P39" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O39" s="5" t="s">
+      <c r="Q39" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P39" s="6" t="s">
+      <c r="R39" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q39" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R39" s="6"/>
-      <c r="S39" s="6"/>
+      <c r="S39" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T39" s="6"/>
       <c r="U39" s="6"/>
-      <c r="V39" s="5" t="str">
+      <c r="V39" s="6"/>
+      <c r="W39" s="6"/>
+      <c r="X39" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/roxan-mae-jao.jpg</v>
       </c>
-      <c r="W39" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="40" spans="1:23">
+      <c r="Y39" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:25">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -4140,33 +4402,35 @@
       <c r="I40" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J40" s="5"/>
-      <c r="K40" s="5"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
       <c r="L40" s="5"/>
       <c r="M40" s="5"/>
-      <c r="N40" s="6" t="s">
+      <c r="N40" s="5"/>
+      <c r="O40" s="5"/>
+      <c r="P40" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O40" s="5" t="s">
+      <c r="Q40" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P40" s="6"/>
-      <c r="Q40" s="6" t="s">
+      <c r="R40" s="6"/>
+      <c r="S40" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R40" s="6"/>
-      <c r="S40" s="6"/>
       <c r="T40" s="6"/>
       <c r="U40" s="6"/>
-      <c r="V40" s="5" t="str">
+      <c r="V40" s="6"/>
+      <c r="W40" s="6"/>
+      <c r="X40" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/fernando-laspiñas.jpg</v>
       </c>
-      <c r="W40" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="41" spans="1:23">
+      <c r="Y40" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:25">
       <c r="A41" s="5">
         <v>40</v>
       </c>
@@ -4194,35 +4458,37 @@
       <c r="I41" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
       <c r="L41" s="5"/>
       <c r="M41" s="5"/>
-      <c r="N41" s="6" t="s">
+      <c r="N41" s="5"/>
+      <c r="O41" s="5"/>
+      <c r="P41" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O41" s="5" t="s">
+      <c r="Q41" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P41" s="6" t="s">
+      <c r="R41" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="Q41" s="6" t="s">
+      <c r="S41" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R41" s="6"/>
-      <c r="S41" s="6"/>
       <c r="T41" s="6"/>
       <c r="U41" s="6"/>
-      <c r="V41" s="5" t="str">
+      <c r="V41" s="6"/>
+      <c r="W41" s="6"/>
+      <c r="X41" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/nerisa-lim.jpg</v>
       </c>
-      <c r="W41" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="42" spans="1:23">
+      <c r="Y41" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:25">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -4248,33 +4514,35 @@
       <c r="I42" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
       <c r="L42" s="5"/>
       <c r="M42" s="5"/>
-      <c r="N42" s="6" t="s">
+      <c r="N42" s="5"/>
+      <c r="O42" s="5"/>
+      <c r="P42" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O42" s="5" t="s">
+      <c r="Q42" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P42" s="6"/>
-      <c r="Q42" s="6" t="s">
+      <c r="R42" s="6"/>
+      <c r="S42" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R42" s="6"/>
-      <c r="S42" s="6"/>
       <c r="T42" s="6"/>
       <c r="U42" s="6"/>
-      <c r="V42" s="5" t="str">
+      <c r="V42" s="6"/>
+      <c r="W42" s="6"/>
+      <c r="X42" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carl-loreto.jpg</v>
       </c>
-      <c r="W42" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43" spans="1:23">
+      <c r="Y42" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:25">
       <c r="A43" s="5">
         <v>42</v>
       </c>
@@ -4300,35 +4568,37 @@
         <v>270</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>383</v>
-      </c>
-      <c r="J43" s="5"/>
-      <c r="K43" s="5"/>
+        <v>382</v>
+      </c>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
       <c r="L43" s="5"/>
       <c r="M43" s="5"/>
-      <c r="N43" s="6" t="s">
+      <c r="N43" s="5"/>
+      <c r="O43" s="5"/>
+      <c r="P43" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O43" s="5" t="s">
+      <c r="Q43" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P43" s="6"/>
-      <c r="Q43" s="6" t="s">
+      <c r="R43" s="6"/>
+      <c r="S43" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R43" s="6"/>
-      <c r="S43" s="6"/>
       <c r="T43" s="6"/>
       <c r="U43" s="6"/>
-      <c r="V43" s="5" t="str">
+      <c r="V43" s="6"/>
+      <c r="W43" s="6"/>
+      <c r="X43" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lyka-mabanag.jpg</v>
       </c>
-      <c r="W43" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="44" spans="1:23">
+      <c r="Y43" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:25">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -4356,39 +4626,41 @@
       <c r="I44" s="10" t="s">
         <v>380</v>
       </c>
-      <c r="J44" s="5" t="s">
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
-      <c r="M44" s="5" t="s">
+      <c r="M44" s="5"/>
+      <c r="N44" s="5"/>
+      <c r="O44" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="N44" s="6" t="s">
+      <c r="P44" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O44" s="5" t="s">
+      <c r="Q44" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P44" s="6" t="s">
+      <c r="R44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q44" s="6" t="s">
+      <c r="S44" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R44" s="6"/>
-      <c r="S44" s="6"/>
       <c r="T44" s="6"/>
       <c r="U44" s="6"/>
-      <c r="V44" s="5" t="str">
+      <c r="V44" s="6"/>
+      <c r="W44" s="6"/>
+      <c r="X44" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/richie-ryan-mabunay.jpg</v>
       </c>
-      <c r="W44" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="45" spans="1:23">
+      <c r="Y44" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:25">
       <c r="A45" s="5">
         <v>44</v>
       </c>
@@ -4416,35 +4688,37 @@
       <c r="I45" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J45" s="5"/>
-      <c r="K45" s="5"/>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10"/>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
-      <c r="N45" s="6" t="s">
+      <c r="N45" s="5"/>
+      <c r="O45" s="5"/>
+      <c r="P45" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O45" s="5" t="s">
+      <c r="Q45" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P45" s="6" t="s">
+      <c r="R45" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="Q45" s="6" t="s">
+      <c r="S45" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R45" s="6"/>
-      <c r="S45" s="6"/>
       <c r="T45" s="6"/>
       <c r="U45" s="6"/>
-      <c r="V45" s="5" t="str">
+      <c r="V45" s="6"/>
+      <c r="W45" s="6"/>
+      <c r="X45" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/maria-jeziel-macanin.jpg</v>
       </c>
-      <c r="W45" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="46" spans="1:23">
+      <c r="Y45" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:25">
       <c r="A46" s="5">
         <v>45</v>
       </c>
@@ -4470,37 +4744,43 @@
         <v>12</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J46" s="5"/>
-      <c r="K46" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J46" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="K46" s="10" t="s">
+        <v>413</v>
+      </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
-      <c r="N46" s="6" t="s">
+      <c r="N46" s="5"/>
+      <c r="O46" s="5"/>
+      <c r="P46" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O46" s="5" t="s">
+      <c r="Q46" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P46" s="6" t="s">
+      <c r="R46" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="Q46" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R46" s="6"/>
-      <c r="S46" s="6"/>
+      <c r="S46" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T46" s="6"/>
       <c r="U46" s="6"/>
-      <c r="V46" s="5" t="str">
+      <c r="V46" s="6"/>
+      <c r="W46" s="6"/>
+      <c r="X46" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeralen-maloloy-on.jpg</v>
       </c>
-      <c r="W46" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="47" spans="1:23">
+      <c r="Y46" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:25">
       <c r="A47" s="5">
         <v>46</v>
       </c>
@@ -4526,37 +4806,43 @@
         <v>12</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>369</v>
-      </c>
-      <c r="J47" s="5"/>
-      <c r="K47" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J47" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="K47" s="10" t="s">
+        <v>414</v>
+      </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
-      <c r="N47" s="6" t="s">
+      <c r="N47" s="5"/>
+      <c r="O47" s="5"/>
+      <c r="P47" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O47" s="5" t="s">
+      <c r="Q47" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P47" s="6" t="s">
+      <c r="R47" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="Q47" s="6" t="s">
+      <c r="S47" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R47" s="6"/>
-      <c r="S47" s="6"/>
       <c r="T47" s="6"/>
       <c r="U47" s="6"/>
-      <c r="V47" s="5" t="str">
+      <c r="V47" s="6"/>
+      <c r="W47" s="6"/>
+      <c r="X47" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/elbert-misterio.jpg</v>
       </c>
-      <c r="W47" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="48" spans="1:23">
+      <c r="Y47" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:25">
       <c r="A48" s="5">
         <v>47</v>
       </c>
@@ -4582,35 +4868,41 @@
         <v>241</v>
       </c>
       <c r="I48" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J48" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="K48" s="10" t="s">
+        <v>415</v>
+      </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
-      <c r="N48" s="6" t="s">
+      <c r="N48" s="5"/>
+      <c r="O48" s="5"/>
+      <c r="P48" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O48" s="5" t="s">
+      <c r="Q48" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P48" s="6"/>
-      <c r="Q48" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R48" s="6"/>
-      <c r="S48" s="6"/>
+      <c r="S48" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T48" s="6"/>
       <c r="U48" s="6"/>
-      <c r="V48" s="5" t="str">
+      <c r="V48" s="6"/>
+      <c r="W48" s="6"/>
+      <c r="X48" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joy-mortal.jpg</v>
       </c>
-      <c r="W48" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="49" spans="1:23">
+      <c r="Y48" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:25">
       <c r="A49" s="5">
         <v>48</v>
       </c>
@@ -4638,33 +4930,35 @@
       <c r="I49" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
       <c r="L49" s="5"/>
       <c r="M49" s="5"/>
-      <c r="N49" s="6" t="s">
+      <c r="N49" s="5"/>
+      <c r="O49" s="5"/>
+      <c r="P49" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O49" s="5" t="s">
+      <c r="Q49" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P49" s="6"/>
-      <c r="Q49" s="6" t="s">
+      <c r="R49" s="6"/>
+      <c r="S49" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R49" s="6"/>
-      <c r="S49" s="6"/>
       <c r="T49" s="6"/>
       <c r="U49" s="6"/>
-      <c r="V49" s="5" t="str">
+      <c r="V49" s="6"/>
+      <c r="W49" s="6"/>
+      <c r="X49" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/claire-medillo.jpg</v>
       </c>
-      <c r="W49" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="50" spans="1:23">
+      <c r="Y49" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:25">
       <c r="A50" s="5">
         <v>49</v>
       </c>
@@ -4690,37 +4984,43 @@
         <v>12</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J50" s="10" t="s">
+        <v>352</v>
+      </c>
+      <c r="K50" s="10" t="s">
+        <v>416</v>
+      </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
-      <c r="N50" s="6" t="s">
+      <c r="N50" s="5"/>
+      <c r="O50" s="5"/>
+      <c r="P50" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O50" s="5" t="s">
+      <c r="Q50" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P50" s="6" t="s">
+      <c r="R50" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="Q50" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R50" s="6"/>
-      <c r="S50" s="6"/>
+      <c r="S50" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T50" s="6"/>
       <c r="U50" s="6"/>
-      <c r="V50" s="5" t="str">
+      <c r="V50" s="6"/>
+      <c r="W50" s="6"/>
+      <c r="X50" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/gwendolyn-olo.jpg</v>
       </c>
-      <c r="W50" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="51" spans="1:23">
+      <c r="Y50" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:25">
       <c r="A51" s="5">
         <v>50</v>
       </c>
@@ -4746,35 +5046,41 @@
         <v>12</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J51" s="5"/>
-      <c r="K51" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J51" s="10" t="s">
+        <v>355</v>
+      </c>
+      <c r="K51" s="10" t="s">
+        <v>417</v>
+      </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
-      <c r="N51" s="6" t="s">
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
+      <c r="P51" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O51" s="5" t="s">
+      <c r="Q51" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P51" s="6"/>
-      <c r="Q51" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R51" s="6"/>
-      <c r="S51" s="6"/>
+      <c r="S51" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T51" s="6"/>
       <c r="U51" s="6"/>
-      <c r="V51" s="5" t="str">
+      <c r="V51" s="6"/>
+      <c r="W51" s="6"/>
+      <c r="X51" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jay-neil-oro.jpg</v>
       </c>
-      <c r="W51" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="52" spans="1:23">
+      <c r="Y51" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:25">
       <c r="A52" s="5">
         <v>51</v>
       </c>
@@ -4800,37 +5106,39 @@
         <v>12</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J52" s="10"/>
+      <c r="K52" s="10"/>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
-      <c r="N52" s="6" t="s">
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O52" s="5" t="s">
+      <c r="Q52" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P52" s="6" t="s">
-        <v>391</v>
-      </c>
-      <c r="Q52" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R52" s="6"/>
-      <c r="S52" s="6"/>
+      <c r="R52" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="S52" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T52" s="6"/>
       <c r="U52" s="6"/>
-      <c r="V52" s="5" t="str">
+      <c r="V52" s="6"/>
+      <c r="W52" s="6"/>
+      <c r="X52" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/glendale-orocay.jpg</v>
       </c>
-      <c r="W52" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="53" spans="1:23">
+      <c r="Y52" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="1:25">
       <c r="A53" s="5">
         <v>52</v>
       </c>
@@ -4856,37 +5164,39 @@
         <v>16</v>
       </c>
       <c r="I53" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J53" s="5"/>
-      <c r="K53" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J53" s="10"/>
+      <c r="K53" s="10"/>
       <c r="L53" s="5"/>
       <c r="M53" s="5"/>
-      <c r="N53" s="6" t="s">
+      <c r="N53" s="5"/>
+      <c r="O53" s="5"/>
+      <c r="P53" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O53" s="5" t="s">
+      <c r="Q53" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P53" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q53" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R53" s="6"/>
-      <c r="S53" s="6"/>
+      <c r="R53" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S53" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T53" s="6"/>
       <c r="U53" s="6"/>
-      <c r="V53" s="5" t="str">
+      <c r="V53" s="6"/>
+      <c r="W53" s="6"/>
+      <c r="X53" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marissa-pintuan.jpg</v>
       </c>
-      <c r="W53" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="54" spans="1:23">
+      <c r="Y53" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="54" spans="1:25">
       <c r="A54" s="5">
         <v>53</v>
       </c>
@@ -4914,35 +5224,37 @@
       <c r="I54" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J54" s="5"/>
-      <c r="K54" s="5"/>
+      <c r="J54" s="10"/>
+      <c r="K54" s="10"/>
       <c r="L54" s="5"/>
       <c r="M54" s="5"/>
-      <c r="N54" s="6" t="s">
+      <c r="N54" s="5"/>
+      <c r="O54" s="5"/>
+      <c r="P54" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O54" s="5" t="s">
+      <c r="Q54" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P54" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="Q54" s="6" t="s">
+      <c r="R54" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="S54" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R54" s="6"/>
-      <c r="S54" s="6"/>
       <c r="T54" s="6"/>
       <c r="U54" s="6"/>
-      <c r="V54" s="5" t="str">
+      <c r="V54" s="6"/>
+      <c r="W54" s="6"/>
+      <c r="X54" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/ma.-lourdes-prajes.jpg</v>
       </c>
-      <c r="W54" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="55" spans="1:23">
+      <c r="Y54" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:25">
       <c r="A55" s="5">
         <v>54</v>
       </c>
@@ -4968,35 +5280,41 @@
         <v>12</v>
       </c>
       <c r="I55" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J55" s="5"/>
-      <c r="K55" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J55" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="K55" s="10" t="s">
+        <v>418</v>
+      </c>
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
-      <c r="N55" s="6" t="s">
+      <c r="N55" s="5"/>
+      <c r="O55" s="5"/>
+      <c r="P55" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O55" s="5" t="s">
+      <c r="Q55" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P55" s="6"/>
-      <c r="Q55" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R55" s="6"/>
-      <c r="S55" s="6"/>
+      <c r="S55" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T55" s="6"/>
       <c r="U55" s="6"/>
-      <c r="V55" s="5" t="str">
+      <c r="V55" s="6"/>
+      <c r="W55" s="6"/>
+      <c r="X55" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/bret-kalvin-primacio.jpg</v>
       </c>
-      <c r="W55" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="56" spans="1:23">
+      <c r="Y55" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="1:25">
       <c r="A56" s="5">
         <v>55</v>
       </c>
@@ -5024,35 +5342,37 @@
       <c r="I56" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J56" s="5"/>
-      <c r="K56" s="5"/>
+      <c r="J56" s="10"/>
+      <c r="K56" s="10"/>
       <c r="L56" s="5"/>
       <c r="M56" s="5"/>
-      <c r="N56" s="6" t="s">
+      <c r="N56" s="5"/>
+      <c r="O56" s="5"/>
+      <c r="P56" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O56" s="5" t="s">
+      <c r="Q56" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P56" s="6" t="s">
+      <c r="R56" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q56" s="6" t="s">
+      <c r="S56" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R56" s="6"/>
-      <c r="S56" s="6"/>
       <c r="T56" s="6"/>
       <c r="U56" s="6"/>
-      <c r="V56" s="5" t="str">
+      <c r="V56" s="6"/>
+      <c r="W56" s="6"/>
+      <c r="X56" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jhea-quiling.jpg</v>
       </c>
-      <c r="W56" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="57" spans="1:23">
+      <c r="Y56" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:25">
       <c r="A57" s="5">
         <v>56</v>
       </c>
@@ -5080,35 +5400,37 @@
       <c r="I57" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
+      <c r="J57" s="10"/>
+      <c r="K57" s="10"/>
       <c r="L57" s="5"/>
       <c r="M57" s="5"/>
-      <c r="N57" s="6" t="s">
+      <c r="N57" s="5"/>
+      <c r="O57" s="5"/>
+      <c r="P57" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O57" s="5" t="s">
+      <c r="Q57" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P57" s="6" t="s">
+      <c r="R57" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="Q57" s="6" t="s">
+      <c r="S57" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R57" s="6"/>
-      <c r="S57" s="6"/>
       <c r="T57" s="6"/>
       <c r="U57" s="6"/>
-      <c r="V57" s="5" t="str">
+      <c r="V57" s="6"/>
+      <c r="W57" s="6"/>
+      <c r="X57" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joyce-racaza.jpg</v>
       </c>
-      <c r="W57" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="58" spans="1:23">
+      <c r="Y57" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:25">
       <c r="A58" s="5">
         <v>57</v>
       </c>
@@ -5136,35 +5458,37 @@
       <c r="I58" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J58" s="5"/>
-      <c r="K58" s="5"/>
+      <c r="J58" s="10"/>
+      <c r="K58" s="10"/>
       <c r="L58" s="5"/>
       <c r="M58" s="5"/>
-      <c r="N58" s="6" t="s">
+      <c r="N58" s="5"/>
+      <c r="O58" s="5"/>
+      <c r="P58" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O58" s="5" t="s">
+      <c r="Q58" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P58" s="6" t="s">
+      <c r="R58" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="Q58" s="6" t="s">
+      <c r="S58" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R58" s="6"/>
-      <c r="S58" s="6"/>
       <c r="T58" s="6"/>
       <c r="U58" s="6"/>
-      <c r="V58" s="5" t="str">
+      <c r="V58" s="6"/>
+      <c r="W58" s="6"/>
+      <c r="X58" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/cromwell-retuya.jpg</v>
       </c>
-      <c r="W58" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="59" spans="1:23">
+      <c r="Y58" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="59" spans="1:25">
       <c r="A59" s="5">
         <v>58</v>
       </c>
@@ -5190,39 +5514,41 @@
         <v>12</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>393</v>
-      </c>
-      <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
+        <v>392</v>
+      </c>
+      <c r="J59" s="10"/>
+      <c r="K59" s="10"/>
       <c r="L59" s="5"/>
       <c r="M59" s="5"/>
-      <c r="N59" s="6" t="s">
+      <c r="N59" s="5"/>
+      <c r="O59" s="5"/>
+      <c r="P59" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O59" s="5" t="s">
+      <c r="Q59" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P59" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="Q59" s="6" t="s">
+      <c r="R59" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="S59" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="R59" s="6"/>
-      <c r="S59" s="6"/>
-      <c r="T59" s="6">
+      <c r="T59" s="6"/>
+      <c r="U59" s="6"/>
+      <c r="V59" s="6">
         <v>5</v>
       </c>
-      <c r="U59" s="6"/>
-      <c r="V59" s="5" t="str">
+      <c r="W59" s="6"/>
+      <c r="X59" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/nancy-reyes.jpg</v>
       </c>
-      <c r="W59" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="60" spans="1:23">
+      <c r="Y59" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60" spans="1:25">
       <c r="A60" s="5">
         <v>59</v>
       </c>
@@ -5248,35 +5574,41 @@
         <v>12</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J60" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="K60" s="10" t="s">
+        <v>419</v>
+      </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5"/>
-      <c r="N60" s="6" t="s">
+      <c r="N60" s="5"/>
+      <c r="O60" s="5"/>
+      <c r="P60" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O60" s="5" t="s">
+      <c r="Q60" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P60" s="6"/>
-      <c r="Q60" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R60" s="6"/>
-      <c r="S60" s="6"/>
+      <c r="S60" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T60" s="6"/>
       <c r="U60" s="6"/>
-      <c r="V60" s="5" t="str">
+      <c r="V60" s="6"/>
+      <c r="W60" s="6"/>
+      <c r="X60" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/angelo-saavedra.jpg</v>
       </c>
-      <c r="W60" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="61" spans="1:23">
+      <c r="Y60" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="61" spans="1:25">
       <c r="A61" s="5">
         <v>60</v>
       </c>
@@ -5302,37 +5634,39 @@
         <v>244</v>
       </c>
       <c r="I61" s="10" t="s">
-        <v>381</v>
-      </c>
-      <c r="J61" s="5"/>
-      <c r="K61" s="5"/>
+        <v>395</v>
+      </c>
+      <c r="J61" s="10"/>
+      <c r="K61" s="10"/>
       <c r="L61" s="5"/>
       <c r="M61" s="5"/>
-      <c r="N61" s="6" t="s">
+      <c r="N61" s="5"/>
+      <c r="O61" s="5"/>
+      <c r="P61" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O61" s="5" t="s">
+      <c r="Q61" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P61" s="6" t="s">
-        <v>392</v>
-      </c>
-      <c r="Q61" s="6" t="s">
+      <c r="R61" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="S61" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R61" s="6"/>
-      <c r="S61" s="6"/>
       <c r="T61" s="6"/>
       <c r="U61" s="6"/>
-      <c r="V61" s="5" t="str">
+      <c r="V61" s="6"/>
+      <c r="W61" s="6"/>
+      <c r="X61" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/brendel-sacaris.jpg</v>
       </c>
-      <c r="W61" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="62" spans="1:23">
+      <c r="Y61" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:25">
       <c r="A62" s="5">
         <v>61</v>
       </c>
@@ -5358,35 +5692,41 @@
         <v>12</v>
       </c>
       <c r="I62" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J62" s="10" t="s">
+        <v>354</v>
+      </c>
+      <c r="K62" s="10" t="s">
+        <v>420</v>
+      </c>
       <c r="L62" s="5"/>
       <c r="M62" s="5"/>
-      <c r="N62" s="6" t="s">
+      <c r="N62" s="5"/>
+      <c r="O62" s="5"/>
+      <c r="P62" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O62" s="5" t="s">
+      <c r="Q62" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P62" s="6"/>
-      <c r="Q62" s="6" t="s">
-        <v>368</v>
-      </c>
       <c r="R62" s="6"/>
-      <c r="S62" s="6"/>
+      <c r="S62" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T62" s="6"/>
       <c r="U62" s="6"/>
-      <c r="V62" s="5" t="str">
+      <c r="V62" s="6"/>
+      <c r="W62" s="6"/>
+      <c r="X62" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C62&amp;" "&amp;B62)," ","-"))&amp;".jpg"</f>
         <v>/personnel/bella-arquine-samontañez.jpg</v>
       </c>
-      <c r="W62" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="63" spans="1:23">
+      <c r="Y62" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="63" spans="1:25">
       <c r="A63" s="5">
         <v>62</v>
       </c>
@@ -5412,37 +5752,39 @@
         <v>249</v>
       </c>
       <c r="I63" s="10" t="s">
-        <v>368</v>
-      </c>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
+        <v>277</v>
+      </c>
+      <c r="J63" s="10"/>
+      <c r="K63" s="10"/>
       <c r="L63" s="5"/>
       <c r="M63" s="5"/>
-      <c r="N63" s="6" t="s">
+      <c r="N63" s="5"/>
+      <c r="O63" s="5"/>
+      <c r="P63" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O63" s="5" t="s">
+      <c r="Q63" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P63" s="6" t="s">
+      <c r="R63" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="Q63" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="R63" s="6"/>
-      <c r="S63" s="6"/>
+      <c r="S63" s="6" t="s">
+        <v>277</v>
+      </c>
       <c r="T63" s="6"/>
       <c r="U63" s="6"/>
-      <c r="V63" s="5" t="str">
+      <c r="V63" s="6"/>
+      <c r="W63" s="6"/>
+      <c r="X63" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jevy-ann-uy.jpg</v>
       </c>
-      <c r="W63" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:23">
+      <c r="Y63" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="1:25">
       <c r="A64" s="5">
         <v>63</v>
       </c>
@@ -5468,37 +5810,39 @@
         <v>12</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>382</v>
-      </c>
-      <c r="J64" s="5"/>
-      <c r="K64" s="5"/>
+        <v>381</v>
+      </c>
+      <c r="J64" s="10"/>
+      <c r="K64" s="10"/>
       <c r="L64" s="5"/>
       <c r="M64" s="5"/>
-      <c r="N64" s="6" t="s">
+      <c r="N64" s="5"/>
+      <c r="O64" s="5"/>
+      <c r="P64" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O64" s="5" t="s">
+      <c r="Q64" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="P64" s="6" t="s">
+      <c r="R64" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="Q64" s="6" t="s">
+      <c r="S64" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="R64" s="6"/>
-      <c r="S64" s="6"/>
       <c r="T64" s="6"/>
       <c r="U64" s="6"/>
-      <c r="V64" s="5" t="str">
+      <c r="V64" s="6"/>
+      <c r="W64" s="6"/>
+      <c r="X64" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/grace-vergara.jpg</v>
       </c>
-      <c r="W64" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="65" spans="1:23">
+      <c r="Y64" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="1:25">
       <c r="A65" s="5">
         <v>64</v>
       </c>
@@ -5526,35 +5870,37 @@
       <c r="I65" s="10" t="s">
         <v>271</v>
       </c>
-      <c r="J65" s="5"/>
-      <c r="K65" s="5"/>
+      <c r="J65" s="10"/>
+      <c r="K65" s="10"/>
       <c r="L65" s="5"/>
       <c r="M65" s="5"/>
-      <c r="N65" s="6" t="s">
+      <c r="N65" s="5"/>
+      <c r="O65" s="5"/>
+      <c r="P65" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="O65" s="5" t="s">
+      <c r="Q65" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="P65" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q65" s="6" t="s">
+      <c r="R65" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S65" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="R65" s="6"/>
-      <c r="S65" s="6"/>
       <c r="T65" s="6"/>
       <c r="U65" s="6"/>
-      <c r="V65" s="5" t="str">
+      <c r="V65" s="6"/>
+      <c r="W65" s="6"/>
+      <c r="X65" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/guillermo-villavelez.jpg</v>
       </c>
-      <c r="W65" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="66" spans="1:23">
+      <c r="Y65" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="66" spans="1:25">
       <c r="A66" s="5">
         <v>65</v>
       </c>
@@ -5582,35 +5928,37 @@
       <c r="I66" s="10" t="s">
         <v>369</v>
       </c>
-      <c r="J66" s="5"/>
-      <c r="K66" s="5"/>
+      <c r="J66" s="10"/>
+      <c r="K66" s="10"/>
       <c r="L66" s="5"/>
       <c r="M66" s="5"/>
-      <c r="N66" s="6" t="s">
+      <c r="N66" s="5"/>
+      <c r="O66" s="5"/>
+      <c r="P66" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O66" s="5" t="s">
+      <c r="Q66" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P66" s="6" t="s">
+      <c r="R66" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="Q66" s="6" t="s">
+      <c r="S66" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R66" s="6"/>
-      <c r="S66" s="6"/>
       <c r="T66" s="6"/>
       <c r="U66" s="6"/>
-      <c r="V66" s="5" t="str">
+      <c r="V66" s="6"/>
+      <c r="W66" s="6"/>
+      <c r="X66" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marilou-villaver.jpg</v>
       </c>
-      <c r="W66" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="67" spans="1:23">
+      <c r="Y66" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="67" spans="1:25">
       <c r="A67" s="5">
         <v>66</v>
       </c>
@@ -5638,35 +5986,37 @@
       <c r="I67" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="J67" s="5"/>
-      <c r="K67" s="5"/>
+      <c r="J67" s="10"/>
+      <c r="K67" s="10"/>
       <c r="L67" s="5"/>
       <c r="M67" s="5"/>
-      <c r="N67" s="6" t="s">
+      <c r="N67" s="5"/>
+      <c r="O67" s="5"/>
+      <c r="P67" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="O67" s="5" t="s">
+      <c r="Q67" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="P67" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q67" s="6" t="s">
+      <c r="R67" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S67" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="R67" s="6"/>
-      <c r="S67" s="6"/>
       <c r="T67" s="6"/>
       <c r="U67" s="6"/>
-      <c r="V67" s="5" t="str">
-        <f t="shared" ref="V67:V68" si="8">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C67&amp;" "&amp;B67)," ","-"))&amp;".jpg"</f>
+      <c r="V67" s="6"/>
+      <c r="W67" s="6"/>
+      <c r="X67" s="5" t="str">
+        <f t="shared" ref="X67:X68" si="8">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C67&amp;" "&amp;B67)," ","-"))&amp;".jpg"</f>
         <v>/personnel/markjil-bacaltos.jpg</v>
       </c>
-      <c r="W67" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="68" spans="1:23">
+      <c r="Y67" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:25">
       <c r="A68" s="5">
         <v>67</v>
       </c>
@@ -5694,35 +6044,37 @@
       <c r="I68" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="J68" s="5"/>
-      <c r="K68" s="5"/>
+      <c r="J68" s="10"/>
+      <c r="K68" s="10"/>
       <c r="L68" s="5"/>
       <c r="M68" s="5"/>
-      <c r="N68" s="6" t="s">
+      <c r="N68" s="5"/>
+      <c r="O68" s="5"/>
+      <c r="P68" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="O68" s="5" t="s">
+      <c r="Q68" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="P68" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q68" s="6" t="s">
+      <c r="R68" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S68" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="R68" s="6"/>
-      <c r="S68" s="6"/>
       <c r="T68" s="6"/>
       <c r="U68" s="6"/>
-      <c r="V68" s="5" t="str">
+      <c r="V68" s="6"/>
+      <c r="W68" s="6"/>
+      <c r="X68" s="5" t="str">
         <f t="shared" si="8"/>
         <v>/personnel/diocel-celocia.jpg</v>
       </c>
-      <c r="W68" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="69" spans="1:23">
+      <c r="Y68" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:25">
       <c r="A69" s="5">
         <v>68</v>
       </c>
@@ -5750,35 +6102,37 @@
       <c r="I69" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="J69" s="5"/>
-      <c r="K69" s="5"/>
+      <c r="J69" s="10"/>
+      <c r="K69" s="10"/>
       <c r="L69" s="5"/>
       <c r="M69" s="5"/>
-      <c r="N69" s="6" t="s">
+      <c r="N69" s="5"/>
+      <c r="O69" s="5"/>
+      <c r="P69" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="O69" s="5" t="s">
+      <c r="Q69" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="P69" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q69" s="6" t="s">
+      <c r="R69" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S69" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="R69" s="6"/>
-      <c r="S69" s="6"/>
       <c r="T69" s="6"/>
       <c r="U69" s="6"/>
-      <c r="V69" s="5" t="str">
-        <f t="shared" ref="V69:V70" si="11">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C69&amp;" "&amp;B69)," ","-"))&amp;".jpg"</f>
+      <c r="V69" s="6"/>
+      <c r="W69" s="6"/>
+      <c r="X69" s="5" t="str">
+        <f t="shared" ref="X69:X70" si="11">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C69&amp;" "&amp;B69)," ","-"))&amp;".jpg"</f>
         <v>/personnel/luie-cabs.jpg</v>
       </c>
-      <c r="W69" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="70" spans="1:23">
+      <c r="Y69" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="70" spans="1:25">
       <c r="A70" s="5">
         <v>69</v>
       </c>
@@ -5806,35 +6160,37 @@
       <c r="I70" s="10" t="s">
         <v>370</v>
       </c>
-      <c r="J70" s="5"/>
-      <c r="K70" s="5"/>
+      <c r="J70" s="10"/>
+      <c r="K70" s="10"/>
       <c r="L70" s="5"/>
       <c r="M70" s="5"/>
-      <c r="N70" s="6" t="s">
+      <c r="N70" s="5"/>
+      <c r="O70" s="5"/>
+      <c r="P70" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="O70" s="5" t="s">
+      <c r="Q70" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="P70" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="Q70" s="6" t="s">
+      <c r="R70" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="S70" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="R70" s="6"/>
-      <c r="S70" s="6"/>
       <c r="T70" s="6"/>
       <c r="U70" s="6"/>
-      <c r="V70" s="5" t="str">
+      <c r="V70" s="6"/>
+      <c r="W70" s="6"/>
+      <c r="X70" s="5" t="str">
         <f t="shared" si="11"/>
         <v>/personnel/luis-mans.jpg</v>
       </c>
-      <c r="W70" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="71" spans="1:23">
+      <c r="Y70" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="71" spans="1:25">
       <c r="A71" s="5">
         <v>70</v>
       </c>
@@ -5849,20 +6205,22 @@
       <c r="G71" s="5"/>
       <c r="H71" s="5"/>
       <c r="I71" s="9"/>
-      <c r="J71" s="5"/>
-      <c r="K71" s="5"/>
+      <c r="J71" s="9"/>
+      <c r="K71" s="9"/>
       <c r="L71" s="5"/>
       <c r="M71" s="5"/>
-      <c r="N71" s="6"/>
+      <c r="N71" s="5"/>
       <c r="O71" s="5"/>
       <c r="P71" s="6"/>
-      <c r="Q71" s="6"/>
+      <c r="Q71" s="5"/>
       <c r="R71" s="6"/>
       <c r="S71" s="6"/>
       <c r="T71" s="6"/>
       <c r="U71" s="6"/>
-      <c r="V71" s="5"/>
+      <c r="V71" s="6"/>
       <c r="W71" s="6"/>
+      <c r="X71" s="5"/>
+      <c r="Y71" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -5877,13 +6235,13 @@
           <x14:formula1>
             <xm:f>Dropdown_Lists!$A$2:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>N71</xm:sqref>
+          <xm:sqref>P71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{F197BE03-BA33-43F0-8353-14B37878E191}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>N2:N70</xm:sqref>
+          <xm:sqref>P2:P70</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{909FCDCA-C40C-4807-A52A-02A68E381F21}">
           <x14:formula1>
@@ -5895,19 +6253,19 @@
           <x14:formula1>
             <xm:f>Dropdown_Lists!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W71</xm:sqref>
+          <xm:sqref>Y2:Y71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{70D54F6E-2A67-40F0-92CA-B6E53F44843D}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$D$2:$D$61</xm:f>
           </x14:formula1>
-          <xm:sqref>Q2:Q71</xm:sqref>
+          <xm:sqref>S2:S71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7834D497-9733-4178-89DF-4B7895726F53}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$E$2:$E$60</xm:f>
           </x14:formula1>
-          <xm:sqref>R2:R71</xm:sqref>
+          <xm:sqref>T2:T71</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Update organization page personnel display
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5296B38E-E333-4736-B431-660CAEBD597D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFE0AE0-5E41-4065-B58F-FE70AA82722B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="21300" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personnel" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="475">
   <si>
     <t>order</t>
   </si>
@@ -1174,9 +1174,6 @@
     <t>Junior High School In-Charge</t>
   </si>
   <si>
-    <t>BSP Coordinator</t>
-  </si>
-  <si>
     <t>SDRRM Coordinator</t>
   </si>
   <si>
@@ -1195,9 +1192,6 @@
     <t>Math</t>
   </si>
   <si>
-    <t>ICT/Progamming</t>
-  </si>
-  <si>
     <t>N/A</t>
   </si>
   <si>
@@ -1319,6 +1313,153 @@
   </si>
   <si>
     <t>Jupiter, Saturn</t>
+  </si>
+  <si>
+    <t>English 10</t>
+  </si>
+  <si>
+    <t>primarySubjectDepartment</t>
+  </si>
+  <si>
+    <t>subject1</t>
+  </si>
+  <si>
+    <t>subject2</t>
+  </si>
+  <si>
+    <t>subject3</t>
+  </si>
+  <si>
+    <t>subject4</t>
+  </si>
+  <si>
+    <t>subject5</t>
+  </si>
+  <si>
+    <t>teachingLevel</t>
+  </si>
+  <si>
+    <t>JHS/SHS</t>
+  </si>
+  <si>
+    <t>MAPEH 8</t>
+  </si>
+  <si>
+    <t>MAPEH 10</t>
+  </si>
+  <si>
+    <t>Life and Career Skills (LCS 11 - SEM1)</t>
+  </si>
+  <si>
+    <t>Values Education 8</t>
+  </si>
+  <si>
+    <t>School Facilities Assistant Coordinator</t>
+  </si>
+  <si>
+    <t>School Sports Assistant Coordinator</t>
+  </si>
+  <si>
+    <t>Drum Lyre and Majorette Corps Coordinator</t>
+  </si>
+  <si>
+    <t>Values Education 9</t>
+  </si>
+  <si>
+    <t>Technical Professional (Tech Pro)</t>
+  </si>
+  <si>
+    <t>Computer Programming (JAVA)</t>
+  </si>
+  <si>
+    <t>Media and Information Literacy</t>
+  </si>
+  <si>
+    <t>Assistant School Testing Coordinator</t>
+  </si>
+  <si>
+    <t>Assistant SHS ICT Coordinator</t>
+  </si>
+  <si>
+    <t>JHS-TLE Coordinator</t>
+  </si>
+  <si>
+    <t>JHS-ICT Coordinator</t>
+  </si>
+  <si>
+    <t>ESP Coordinator</t>
+  </si>
+  <si>
+    <t>School Religious Act Coordinator</t>
+  </si>
+  <si>
+    <t>Edukasyon sa Pagpapakatao 10</t>
+  </si>
+  <si>
+    <t>Wash in School Coordinator</t>
+  </si>
+  <si>
+    <t>Science 8</t>
+  </si>
+  <si>
+    <t>Boys Scout of the Philippines Coordinator</t>
+  </si>
+  <si>
+    <t>Araling Panlipunan Coordinator (SHS)</t>
+  </si>
+  <si>
+    <t>AP</t>
+  </si>
+  <si>
+    <t>Araling Panlipunan 9</t>
+  </si>
+  <si>
+    <t>Elective 2-Introduction to World Religions and Belief Systems</t>
+  </si>
+  <si>
+    <t>School Health Aide Coordinator (JHS)</t>
+  </si>
+  <si>
+    <t>Technology and Livelihood Education 8 &amp; 9</t>
+  </si>
+  <si>
+    <t>Technology and Livelihood Education 9 &amp; 10</t>
+  </si>
+  <si>
+    <t>Mathematics 9 &amp; 10</t>
+  </si>
+  <si>
+    <t>MAPEH 7 &amp; 10</t>
+  </si>
+  <si>
+    <t>SHS Mathematics Coordinator</t>
+  </si>
+  <si>
+    <t>Mathematics 7 &amp; 8</t>
+  </si>
+  <si>
+    <t>General Mathemathics</t>
+  </si>
+  <si>
+    <t>SHS English Coordinator</t>
+  </si>
+  <si>
+    <t>Learning Action Cell (LAC) Coordinator for SHS</t>
+  </si>
+  <si>
+    <t>Contemporary Philippine Arts from the Regions</t>
+  </si>
+  <si>
+    <t>Research for Daily Life 2</t>
+  </si>
+  <si>
+    <t>SHS Work Immersion Coordinator, Alternate</t>
+  </si>
+  <si>
+    <t>Life and Career Skills</t>
+  </si>
+  <si>
+    <t>English 7 &amp; 8</t>
   </si>
 </sst>
 </file>
@@ -1424,7 +1565,140 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="28">
+  <dxfs count="35">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1871,37 +2145,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:Y71" headerRowDxfId="27" dataDxfId="26" totalsRowDxfId="25">
-  <tableColumns count="25">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="23"/>
-    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="22"/>
-    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:AF71" headerRowDxfId="34" dataDxfId="33" totalsRowDxfId="32">
+  <tableColumns count="32">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="29"/>
+    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="28"/>
+    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="27">
       <calculatedColumnFormula>IF(D2="","",LEFT(TRIM(D2),1)&amp;".")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="19"/>
-    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="18">
+    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="26"/>
+    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="25">
       <calculatedColumnFormula>TRIM(_xlfn.TEXTJOIN(" ",TRUE,C2,IF(E2&lt;&gt;"",IF(RIGHT(E2,1)=".",E2,E2&amp;"."),D2),B2,F2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="17"/>
-    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="16"/>
-    <tableColumn id="24" xr3:uid="{9E70E31F-1B17-4E67-A99E-4037A94153C1}" name="advisoryGradeLevel" dataDxfId="15"/>
-    <tableColumn id="25" xr3:uid="{82F63A8C-E0AF-4172-B1EB-CC758DA39858}" name="advisorySection" dataDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="7"/>
-    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="6"/>
-    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="5"/>
-    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="3"/>
-    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="23"/>
+    <tableColumn id="24" xr3:uid="{9E70E31F-1B17-4E67-A99E-4037A94153C1}" name="advisoryGradeLevel" dataDxfId="22"/>
+    <tableColumn id="25" xr3:uid="{82F63A8C-E0AF-4172-B1EB-CC758DA39858}" name="advisorySection" dataDxfId="21"/>
+    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="20"/>
+    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="19"/>
+    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="18"/>
+    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="14"/>
+    <tableColumn id="26" xr3:uid="{9234D872-27E9-4981-9849-3B92B3D703D7}" name="primarySubjectDepartment" dataDxfId="6"/>
+    <tableColumn id="27" xr3:uid="{BAF0BAF6-D68C-494F-94BF-9DBEAC627028}" name="subject1" dataDxfId="5"/>
+    <tableColumn id="28" xr3:uid="{8B540991-2968-4F70-8AAC-FCFC355A419A}" name="subject2" dataDxfId="4"/>
+    <tableColumn id="29" xr3:uid="{1D6F7D4B-4E56-4246-A153-8FAB0BEB4811}" name="subject3" dataDxfId="3"/>
+    <tableColumn id="30" xr3:uid="{E295C211-F74A-4E2B-893A-E9FDF18B7EE9}" name="subject4" dataDxfId="2"/>
+    <tableColumn id="31" xr3:uid="{B93E7C74-87A6-4CBE-9E54-1C7E4E717375}" name="subject5" dataDxfId="1"/>
+    <tableColumn id="32" xr3:uid="{AE0F403C-1544-4D9E-929C-27676144B2E2}" name="teachingLevel" dataDxfId="0"/>
+    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="13"/>
+    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="12"/>
+    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="11"/>
+    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="10"/>
+    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="9"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="8"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2056,7 +2337,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y71"/>
+  <dimension ref="A1:AF71"/>
   <sheetFormatPr defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="5.59765625" style="4" bestFit="1" customWidth="1"/>
@@ -2075,14 +2356,14 @@
     <col min="15" max="15" width="32.8984375" style="4" customWidth="1"/>
     <col min="16" max="16" width="26.69921875" style="4" customWidth="1"/>
     <col min="17" max="17" width="20.09765625" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="45.19921875" style="7" customWidth="1"/>
-    <col min="19" max="23" width="24.19921875" style="7" customWidth="1"/>
-    <col min="24" max="24" width="36.69921875" style="4" customWidth="1"/>
-    <col min="25" max="25" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="26" max="16384" width="8.796875" style="4"/>
+    <col min="18" max="25" width="45.19921875" style="7" customWidth="1"/>
+    <col min="26" max="30" width="24.19921875" style="7" customWidth="1"/>
+    <col min="31" max="31" width="36.69921875" style="4" customWidth="1"/>
+    <col min="32" max="32" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="33" max="16384" width="8.796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="20.399999999999999" customHeight="1">
+    <row r="1" spans="1:32" ht="20.399999999999999" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -2111,10 +2392,10 @@
         <v>324</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>325</v>
@@ -2138,28 +2419,49 @@
         <v>4</v>
       </c>
       <c r="S1" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>428</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>429</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>431</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>432</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="Z1" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="AA1" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="AB1" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="AC1" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="AD1" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="AF1" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:32">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2202,22 +2504,37 @@
       <c r="R2" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
+      <c r="S2" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>426</v>
+      </c>
       <c r="U2" s="6"/>
-      <c r="V2" s="6">
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
+      <c r="Y2" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z2" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="AA2" s="6"/>
+      <c r="AB2" s="6"/>
+      <c r="AC2" s="6">
         <v>2</v>
       </c>
-      <c r="W2" s="6"/>
-      <c r="X2" s="5" t="str">
+      <c r="AD2" s="6"/>
+      <c r="AE2" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C2&amp;" "&amp;B2)," ","-"))&amp;".jpg"</f>
         <v>/personnel/paz-abad.jpg</v>
       </c>
-      <c r="Y2" s="6" t="s">
+      <c r="AF2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:32">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -2249,7 +2566,7 @@
         <v>353</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
@@ -2265,21 +2582,38 @@
         <v>343</v>
       </c>
       <c r="S3" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="T3" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="U3" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="V3" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="Z3" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="T3" s="6"/>
-      <c r="U3" s="6"/>
-      <c r="V3" s="6"/>
-      <c r="W3" s="6"/>
-      <c r="X3" s="5" t="str">
-        <f t="shared" ref="X3:X66" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C3&amp;" "&amp;B3)," ","-"))&amp;".jpg"</f>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="5" t="str">
+        <f t="shared" ref="AE3:AE66" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C3&amp;" "&amp;B3)," ","-"))&amp;".jpg"</f>
         <v>/personnel/marissa-abalo.jpg</v>
       </c>
-      <c r="Y3" s="6" t="s">
+      <c r="AF3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
+    <row r="4" spans="1:32">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -2304,7 +2638,9 @@
       <c r="H4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I4" s="10"/>
+      <c r="I4" s="10" t="s">
+        <v>439</v>
+      </c>
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
       <c r="L4" s="5"/>
@@ -2318,22 +2654,37 @@
         <v>17</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="S4" s="6"/>
-      <c r="T4" s="6"/>
+        <v>384</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>463</v>
+      </c>
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
       <c r="W4" s="6"/>
-      <c r="X4" s="5" t="str">
+      <c r="X4" s="6"/>
+      <c r="Y4" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z4" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA4" s="6"/>
+      <c r="AB4" s="6"/>
+      <c r="AC4" s="6"/>
+      <c r="AD4" s="6"/>
+      <c r="AE4" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joseph-allosada.jpg</v>
       </c>
-      <c r="Y4" s="6" t="s">
+      <c r="AF4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:32" ht="33.6">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -2365,10 +2716,14 @@
         <v>355</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>399</v>
-      </c>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
+        <v>397</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>441</v>
+      </c>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
       <c r="P5" s="6" t="s">
@@ -2381,21 +2736,36 @@
         <v>343</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T5" s="6"/>
-      <c r="U5" s="6"/>
+        <v>343</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="U5" s="6" t="s">
+        <v>436</v>
+      </c>
       <c r="V5" s="6"/>
       <c r="W5" s="6"/>
-      <c r="X5" s="5" t="str">
+      <c r="X5" s="6"/>
+      <c r="Y5" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z5" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA5" s="6"/>
+      <c r="AB5" s="6"/>
+      <c r="AC5" s="6"/>
+      <c r="AD5" s="6"/>
+      <c r="AE5" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/sharon-gay-alsa.jpg</v>
       </c>
-      <c r="Y5" s="6" t="s">
+      <c r="AF5" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="33.6">
+    <row r="6" spans="1:32" ht="33.6">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -2427,7 +2797,7 @@
         <v>356</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
@@ -2440,24 +2810,39 @@
         <v>14</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>386</v>
+        <v>443</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
+        <v>345</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="U6" s="6" t="s">
+        <v>445</v>
+      </c>
       <c r="V6" s="6"/>
       <c r="W6" s="6"/>
-      <c r="X6" s="5" t="str">
+      <c r="X6" s="6"/>
+      <c r="Y6" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="Z6" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA6" s="6"/>
+      <c r="AB6" s="6"/>
+      <c r="AC6" s="6"/>
+      <c r="AD6" s="6"/>
+      <c r="AE6" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lonier-andrade.jpg</v>
       </c>
-      <c r="Y6" s="6" t="s">
+      <c r="AF6" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:32">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -2489,10 +2874,14 @@
         <v>354</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
+        <v>398</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>447</v>
+      </c>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
       <c r="P7" s="6" t="s">
@@ -2505,21 +2894,34 @@
         <v>344</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T7" s="6"/>
+        <v>344</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>461</v>
+      </c>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
-      <c r="X7" s="5" t="str">
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z7" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA7" s="6"/>
+      <c r="AB7" s="6"/>
+      <c r="AC7" s="6"/>
+      <c r="AD7" s="6"/>
+      <c r="AE7" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/allan-raul-aparicio.jpg</v>
       </c>
-      <c r="Y7" s="6" t="s">
+      <c r="AF7" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:32">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -2558,22 +2960,31 @@
         <v>7</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="S8" s="6"/>
       <c r="T8" s="6"/>
       <c r="U8" s="6"/>
       <c r="V8" s="6"/>
       <c r="W8" s="6"/>
-      <c r="X8" s="5" t="str">
+      <c r="X8" s="6"/>
+      <c r="Y8" s="6"/>
+      <c r="Z8" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="AA8" s="6"/>
+      <c r="AB8" s="6"/>
+      <c r="AC8" s="6"/>
+      <c r="AD8" s="6"/>
+      <c r="AE8" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/niña-kristine-ayos.jpg</v>
       </c>
-      <c r="Y8" s="6" t="s">
+      <c r="AF8" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:32">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -2598,10 +3009,14 @@
       <c r="H9" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="I9" s="10"/>
+      <c r="I9" s="10" t="s">
+        <v>448</v>
+      </c>
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
-      <c r="L9" s="5"/>
+      <c r="L9" s="5" t="s">
+        <v>449</v>
+      </c>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
       <c r="O9" s="5"/>
@@ -2614,20 +3029,35 @@
       <c r="R9" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="S9" s="6"/>
-      <c r="T9" s="6"/>
+      <c r="S9" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>462</v>
+      </c>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
       <c r="W9" s="6"/>
-      <c r="X9" s="5" t="str">
+      <c r="X9" s="6"/>
+      <c r="Y9" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z9" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="AA9" s="6"/>
+      <c r="AB9" s="6"/>
+      <c r="AC9" s="6"/>
+      <c r="AD9" s="6"/>
+      <c r="AE9" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/glenn-barangan.jpg</v>
       </c>
-      <c r="Y9" s="6" t="s">
+      <c r="AF9" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:32">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -2659,10 +3089,14 @@
         <v>355</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>401</v>
-      </c>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
+        <v>399</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>451</v>
+      </c>
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
       <c r="P10" s="6" t="s">
@@ -2672,24 +3106,37 @@
         <v>14</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T10" s="6"/>
+        <v>386</v>
+      </c>
+      <c r="T10" s="6" t="s">
+        <v>452</v>
+      </c>
       <c r="U10" s="6"/>
       <c r="V10" s="6"/>
       <c r="W10" s="6"/>
-      <c r="X10" s="5" t="str">
+      <c r="X10" s="6"/>
+      <c r="Y10" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z10" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA10" s="6"/>
+      <c r="AB10" s="6"/>
+      <c r="AC10" s="6"/>
+      <c r="AD10" s="6"/>
+      <c r="AE10" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jake-barcenas.jpg</v>
       </c>
-      <c r="Y10" s="6" t="s">
+      <c r="AF10" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:32">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -2721,9 +3168,11 @@
         <v>353</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>402</v>
-      </c>
-      <c r="L11" s="5"/>
+        <v>400</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>453</v>
+      </c>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
       <c r="O11" s="5"/>
@@ -2733,23 +3182,38 @@
       <c r="Q11" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="R11" s="6"/>
+      <c r="R11" s="6" t="s">
+        <v>341</v>
+      </c>
       <c r="S11" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T11" s="6"/>
+        <v>341</v>
+      </c>
+      <c r="T11" s="6" t="s">
+        <v>454</v>
+      </c>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
       <c r="W11" s="6"/>
-      <c r="X11" s="5" t="str">
+      <c r="X11" s="6"/>
+      <c r="Y11" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z11" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA11" s="6"/>
+      <c r="AB11" s="6"/>
+      <c r="AC11" s="6"/>
+      <c r="AD11" s="6"/>
+      <c r="AE11" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/eljoy-barroca.jpg</v>
       </c>
-      <c r="Y11" s="6" t="s">
+      <c r="AF11" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:25">
+    <row r="12" spans="1:32" ht="33.6">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -2781,12 +3245,14 @@
         <v>357</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="M12" s="5"/>
+        <v>455</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>456</v>
+      </c>
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
       <c r="P12" s="6" t="s">
@@ -2795,23 +3261,40 @@
       <c r="Q12" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="R12" s="6"/>
+      <c r="R12" s="6" t="s">
+        <v>342</v>
+      </c>
       <c r="S12" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T12" s="6"/>
-      <c r="U12" s="6"/>
+        <v>457</v>
+      </c>
+      <c r="T12" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="U12" s="6" t="s">
+        <v>459</v>
+      </c>
       <c r="V12" s="6"/>
       <c r="W12" s="6"/>
-      <c r="X12" s="5" t="str">
+      <c r="X12" s="6"/>
+      <c r="Y12" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="Z12" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA12" s="6"/>
+      <c r="AB12" s="6"/>
+      <c r="AC12" s="6"/>
+      <c r="AD12" s="6"/>
+      <c r="AE12" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/angel-batuigas.jpg</v>
       </c>
-      <c r="Y12" s="6" t="s">
+      <c r="AF12" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:32">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -2836,7 +3319,9 @@
       <c r="H13" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="I13" s="10"/>
+      <c r="I13" s="10" t="s">
+        <v>460</v>
+      </c>
       <c r="J13" s="10"/>
       <c r="K13" s="10"/>
       <c r="L13" s="5"/>
@@ -2852,20 +3337,35 @@
       <c r="R13" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S13" s="6"/>
-      <c r="T13" s="6"/>
+      <c r="S13" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="T13" s="6" t="s">
+        <v>464</v>
+      </c>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
       <c r="W13" s="6"/>
-      <c r="X13" s="5" t="str">
+      <c r="X13" s="6"/>
+      <c r="Y13" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z13" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA13" s="6"/>
+      <c r="AB13" s="6"/>
+      <c r="AC13" s="6"/>
+      <c r="AD13" s="6"/>
+      <c r="AE13" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/mary-josephine-bawiga.jpg</v>
       </c>
-      <c r="Y13" s="6" t="s">
+      <c r="AF13" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:32">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -2897,9 +3397,11 @@
         <v>352</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>403</v>
-      </c>
-      <c r="L14" s="5"/>
+        <v>401</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>465</v>
+      </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
@@ -2907,27 +3409,42 @@
         <v>13</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="S14" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
+        <v>384</v>
+      </c>
+      <c r="T14" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="U14" s="6" t="s">
+        <v>466</v>
+      </c>
       <c r="V14" s="6"/>
       <c r="W14" s="6"/>
-      <c r="X14" s="5" t="str">
+      <c r="X14" s="6"/>
+      <c r="Y14" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="Z14" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA14" s="6"/>
+      <c r="AB14" s="6"/>
+      <c r="AC14" s="6"/>
+      <c r="AD14" s="6"/>
+      <c r="AE14" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/endrie-bohol.jpg</v>
       </c>
-      <c r="Y14" s="6" t="s">
+      <c r="AF14" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:32" ht="33.6">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -2957,8 +3474,12 @@
       </c>
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="5"/>
+      <c r="L15" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>469</v>
+      </c>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
       <c r="P15" s="6" t="s">
@@ -2968,26 +3489,41 @@
         <v>14</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>385</v>
+        <v>334</v>
       </c>
       <c r="S15" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="U15" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="V15" s="6"/>
+      <c r="W15" s="6"/>
+      <c r="X15" s="6"/>
+      <c r="Y15" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="Z15" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="T15" s="6"/>
-      <c r="U15" s="6"/>
-      <c r="V15" s="6">
+      <c r="AA15" s="6"/>
+      <c r="AB15" s="6"/>
+      <c r="AC15" s="6">
         <v>1</v>
       </c>
-      <c r="W15" s="6"/>
-      <c r="X15" s="5" t="str">
+      <c r="AD15" s="6"/>
+      <c r="AE15" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/maine-bongas.jpg</v>
       </c>
-      <c r="Y15" s="6" t="s">
+      <c r="AF15" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:32" ht="33.6">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -3017,9 +3553,11 @@
         <v>352</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>421</v>
-      </c>
-      <c r="L16" s="5"/>
+        <v>419</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>472</v>
+      </c>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
@@ -3029,23 +3567,40 @@
       <c r="Q16" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="R16" s="6"/>
+      <c r="R16" s="6" t="s">
+        <v>334</v>
+      </c>
       <c r="S16" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="T16" s="6"/>
-      <c r="U16" s="6"/>
+        <v>334</v>
+      </c>
+      <c r="T16" s="6" t="s">
+        <v>473</v>
+      </c>
+      <c r="U16" s="6" t="s">
+        <v>474</v>
+      </c>
       <c r="V16" s="6"/>
       <c r="W16" s="6"/>
-      <c r="X16" s="5" t="str">
+      <c r="X16" s="6"/>
+      <c r="Y16" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="Z16" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA16" s="6"/>
+      <c r="AB16" s="6"/>
+      <c r="AC16" s="6"/>
+      <c r="AD16" s="6"/>
+      <c r="AE16" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/ruth-briones.jpg</v>
       </c>
-      <c r="Y16" s="6" t="s">
+      <c r="AF16" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:25">
+    <row r="17" spans="1:32">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -3089,15 +3644,22 @@
       <c r="U17" s="6"/>
       <c r="V17" s="6"/>
       <c r="W17" s="6"/>
-      <c r="X17" s="5" t="str">
+      <c r="X17" s="6"/>
+      <c r="Y17" s="6"/>
+      <c r="Z17" s="6"/>
+      <c r="AA17" s="6"/>
+      <c r="AB17" s="6"/>
+      <c r="AC17" s="6"/>
+      <c r="AD17" s="6"/>
+      <c r="AE17" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/sharon-broñola.jpg</v>
       </c>
-      <c r="Y17" s="6" t="s">
+      <c r="AF17" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:25">
+    <row r="18" spans="1:32">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -3138,22 +3700,29 @@
         <v>14</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="S18" s="6"/>
       <c r="T18" s="6"/>
       <c r="U18" s="6"/>
       <c r="V18" s="6"/>
       <c r="W18" s="6"/>
-      <c r="X18" s="5" t="str">
+      <c r="X18" s="6"/>
+      <c r="Y18" s="6"/>
+      <c r="Z18" s="6"/>
+      <c r="AA18" s="6"/>
+      <c r="AB18" s="6"/>
+      <c r="AC18" s="6"/>
+      <c r="AD18" s="6"/>
+      <c r="AE18" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joan-cabalda.jpg</v>
       </c>
-      <c r="Y18" s="6" t="s">
+      <c r="AF18" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:25">
+    <row r="19" spans="1:32">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -3179,7 +3748,7 @@
         <v>249</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="J19" s="10"/>
       <c r="K19" s="10"/>
@@ -3196,22 +3765,29 @@
       <c r="R19" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S19" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="S19" s="6"/>
       <c r="T19" s="6"/>
       <c r="U19" s="6"/>
       <c r="V19" s="6"/>
       <c r="W19" s="6"/>
-      <c r="X19" s="5" t="str">
+      <c r="X19" s="6"/>
+      <c r="Y19" s="6"/>
+      <c r="Z19" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA19" s="6"/>
+      <c r="AB19" s="6"/>
+      <c r="AC19" s="6"/>
+      <c r="AD19" s="6"/>
+      <c r="AE19" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/gracelyn-cabunag.jpg</v>
       </c>
-      <c r="Y19" s="6" t="s">
+      <c r="AF19" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:25">
+    <row r="20" spans="1:32">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -3257,19 +3833,26 @@
       <c r="S20" s="6"/>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
-      <c r="V20" s="6">
+      <c r="V20" s="6"/>
+      <c r="W20" s="6"/>
+      <c r="X20" s="6"/>
+      <c r="Y20" s="6"/>
+      <c r="Z20" s="6"/>
+      <c r="AA20" s="6"/>
+      <c r="AB20" s="6"/>
+      <c r="AC20" s="6">
         <v>3</v>
       </c>
-      <c r="W20" s="6"/>
-      <c r="X20" s="5" t="str">
+      <c r="AD20" s="6"/>
+      <c r="AE20" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/hector-cabanca.jpg</v>
       </c>
-      <c r="Y20" s="6" t="s">
+      <c r="AF20" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:25">
+    <row r="21" spans="1:32">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -3301,7 +3884,7 @@
         <v>354</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
@@ -3316,22 +3899,29 @@
       <c r="R21" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S21" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S21" s="6"/>
       <c r="T21" s="6"/>
       <c r="U21" s="6"/>
       <c r="V21" s="6"/>
       <c r="W21" s="6"/>
-      <c r="X21" s="5" t="str">
+      <c r="X21" s="6"/>
+      <c r="Y21" s="6"/>
+      <c r="Z21" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA21" s="6"/>
+      <c r="AB21" s="6"/>
+      <c r="AC21" s="6"/>
+      <c r="AD21" s="6"/>
+      <c r="AE21" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeffrey-caberte.jpg</v>
       </c>
-      <c r="Y21" s="6" t="s">
+      <c r="AF21" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:25">
+    <row r="22" spans="1:32">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -3363,7 +3953,7 @@
         <v>355</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
@@ -3376,22 +3966,29 @@
         <v>17</v>
       </c>
       <c r="R22" s="6"/>
-      <c r="S22" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S22" s="6"/>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
       <c r="V22" s="6"/>
       <c r="W22" s="6"/>
-      <c r="X22" s="5" t="str">
+      <c r="X22" s="6"/>
+      <c r="Y22" s="6"/>
+      <c r="Z22" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA22" s="6"/>
+      <c r="AB22" s="6"/>
+      <c r="AC22" s="6"/>
+      <c r="AD22" s="6"/>
+      <c r="AE22" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marilou-cabriana.jpg</v>
       </c>
-      <c r="Y22" s="6" t="s">
+      <c r="AF22" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:25">
+    <row r="23" spans="1:32">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -3432,24 +4029,31 @@
         <v>7</v>
       </c>
       <c r="R23" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S23" s="6" t="s">
-        <v>364</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S23" s="6"/>
       <c r="T23" s="6"/>
       <c r="U23" s="6"/>
       <c r="V23" s="6"/>
       <c r="W23" s="6"/>
-      <c r="X23" s="5" t="str">
+      <c r="X23" s="6"/>
+      <c r="Y23" s="6"/>
+      <c r="Z23" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="AA23" s="6"/>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+      <c r="AD23" s="6"/>
+      <c r="AE23" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jasmin-cabuenas.jpg</v>
       </c>
-      <c r="Y23" s="6" t="s">
+      <c r="AF23" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:25">
+    <row r="24" spans="1:32">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -3475,7 +4079,7 @@
         <v>12</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>
@@ -3492,22 +4096,29 @@
       <c r="R24" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S24" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S24" s="6"/>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
       <c r="W24" s="6"/>
-      <c r="X24" s="5" t="str">
+      <c r="X24" s="6"/>
+      <c r="Y24" s="6"/>
+      <c r="Z24" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA24" s="6"/>
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+      <c r="AD24" s="6"/>
+      <c r="AE24" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/elsa-calunod.jpg</v>
       </c>
-      <c r="Y24" s="6" t="s">
+      <c r="AF24" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:25">
+    <row r="25" spans="1:32">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -3539,7 +4150,7 @@
         <v>352</v>
       </c>
       <c r="K25" s="10" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
@@ -3554,22 +4165,29 @@
       <c r="R25" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S25" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S25" s="6"/>
       <c r="T25" s="6"/>
       <c r="U25" s="6"/>
       <c r="V25" s="6"/>
       <c r="W25" s="6"/>
-      <c r="X25" s="5" t="str">
+      <c r="X25" s="6"/>
+      <c r="Y25" s="6"/>
+      <c r="Z25" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA25" s="6"/>
+      <c r="AB25" s="6"/>
+      <c r="AC25" s="6"/>
+      <c r="AD25" s="6"/>
+      <c r="AE25" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/leslyn-rose-camero.jpg</v>
       </c>
-      <c r="Y25" s="6" t="s">
+      <c r="AF25" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:25">
+    <row r="26" spans="1:32">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -3610,24 +4228,31 @@
         <v>17</v>
       </c>
       <c r="R26" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S26" s="6" t="s">
-        <v>364</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S26" s="6"/>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
       <c r="W26" s="6"/>
-      <c r="X26" s="5" t="str">
+      <c r="X26" s="6"/>
+      <c r="Y26" s="6"/>
+      <c r="Z26" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="AA26" s="6"/>
+      <c r="AB26" s="6"/>
+      <c r="AC26" s="6"/>
+      <c r="AD26" s="6"/>
+      <c r="AE26" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/dawn-camille-caparida.jpg</v>
       </c>
-      <c r="Y26" s="6" t="s">
+      <c r="AF26" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:25">
+    <row r="27" spans="1:32">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -3657,7 +4282,7 @@
         <v>354</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
@@ -3670,24 +4295,31 @@
         <v>17</v>
       </c>
       <c r="R27" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="S27" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="S27" s="6"/>
       <c r="T27" s="6"/>
       <c r="U27" s="6"/>
       <c r="V27" s="6"/>
       <c r="W27" s="6"/>
-      <c r="X27" s="5" t="str">
+      <c r="X27" s="6"/>
+      <c r="Y27" s="6"/>
+      <c r="Z27" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA27" s="6"/>
+      <c r="AB27" s="6"/>
+      <c r="AC27" s="6"/>
+      <c r="AD27" s="6"/>
+      <c r="AE27" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lourence-capa.jpg</v>
       </c>
-      <c r="Y27" s="6" t="s">
+      <c r="AF27" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:25">
+    <row r="28" spans="1:32">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -3719,7 +4351,7 @@
         <v>355</v>
       </c>
       <c r="K28" s="10" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
@@ -3734,22 +4366,29 @@
       <c r="R28" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S28" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S28" s="6"/>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
       <c r="W28" s="6"/>
-      <c r="X28" s="5" t="str">
+      <c r="X28" s="6"/>
+      <c r="Y28" s="6"/>
+      <c r="Z28" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA28" s="6"/>
+      <c r="AB28" s="6"/>
+      <c r="AC28" s="6"/>
+      <c r="AD28" s="6"/>
+      <c r="AE28" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joan-cavite.jpg</v>
       </c>
-      <c r="Y28" s="6" t="s">
+      <c r="AF28" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:25" ht="33.6">
+    <row r="29" spans="1:32" ht="33.6">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -3783,7 +4422,7 @@
         <v>356</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -3796,24 +4435,31 @@
         <v>14</v>
       </c>
       <c r="R29" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="S29" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="S29" s="6"/>
       <c r="T29" s="6"/>
       <c r="U29" s="6"/>
       <c r="V29" s="6"/>
       <c r="W29" s="6"/>
-      <c r="X29" s="5" t="str">
+      <c r="X29" s="6"/>
+      <c r="Y29" s="6"/>
+      <c r="Z29" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA29" s="6"/>
+      <c r="AB29" s="6"/>
+      <c r="AC29" s="6"/>
+      <c r="AD29" s="6"/>
+      <c r="AE29" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joseph-dagaraga.jpg</v>
       </c>
-      <c r="Y29" s="6" t="s">
+      <c r="AF29" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:25">
+    <row r="30" spans="1:32">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -3856,22 +4502,29 @@
       <c r="R30" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S30" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S30" s="6"/>
       <c r="T30" s="6"/>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
       <c r="W30" s="6"/>
-      <c r="X30" s="5" t="str">
+      <c r="X30" s="6"/>
+      <c r="Y30" s="6"/>
+      <c r="Z30" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA30" s="6"/>
+      <c r="AB30" s="6"/>
+      <c r="AC30" s="6"/>
+      <c r="AD30" s="6"/>
+      <c r="AE30" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carolyn-delos-reyes.jpg</v>
       </c>
-      <c r="Y30" s="6" t="s">
+      <c r="AF30" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:25">
+    <row r="31" spans="1:32">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -3914,22 +4567,29 @@
       <c r="R31" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S31" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S31" s="6"/>
       <c r="T31" s="6"/>
       <c r="U31" s="6"/>
       <c r="V31" s="6"/>
       <c r="W31" s="6"/>
-      <c r="X31" s="5" t="str">
+      <c r="X31" s="6"/>
+      <c r="Y31" s="6"/>
+      <c r="Z31" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA31" s="6"/>
+      <c r="AB31" s="6"/>
+      <c r="AC31" s="6"/>
+      <c r="AD31" s="6"/>
+      <c r="AE31" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lucille-echavez.jpg</v>
       </c>
-      <c r="Y31" s="6" t="s">
+      <c r="AF31" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:25">
+    <row r="32" spans="1:32">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -3970,24 +4630,31 @@
         <v>14</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="S32" s="6" t="s">
-        <v>365</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="S32" s="6"/>
       <c r="T32" s="6"/>
       <c r="U32" s="6"/>
       <c r="V32" s="6"/>
       <c r="W32" s="6"/>
-      <c r="X32" s="5" t="str">
+      <c r="X32" s="6"/>
+      <c r="Y32" s="6"/>
+      <c r="Z32" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA32" s="6"/>
+      <c r="AB32" s="6"/>
+      <c r="AC32" s="6"/>
+      <c r="AD32" s="6"/>
+      <c r="AE32" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/benerando-erediano.jpg</v>
       </c>
-      <c r="Y32" s="6" t="s">
+      <c r="AF32" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:25">
+    <row r="33" spans="1:32">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -4013,7 +4680,7 @@
         <v>244</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="J33" s="10"/>
       <c r="K33" s="10"/>
@@ -4030,24 +4697,31 @@
       <c r="R33" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S33" s="6" t="s">
-        <v>367</v>
-      </c>
+      <c r="S33" s="6"/>
       <c r="T33" s="6"/>
       <c r="U33" s="6"/>
-      <c r="V33" s="6">
+      <c r="V33" s="6"/>
+      <c r="W33" s="6"/>
+      <c r="X33" s="6"/>
+      <c r="Y33" s="6"/>
+      <c r="Z33" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="AA33" s="6"/>
+      <c r="AB33" s="6"/>
+      <c r="AC33" s="6">
         <v>4</v>
       </c>
-      <c r="W33" s="6"/>
-      <c r="X33" s="5" t="str">
+      <c r="AD33" s="6"/>
+      <c r="AE33" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/metchie-gay-gastanes.jpg</v>
       </c>
-      <c r="Y33" s="6" t="s">
+      <c r="AF33" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:25">
+    <row r="34" spans="1:32">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -4073,7 +4747,7 @@
         <v>12</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="J34" s="10"/>
       <c r="K34" s="10"/>
@@ -4090,22 +4764,29 @@
       <c r="R34" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="S34" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="S34" s="6"/>
       <c r="T34" s="6"/>
       <c r="U34" s="6"/>
       <c r="V34" s="6"/>
       <c r="W34" s="6"/>
-      <c r="X34" s="5" t="str">
+      <c r="X34" s="6"/>
+      <c r="Y34" s="6"/>
+      <c r="Z34" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA34" s="6"/>
+      <c r="AB34" s="6"/>
+      <c r="AC34" s="6"/>
+      <c r="AD34" s="6"/>
+      <c r="AE34" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jasmin-gerodias.jpg</v>
       </c>
-      <c r="Y34" s="6" t="s">
+      <c r="AF34" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:25">
+    <row r="35" spans="1:32">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -4137,7 +4818,7 @@
         <v>353</v>
       </c>
       <c r="K35" s="10" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
@@ -4152,22 +4833,29 @@
       <c r="R35" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S35" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S35" s="6"/>
       <c r="T35" s="6"/>
       <c r="U35" s="6"/>
       <c r="V35" s="6"/>
       <c r="W35" s="6"/>
-      <c r="X35" s="5" t="str">
+      <c r="X35" s="6"/>
+      <c r="Y35" s="6"/>
+      <c r="Z35" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA35" s="6"/>
+      <c r="AB35" s="6"/>
+      <c r="AC35" s="6"/>
+      <c r="AD35" s="6"/>
+      <c r="AE35" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeralyn-gerra.jpg</v>
       </c>
-      <c r="Y35" s="6" t="s">
+      <c r="AF35" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:25">
+    <row r="36" spans="1:32">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -4199,7 +4887,7 @@
         <v>353</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
@@ -4214,22 +4902,29 @@
       <c r="R36" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S36" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S36" s="6"/>
       <c r="T36" s="6"/>
       <c r="U36" s="6"/>
       <c r="V36" s="6"/>
       <c r="W36" s="6"/>
-      <c r="X36" s="5" t="str">
+      <c r="X36" s="6"/>
+      <c r="Y36" s="6"/>
+      <c r="Z36" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA36" s="6"/>
+      <c r="AB36" s="6"/>
+      <c r="AC36" s="6"/>
+      <c r="AD36" s="6"/>
+      <c r="AE36" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/genesa-goc-ong.jpg</v>
       </c>
-      <c r="Y36" s="6" t="s">
+      <c r="AF36" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:25">
+    <row r="37" spans="1:32">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -4272,22 +4967,29 @@
       <c r="R37" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S37" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S37" s="6"/>
       <c r="T37" s="6"/>
       <c r="U37" s="6"/>
       <c r="V37" s="6"/>
       <c r="W37" s="6"/>
-      <c r="X37" s="5" t="str">
+      <c r="X37" s="6"/>
+      <c r="Y37" s="6"/>
+      <c r="Z37" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA37" s="6"/>
+      <c r="AB37" s="6"/>
+      <c r="AC37" s="6"/>
+      <c r="AD37" s="6"/>
+      <c r="AE37" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/janelou-gomez.jpg</v>
       </c>
-      <c r="Y37" s="6" t="s">
+      <c r="AF37" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:25">
+    <row r="38" spans="1:32">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -4319,7 +5021,7 @@
         <v>352</v>
       </c>
       <c r="K38" s="10" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
@@ -4334,22 +5036,29 @@
       <c r="R38" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S38" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S38" s="6"/>
       <c r="T38" s="6"/>
       <c r="U38" s="6"/>
       <c r="V38" s="6"/>
       <c r="W38" s="6"/>
-      <c r="X38" s="5" t="str">
+      <c r="X38" s="6"/>
+      <c r="Y38" s="6"/>
+      <c r="Z38" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA38" s="6"/>
+      <c r="AB38" s="6"/>
+      <c r="AC38" s="6"/>
+      <c r="AD38" s="6"/>
+      <c r="AE38" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/junnelyn-herbito.jpg</v>
       </c>
-      <c r="Y38" s="6" t="s">
+      <c r="AF38" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:25">
+    <row r="39" spans="1:32">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -4381,7 +5090,7 @@
         <v>355</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -4396,22 +5105,29 @@
       <c r="R39" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S39" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S39" s="6"/>
       <c r="T39" s="6"/>
       <c r="U39" s="6"/>
       <c r="V39" s="6"/>
       <c r="W39" s="6"/>
-      <c r="X39" s="5" t="str">
+      <c r="X39" s="6"/>
+      <c r="Y39" s="6"/>
+      <c r="Z39" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA39" s="6"/>
+      <c r="AB39" s="6"/>
+      <c r="AC39" s="6"/>
+      <c r="AD39" s="6"/>
+      <c r="AE39" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/roxan-mae-jao.jpg</v>
       </c>
-      <c r="Y39" s="6" t="s">
+      <c r="AF39" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:25">
+    <row r="40" spans="1:32">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -4452,22 +5168,29 @@
         <v>17</v>
       </c>
       <c r="R40" s="6"/>
-      <c r="S40" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S40" s="6"/>
       <c r="T40" s="6"/>
       <c r="U40" s="6"/>
       <c r="V40" s="6"/>
       <c r="W40" s="6"/>
-      <c r="X40" s="5" t="str">
+      <c r="X40" s="6"/>
+      <c r="Y40" s="6"/>
+      <c r="Z40" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA40" s="6"/>
+      <c r="AB40" s="6"/>
+      <c r="AC40" s="6"/>
+      <c r="AD40" s="6"/>
+      <c r="AE40" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/fernando-laspiñas.jpg</v>
       </c>
-      <c r="Y40" s="6" t="s">
+      <c r="AF40" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:25">
+    <row r="41" spans="1:32">
       <c r="A41" s="5">
         <v>40</v>
       </c>
@@ -4510,22 +5233,29 @@
       <c r="R41" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S41" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S41" s="6"/>
       <c r="T41" s="6"/>
       <c r="U41" s="6"/>
       <c r="V41" s="6"/>
       <c r="W41" s="6"/>
-      <c r="X41" s="5" t="str">
+      <c r="X41" s="6"/>
+      <c r="Y41" s="6"/>
+      <c r="Z41" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA41" s="6"/>
+      <c r="AB41" s="6"/>
+      <c r="AC41" s="6"/>
+      <c r="AD41" s="6"/>
+      <c r="AE41" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/nerisa-lim.jpg</v>
       </c>
-      <c r="Y41" s="6" t="s">
+      <c r="AF41" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:25">
+    <row r="42" spans="1:32">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -4564,22 +5294,29 @@
         <v>17</v>
       </c>
       <c r="R42" s="6"/>
-      <c r="S42" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S42" s="6"/>
       <c r="T42" s="6"/>
       <c r="U42" s="6"/>
       <c r="V42" s="6"/>
       <c r="W42" s="6"/>
-      <c r="X42" s="5" t="str">
+      <c r="X42" s="6"/>
+      <c r="Y42" s="6"/>
+      <c r="Z42" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA42" s="6"/>
+      <c r="AB42" s="6"/>
+      <c r="AC42" s="6"/>
+      <c r="AD42" s="6"/>
+      <c r="AE42" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carl-loreto.jpg</v>
       </c>
-      <c r="Y42" s="6" t="s">
+      <c r="AF42" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:25">
+    <row r="43" spans="1:32">
       <c r="A43" s="5">
         <v>42</v>
       </c>
@@ -4605,7 +5342,7 @@
         <v>270</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="J43" s="10"/>
       <c r="K43" s="10"/>
@@ -4620,22 +5357,29 @@
         <v>14</v>
       </c>
       <c r="R43" s="6"/>
-      <c r="S43" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="S43" s="6"/>
       <c r="T43" s="6"/>
       <c r="U43" s="6"/>
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
-      <c r="X43" s="5" t="str">
+      <c r="X43" s="6"/>
+      <c r="Y43" s="6"/>
+      <c r="Z43" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA43" s="6"/>
+      <c r="AB43" s="6"/>
+      <c r="AC43" s="6"/>
+      <c r="AD43" s="6"/>
+      <c r="AE43" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lyka-mabanag.jpg</v>
       </c>
-      <c r="Y43" s="6" t="s">
+      <c r="AF43" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:25">
+    <row r="44" spans="1:32">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -4661,7 +5405,7 @@
         <v>250</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="J44" s="10"/>
       <c r="K44" s="10"/>
@@ -4682,22 +5426,29 @@
       <c r="R44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="S44" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="S44" s="6"/>
       <c r="T44" s="6"/>
       <c r="U44" s="6"/>
       <c r="V44" s="6"/>
       <c r="W44" s="6"/>
-      <c r="X44" s="5" t="str">
+      <c r="X44" s="6"/>
+      <c r="Y44" s="6"/>
+      <c r="Z44" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA44" s="6"/>
+      <c r="AB44" s="6"/>
+      <c r="AC44" s="6"/>
+      <c r="AD44" s="6"/>
+      <c r="AE44" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/richie-ryan-mabunay.jpg</v>
       </c>
-      <c r="Y44" s="6" t="s">
+      <c r="AF44" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:25">
+    <row r="45" spans="1:32">
       <c r="A45" s="5">
         <v>44</v>
       </c>
@@ -4740,22 +5491,29 @@
       <c r="R45" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S45" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S45" s="6"/>
       <c r="T45" s="6"/>
       <c r="U45" s="6"/>
       <c r="V45" s="6"/>
       <c r="W45" s="6"/>
-      <c r="X45" s="5" t="str">
+      <c r="X45" s="6"/>
+      <c r="Y45" s="6"/>
+      <c r="Z45" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA45" s="6"/>
+      <c r="AB45" s="6"/>
+      <c r="AC45" s="6"/>
+      <c r="AD45" s="6"/>
+      <c r="AE45" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/maria-jeziel-macanin.jpg</v>
       </c>
-      <c r="Y45" s="6" t="s">
+      <c r="AF45" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:25">
+    <row r="46" spans="1:32">
       <c r="A46" s="5">
         <v>45</v>
       </c>
@@ -4787,7 +5545,7 @@
         <v>354</v>
       </c>
       <c r="K46" s="10" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
@@ -4802,22 +5560,29 @@
       <c r="R46" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S46" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S46" s="6"/>
       <c r="T46" s="6"/>
       <c r="U46" s="6"/>
       <c r="V46" s="6"/>
       <c r="W46" s="6"/>
-      <c r="X46" s="5" t="str">
+      <c r="X46" s="6"/>
+      <c r="Y46" s="6"/>
+      <c r="Z46" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA46" s="6"/>
+      <c r="AB46" s="6"/>
+      <c r="AC46" s="6"/>
+      <c r="AD46" s="6"/>
+      <c r="AE46" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeralen-maloloy-on.jpg</v>
       </c>
-      <c r="Y46" s="6" t="s">
+      <c r="AF46" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:25">
+    <row r="47" spans="1:32">
       <c r="A47" s="5">
         <v>46</v>
       </c>
@@ -4849,7 +5614,7 @@
         <v>352</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
@@ -4864,22 +5629,29 @@
       <c r="R47" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S47" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S47" s="6"/>
       <c r="T47" s="6"/>
       <c r="U47" s="6"/>
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
-      <c r="X47" s="5" t="str">
+      <c r="X47" s="6"/>
+      <c r="Y47" s="6"/>
+      <c r="Z47" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA47" s="6"/>
+      <c r="AB47" s="6"/>
+      <c r="AC47" s="6"/>
+      <c r="AD47" s="6"/>
+      <c r="AE47" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/elbert-misterio.jpg</v>
       </c>
-      <c r="Y47" s="6" t="s">
+      <c r="AF47" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:25">
+    <row r="48" spans="1:32">
       <c r="A48" s="5">
         <v>47</v>
       </c>
@@ -4911,7 +5683,7 @@
         <v>353</v>
       </c>
       <c r="K48" s="10" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
@@ -4924,22 +5696,29 @@
         <v>17</v>
       </c>
       <c r="R48" s="6"/>
-      <c r="S48" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S48" s="6"/>
       <c r="T48" s="6"/>
       <c r="U48" s="6"/>
       <c r="V48" s="6"/>
       <c r="W48" s="6"/>
-      <c r="X48" s="5" t="str">
+      <c r="X48" s="6"/>
+      <c r="Y48" s="6"/>
+      <c r="Z48" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA48" s="6"/>
+      <c r="AB48" s="6"/>
+      <c r="AC48" s="6"/>
+      <c r="AD48" s="6"/>
+      <c r="AE48" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joy-mortal.jpg</v>
       </c>
-      <c r="Y48" s="6" t="s">
+      <c r="AF48" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:25">
+    <row r="49" spans="1:32">
       <c r="A49" s="5">
         <v>48</v>
       </c>
@@ -4980,22 +5759,29 @@
         <v>17</v>
       </c>
       <c r="R49" s="6"/>
-      <c r="S49" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S49" s="6"/>
       <c r="T49" s="6"/>
       <c r="U49" s="6"/>
       <c r="V49" s="6"/>
       <c r="W49" s="6"/>
-      <c r="X49" s="5" t="str">
+      <c r="X49" s="6"/>
+      <c r="Y49" s="6"/>
+      <c r="Z49" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA49" s="6"/>
+      <c r="AB49" s="6"/>
+      <c r="AC49" s="6"/>
+      <c r="AD49" s="6"/>
+      <c r="AE49" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/claire-medillo.jpg</v>
       </c>
-      <c r="Y49" s="6" t="s">
+      <c r="AF49" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:25">
+    <row r="50" spans="1:32">
       <c r="A50" s="5">
         <v>49</v>
       </c>
@@ -5027,7 +5813,7 @@
         <v>352</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
@@ -5042,22 +5828,29 @@
       <c r="R50" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S50" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S50" s="6"/>
       <c r="T50" s="6"/>
       <c r="U50" s="6"/>
       <c r="V50" s="6"/>
       <c r="W50" s="6"/>
-      <c r="X50" s="5" t="str">
+      <c r="X50" s="6"/>
+      <c r="Y50" s="6"/>
+      <c r="Z50" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA50" s="6"/>
+      <c r="AB50" s="6"/>
+      <c r="AC50" s="6"/>
+      <c r="AD50" s="6"/>
+      <c r="AE50" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/gwendolyn-olo.jpg</v>
       </c>
-      <c r="Y50" s="6" t="s">
+      <c r="AF50" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:25">
+    <row r="51" spans="1:32">
       <c r="A51" s="5">
         <v>50</v>
       </c>
@@ -5089,7 +5882,7 @@
         <v>355</v>
       </c>
       <c r="K51" s="10" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
@@ -5102,22 +5895,29 @@
         <v>17</v>
       </c>
       <c r="R51" s="6"/>
-      <c r="S51" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S51" s="6"/>
       <c r="T51" s="6"/>
       <c r="U51" s="6"/>
       <c r="V51" s="6"/>
       <c r="W51" s="6"/>
-      <c r="X51" s="5" t="str">
+      <c r="X51" s="6"/>
+      <c r="Y51" s="6"/>
+      <c r="Z51" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA51" s="6"/>
+      <c r="AB51" s="6"/>
+      <c r="AC51" s="6"/>
+      <c r="AD51" s="6"/>
+      <c r="AE51" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jay-neil-oro.jpg</v>
       </c>
-      <c r="Y51" s="6" t="s">
+      <c r="AF51" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:25">
+    <row r="52" spans="1:32">
       <c r="A52" s="5">
         <v>51</v>
       </c>
@@ -5149,7 +5949,7 @@
         <v>357</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
@@ -5162,24 +5962,31 @@
         <v>14</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>390</v>
-      </c>
-      <c r="S52" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>388</v>
+      </c>
+      <c r="S52" s="6"/>
       <c r="T52" s="6"/>
       <c r="U52" s="6"/>
       <c r="V52" s="6"/>
       <c r="W52" s="6"/>
-      <c r="X52" s="5" t="str">
+      <c r="X52" s="6"/>
+      <c r="Y52" s="6"/>
+      <c r="Z52" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA52" s="6"/>
+      <c r="AB52" s="6"/>
+      <c r="AC52" s="6"/>
+      <c r="AD52" s="6"/>
+      <c r="AE52" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/glendale-orocay.jpg</v>
       </c>
-      <c r="Y52" s="6" t="s">
+      <c r="AF52" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:25" ht="33.6">
+    <row r="53" spans="1:32" ht="33.6">
       <c r="A53" s="5">
         <v>52</v>
       </c>
@@ -5211,7 +6018,7 @@
         <v>356</v>
       </c>
       <c r="K53" s="10" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="L53" s="5"/>
       <c r="M53" s="5"/>
@@ -5224,24 +6031,31 @@
         <v>17</v>
       </c>
       <c r="R53" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="S53" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="S53" s="6"/>
       <c r="T53" s="6"/>
       <c r="U53" s="6"/>
       <c r="V53" s="6"/>
       <c r="W53" s="6"/>
-      <c r="X53" s="5" t="str">
+      <c r="X53" s="6"/>
+      <c r="Y53" s="6"/>
+      <c r="Z53" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA53" s="6"/>
+      <c r="AB53" s="6"/>
+      <c r="AC53" s="6"/>
+      <c r="AD53" s="6"/>
+      <c r="AE53" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marissa-pintuan.jpg</v>
       </c>
-      <c r="Y53" s="6" t="s">
+      <c r="AF53" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:25">
+    <row r="54" spans="1:32">
       <c r="A54" s="5">
         <v>53</v>
       </c>
@@ -5282,24 +6096,31 @@
         <v>17</v>
       </c>
       <c r="R54" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="S54" s="6" t="s">
-        <v>369</v>
-      </c>
+        <v>386</v>
+      </c>
+      <c r="S54" s="6"/>
       <c r="T54" s="6"/>
       <c r="U54" s="6"/>
       <c r="V54" s="6"/>
       <c r="W54" s="6"/>
-      <c r="X54" s="5" t="str">
+      <c r="X54" s="6"/>
+      <c r="Y54" s="6"/>
+      <c r="Z54" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA54" s="6"/>
+      <c r="AB54" s="6"/>
+      <c r="AC54" s="6"/>
+      <c r="AD54" s="6"/>
+      <c r="AE54" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/ma.-lourdes-prajes.jpg</v>
       </c>
-      <c r="Y54" s="6" t="s">
+      <c r="AF54" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:25">
+    <row r="55" spans="1:32">
       <c r="A55" s="5">
         <v>54</v>
       </c>
@@ -5331,7 +6152,7 @@
         <v>353</v>
       </c>
       <c r="K55" s="10" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
@@ -5344,22 +6165,29 @@
         <v>17</v>
       </c>
       <c r="R55" s="6"/>
-      <c r="S55" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S55" s="6"/>
       <c r="T55" s="6"/>
       <c r="U55" s="6"/>
       <c r="V55" s="6"/>
       <c r="W55" s="6"/>
-      <c r="X55" s="5" t="str">
+      <c r="X55" s="6"/>
+      <c r="Y55" s="6"/>
+      <c r="Z55" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA55" s="6"/>
+      <c r="AB55" s="6"/>
+      <c r="AC55" s="6"/>
+      <c r="AD55" s="6"/>
+      <c r="AE55" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/bret-kalvin-primacio.jpg</v>
       </c>
-      <c r="Y55" s="6" t="s">
+      <c r="AF55" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:25">
+    <row r="56" spans="1:32">
       <c r="A56" s="5">
         <v>55</v>
       </c>
@@ -5402,22 +6230,29 @@
       <c r="R56" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S56" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S56" s="6"/>
       <c r="T56" s="6"/>
       <c r="U56" s="6"/>
       <c r="V56" s="6"/>
       <c r="W56" s="6"/>
-      <c r="X56" s="5" t="str">
+      <c r="X56" s="6"/>
+      <c r="Y56" s="6"/>
+      <c r="Z56" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA56" s="6"/>
+      <c r="AB56" s="6"/>
+      <c r="AC56" s="6"/>
+      <c r="AD56" s="6"/>
+      <c r="AE56" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jhea-quiling.jpg</v>
       </c>
-      <c r="Y56" s="6" t="s">
+      <c r="AF56" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:25">
+    <row r="57" spans="1:32">
       <c r="A57" s="5">
         <v>56</v>
       </c>
@@ -5460,22 +6295,29 @@
       <c r="R57" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S57" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S57" s="6"/>
       <c r="T57" s="6"/>
       <c r="U57" s="6"/>
       <c r="V57" s="6"/>
       <c r="W57" s="6"/>
-      <c r="X57" s="5" t="str">
+      <c r="X57" s="6"/>
+      <c r="Y57" s="6"/>
+      <c r="Z57" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA57" s="6"/>
+      <c r="AB57" s="6"/>
+      <c r="AC57" s="6"/>
+      <c r="AD57" s="6"/>
+      <c r="AE57" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joyce-racaza.jpg</v>
       </c>
-      <c r="Y57" s="6" t="s">
+      <c r="AF57" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:25">
+    <row r="58" spans="1:32">
       <c r="A58" s="5">
         <v>57</v>
       </c>
@@ -5518,22 +6360,29 @@
       <c r="R58" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="S58" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S58" s="6"/>
       <c r="T58" s="6"/>
       <c r="U58" s="6"/>
       <c r="V58" s="6"/>
       <c r="W58" s="6"/>
-      <c r="X58" s="5" t="str">
+      <c r="X58" s="6"/>
+      <c r="Y58" s="6"/>
+      <c r="Z58" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA58" s="6"/>
+      <c r="AB58" s="6"/>
+      <c r="AC58" s="6"/>
+      <c r="AD58" s="6"/>
+      <c r="AE58" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/cromwell-retuya.jpg</v>
       </c>
-      <c r="Y58" s="6" t="s">
+      <c r="AF58" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:25">
+    <row r="59" spans="1:32">
       <c r="A59" s="5">
         <v>58</v>
       </c>
@@ -5559,7 +6408,7 @@
         <v>12</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="J59" s="10"/>
       <c r="K59" s="10"/>
@@ -5574,26 +6423,33 @@
         <v>17</v>
       </c>
       <c r="R59" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="S59" s="6" t="s">
-        <v>367</v>
-      </c>
+        <v>384</v>
+      </c>
+      <c r="S59" s="6"/>
       <c r="T59" s="6"/>
       <c r="U59" s="6"/>
-      <c r="V59" s="6">
+      <c r="V59" s="6"/>
+      <c r="W59" s="6"/>
+      <c r="X59" s="6"/>
+      <c r="Y59" s="6"/>
+      <c r="Z59" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="AA59" s="6"/>
+      <c r="AB59" s="6"/>
+      <c r="AC59" s="6">
         <v>5</v>
       </c>
-      <c r="W59" s="6"/>
-      <c r="X59" s="5" t="str">
+      <c r="AD59" s="6"/>
+      <c r="AE59" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/nancy-reyes.jpg</v>
       </c>
-      <c r="Y59" s="6" t="s">
+      <c r="AF59" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:25">
+    <row r="60" spans="1:32">
       <c r="A60" s="5">
         <v>59</v>
       </c>
@@ -5625,7 +6481,7 @@
         <v>354</v>
       </c>
       <c r="K60" s="10" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5"/>
@@ -5638,22 +6494,29 @@
         <v>17</v>
       </c>
       <c r="R60" s="6"/>
-      <c r="S60" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S60" s="6"/>
       <c r="T60" s="6"/>
       <c r="U60" s="6"/>
       <c r="V60" s="6"/>
       <c r="W60" s="6"/>
-      <c r="X60" s="5" t="str">
+      <c r="X60" s="6"/>
+      <c r="Y60" s="6"/>
+      <c r="Z60" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA60" s="6"/>
+      <c r="AB60" s="6"/>
+      <c r="AC60" s="6"/>
+      <c r="AD60" s="6"/>
+      <c r="AE60" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/angelo-saavedra.jpg</v>
       </c>
-      <c r="Y60" s="6" t="s">
+      <c r="AF60" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:25">
+    <row r="61" spans="1:32">
       <c r="A61" s="5">
         <v>60</v>
       </c>
@@ -5679,7 +6542,7 @@
         <v>244</v>
       </c>
       <c r="I61" s="10" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="J61" s="10"/>
       <c r="K61" s="10"/>
@@ -5694,24 +6557,31 @@
         <v>17</v>
       </c>
       <c r="R61" s="6" t="s">
-        <v>391</v>
-      </c>
-      <c r="S61" s="6" t="s">
-        <v>365</v>
-      </c>
+        <v>389</v>
+      </c>
+      <c r="S61" s="6"/>
       <c r="T61" s="6"/>
       <c r="U61" s="6"/>
       <c r="V61" s="6"/>
       <c r="W61" s="6"/>
-      <c r="X61" s="5" t="str">
+      <c r="X61" s="6"/>
+      <c r="Y61" s="6"/>
+      <c r="Z61" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA61" s="6"/>
+      <c r="AB61" s="6"/>
+      <c r="AC61" s="6"/>
+      <c r="AD61" s="6"/>
+      <c r="AE61" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/brendel-sacaris.jpg</v>
       </c>
-      <c r="Y61" s="6" t="s">
+      <c r="AF61" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:25">
+    <row r="62" spans="1:32">
       <c r="A62" s="5">
         <v>61</v>
       </c>
@@ -5743,7 +6613,7 @@
         <v>354</v>
       </c>
       <c r="K62" s="10" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="L62" s="5"/>
       <c r="M62" s="5"/>
@@ -5756,22 +6626,29 @@
         <v>17</v>
       </c>
       <c r="R62" s="6"/>
-      <c r="S62" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S62" s="6"/>
       <c r="T62" s="6"/>
       <c r="U62" s="6"/>
       <c r="V62" s="6"/>
       <c r="W62" s="6"/>
-      <c r="X62" s="5" t="str">
+      <c r="X62" s="6"/>
+      <c r="Y62" s="6"/>
+      <c r="Z62" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA62" s="6"/>
+      <c r="AB62" s="6"/>
+      <c r="AC62" s="6"/>
+      <c r="AD62" s="6"/>
+      <c r="AE62" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C62&amp;" "&amp;B62)," ","-"))&amp;".jpg"</f>
         <v>/personnel/bella-arquine-samontañez.jpg</v>
       </c>
-      <c r="Y62" s="6" t="s">
+      <c r="AF62" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:25">
+    <row r="63" spans="1:32">
       <c r="A63" s="5">
         <v>62</v>
       </c>
@@ -5803,7 +6680,7 @@
         <v>357</v>
       </c>
       <c r="K63" s="10" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="L63" s="5"/>
       <c r="M63" s="5"/>
@@ -5818,22 +6695,29 @@
       <c r="R63" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S63" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="S63" s="6"/>
       <c r="T63" s="6"/>
       <c r="U63" s="6"/>
       <c r="V63" s="6"/>
       <c r="W63" s="6"/>
-      <c r="X63" s="5" t="str">
+      <c r="X63" s="6"/>
+      <c r="Y63" s="6"/>
+      <c r="Z63" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AA63" s="6"/>
+      <c r="AB63" s="6"/>
+      <c r="AC63" s="6"/>
+      <c r="AD63" s="6"/>
+      <c r="AE63" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jevy-ann-uy.jpg</v>
       </c>
-      <c r="Y63" s="6" t="s">
+      <c r="AF63" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:25">
+    <row r="64" spans="1:32">
       <c r="A64" s="5">
         <v>63</v>
       </c>
@@ -5859,7 +6743,7 @@
         <v>12</v>
       </c>
       <c r="I64" s="10" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="J64" s="10"/>
       <c r="K64" s="10"/>
@@ -5876,22 +6760,29 @@
       <c r="R64" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S64" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="S64" s="6"/>
       <c r="T64" s="6"/>
       <c r="U64" s="6"/>
       <c r="V64" s="6"/>
       <c r="W64" s="6"/>
-      <c r="X64" s="5" t="str">
+      <c r="X64" s="6"/>
+      <c r="Y64" s="6"/>
+      <c r="Z64" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA64" s="6"/>
+      <c r="AB64" s="6"/>
+      <c r="AC64" s="6"/>
+      <c r="AD64" s="6"/>
+      <c r="AE64" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/grace-vergara.jpg</v>
       </c>
-      <c r="Y64" s="6" t="s">
+      <c r="AF64" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:25">
+    <row r="65" spans="1:32">
       <c r="A65" s="5">
         <v>64</v>
       </c>
@@ -5932,24 +6823,31 @@
         <v>7</v>
       </c>
       <c r="R65" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S65" s="6" t="s">
-        <v>271</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S65" s="6"/>
       <c r="T65" s="6"/>
       <c r="U65" s="6"/>
       <c r="V65" s="6"/>
       <c r="W65" s="6"/>
-      <c r="X65" s="5" t="str">
+      <c r="X65" s="6"/>
+      <c r="Y65" s="6"/>
+      <c r="Z65" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="AA65" s="6"/>
+      <c r="AB65" s="6"/>
+      <c r="AC65" s="6"/>
+      <c r="AD65" s="6"/>
+      <c r="AE65" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/guillermo-villavelez.jpg</v>
       </c>
-      <c r="Y65" s="6" t="s">
+      <c r="AF65" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:25">
+    <row r="66" spans="1:32">
       <c r="A66" s="5">
         <v>65</v>
       </c>
@@ -5992,22 +6890,29 @@
       <c r="R66" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S66" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="S66" s="6"/>
       <c r="T66" s="6"/>
       <c r="U66" s="6"/>
       <c r="V66" s="6"/>
       <c r="W66" s="6"/>
-      <c r="X66" s="5" t="str">
+      <c r="X66" s="6"/>
+      <c r="Y66" s="6"/>
+      <c r="Z66" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA66" s="6"/>
+      <c r="AB66" s="6"/>
+      <c r="AC66" s="6"/>
+      <c r="AD66" s="6"/>
+      <c r="AE66" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marilou-villaver.jpg</v>
       </c>
-      <c r="Y66" s="6" t="s">
+      <c r="AF66" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:25">
+    <row r="67" spans="1:32">
       <c r="A67" s="5">
         <v>66</v>
       </c>
@@ -6048,24 +6953,31 @@
         <v>371</v>
       </c>
       <c r="R67" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S67" s="6" t="s">
-        <v>370</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S67" s="6"/>
       <c r="T67" s="6"/>
       <c r="U67" s="6"/>
       <c r="V67" s="6"/>
       <c r="W67" s="6"/>
-      <c r="X67" s="5" t="str">
-        <f t="shared" ref="X67:X68" si="8">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C67&amp;" "&amp;B67)," ","-"))&amp;".jpg"</f>
+      <c r="X67" s="6"/>
+      <c r="Y67" s="6"/>
+      <c r="Z67" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AA67" s="6"/>
+      <c r="AB67" s="6"/>
+      <c r="AC67" s="6"/>
+      <c r="AD67" s="6"/>
+      <c r="AE67" s="5" t="str">
+        <f t="shared" ref="AE67:AE68" si="8">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C67&amp;" "&amp;B67)," ","-"))&amp;".jpg"</f>
         <v>/personnel/markjil-bacaltos.jpg</v>
       </c>
-      <c r="Y67" s="6" t="s">
+      <c r="AF67" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:25">
+    <row r="68" spans="1:32">
       <c r="A68" s="5">
         <v>67</v>
       </c>
@@ -6106,24 +7018,31 @@
         <v>371</v>
       </c>
       <c r="R68" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S68" s="6" t="s">
-        <v>370</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S68" s="6"/>
       <c r="T68" s="6"/>
       <c r="U68" s="6"/>
       <c r="V68" s="6"/>
       <c r="W68" s="6"/>
-      <c r="X68" s="5" t="str">
+      <c r="X68" s="6"/>
+      <c r="Y68" s="6"/>
+      <c r="Z68" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AA68" s="6"/>
+      <c r="AB68" s="6"/>
+      <c r="AC68" s="6"/>
+      <c r="AD68" s="6"/>
+      <c r="AE68" s="5" t="str">
         <f t="shared" si="8"/>
         <v>/personnel/diocel-celocia.jpg</v>
       </c>
-      <c r="Y68" s="6" t="s">
+      <c r="AF68" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:25">
+    <row r="69" spans="1:32">
       <c r="A69" s="5">
         <v>68</v>
       </c>
@@ -6164,24 +7083,31 @@
         <v>371</v>
       </c>
       <c r="R69" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S69" s="6" t="s">
-        <v>370</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S69" s="6"/>
       <c r="T69" s="6"/>
       <c r="U69" s="6"/>
       <c r="V69" s="6"/>
       <c r="W69" s="6"/>
-      <c r="X69" s="5" t="str">
-        <f t="shared" ref="X69:X70" si="11">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C69&amp;" "&amp;B69)," ","-"))&amp;".jpg"</f>
+      <c r="X69" s="6"/>
+      <c r="Y69" s="6"/>
+      <c r="Z69" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AA69" s="6"/>
+      <c r="AB69" s="6"/>
+      <c r="AC69" s="6"/>
+      <c r="AD69" s="6"/>
+      <c r="AE69" s="5" t="str">
+        <f t="shared" ref="AE69:AE70" si="11">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C69&amp;" "&amp;B69)," ","-"))&amp;".jpg"</f>
         <v>/personnel/luie-cabs.jpg</v>
       </c>
-      <c r="Y69" s="6" t="s">
+      <c r="AF69" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:25">
+    <row r="70" spans="1:32">
       <c r="A70" s="5">
         <v>69</v>
       </c>
@@ -6222,24 +7148,31 @@
         <v>371</v>
       </c>
       <c r="R70" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S70" s="6" t="s">
-        <v>370</v>
-      </c>
+        <v>385</v>
+      </c>
+      <c r="S70" s="6"/>
       <c r="T70" s="6"/>
       <c r="U70" s="6"/>
       <c r="V70" s="6"/>
       <c r="W70" s="6"/>
-      <c r="X70" s="5" t="str">
+      <c r="X70" s="6"/>
+      <c r="Y70" s="6"/>
+      <c r="Z70" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AA70" s="6"/>
+      <c r="AB70" s="6"/>
+      <c r="AC70" s="6"/>
+      <c r="AD70" s="6"/>
+      <c r="AE70" s="5" t="str">
         <f t="shared" si="11"/>
         <v>/personnel/luis-mans.jpg</v>
       </c>
-      <c r="Y70" s="6" t="s">
+      <c r="AF70" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:25">
+    <row r="71" spans="1:32">
       <c r="A71" s="5">
         <v>70</v>
       </c>
@@ -6268,8 +7201,15 @@
       <c r="U71" s="6"/>
       <c r="V71" s="6"/>
       <c r="W71" s="6"/>
-      <c r="X71" s="5"/>
+      <c r="X71" s="6"/>
       <c r="Y71" s="6"/>
+      <c r="Z71" s="6"/>
+      <c r="AA71" s="6"/>
+      <c r="AB71" s="6"/>
+      <c r="AC71" s="6"/>
+      <c r="AD71" s="6"/>
+      <c r="AE71" s="5"/>
+      <c r="AF71" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -6302,19 +7242,19 @@
           <x14:formula1>
             <xm:f>Dropdown_Lists!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>Y2:Y71</xm:sqref>
+          <xm:sqref>AF2:AF71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{70D54F6E-2A67-40F0-92CA-B6E53F44843D}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$D$2:$D$61</xm:f>
           </x14:formula1>
-          <xm:sqref>S2:S71</xm:sqref>
+          <xm:sqref>Z2:Z71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7834D497-9733-4178-89DF-4B7895726F53}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$E$2:$E$60</xm:f>
           </x14:formula1>
-          <xm:sqref>T2:T71</xm:sqref>
+          <xm:sqref>AA2:AA71</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Update organization page responsive card layout
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFE0AE0-5E41-4065-B58F-FE70AA82722B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0C289C-C94D-47D0-869F-434C983C10DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="21300" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="21315" windowHeight="16200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="personnel" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="482">
   <si>
     <t>order</t>
   </si>
@@ -1198,9 +1198,6 @@
     <t>EPP</t>
   </si>
   <si>
-    <t>Electronic Product Assembly and Servicing</t>
-  </si>
-  <si>
     <t>Hairdressing/Beauty Care</t>
   </si>
   <si>
@@ -1460,6 +1457,30 @@
   </si>
   <si>
     <t>English 7 &amp; 8</t>
+  </si>
+  <si>
+    <t>Guidance and Student Support</t>
+  </si>
+  <si>
+    <t>Electronic Products Assembly and Servicing</t>
+  </si>
+  <si>
+    <t>Technical-Vocational-Livelihood (TVL)</t>
+  </si>
+  <si>
+    <t>Technology and Livelihood Education (TLE)</t>
+  </si>
+  <si>
+    <t>SubjectDepartment2</t>
+  </si>
+  <si>
+    <t>SubjectDepartment3</t>
+  </si>
+  <si>
+    <t>SubjectDepartment4</t>
+  </si>
+  <si>
+    <t>SubjectDepartment5</t>
   </si>
 </sst>
 </file>
@@ -1565,7 +1586,110 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="39">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1698,33 +1822,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Segoe UI"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -2145,44 +2242,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:AF71" headerRowDxfId="34" dataDxfId="33" totalsRowDxfId="32">
-  <tableColumns count="32">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="29"/>
-    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="28"/>
-    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PersonnelRosterTable" displayName="PersonnelRosterTable" ref="A1:AJ71" headerRowDxfId="38" dataDxfId="37" totalsRowDxfId="36">
+  <tableColumns count="36">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="order" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="lastName" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{AF2D5150-6C8E-4586-A045-6EA7C80A524C}" name="firstName" dataDxfId="33"/>
+    <tableColumn id="12" xr3:uid="{DEB63105-4C35-428E-B5D1-A14E3164B3DA}" name="middleName" dataDxfId="32"/>
+    <tableColumn id="11" xr3:uid="{CFE5C25B-9704-4E8F-ACBC-C9336567385E}" name="middleInitial" dataDxfId="31">
       <calculatedColumnFormula>IF(D2="","",LEFT(TRIM(D2),1)&amp;".")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="26"/>
-    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="25">
+    <tableColumn id="9" xr3:uid="{C15E3D36-7D44-4129-AD8E-8A7781CC6A93}" name="suffix" dataDxfId="30"/>
+    <tableColumn id="13" xr3:uid="{1E3C14F7-2268-499C-B881-A1FE0A7127D7}" name="displayName" dataDxfId="29">
       <calculatedColumnFormula>TRIM(_xlfn.TEXTJOIN(" ",TRUE,C2,IF(E2&lt;&gt;"",IF(RIGHT(E2,1)=".",E2,E2&amp;"."),D2),B2,F2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="24"/>
-    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="23"/>
-    <tableColumn id="24" xr3:uid="{9E70E31F-1B17-4E67-A99E-4037A94153C1}" name="advisoryGradeLevel" dataDxfId="22"/>
-    <tableColumn id="25" xr3:uid="{82F63A8C-E0AF-4172-B1EB-CC758DA39858}" name="advisorySection" dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="20"/>
-    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="19"/>
-    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="18"/>
-    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="14"/>
-    <tableColumn id="26" xr3:uid="{9234D872-27E9-4981-9849-3B92B3D703D7}" name="primarySubjectDepartment" dataDxfId="6"/>
-    <tableColumn id="27" xr3:uid="{BAF0BAF6-D68C-494F-94BF-9DBEAC627028}" name="subject1" dataDxfId="5"/>
-    <tableColumn id="28" xr3:uid="{8B540991-2968-4F70-8AAC-FCFC355A419A}" name="subject2" dataDxfId="4"/>
-    <tableColumn id="29" xr3:uid="{1D6F7D4B-4E56-4246-A153-8FAB0BEB4811}" name="subject3" dataDxfId="3"/>
-    <tableColumn id="30" xr3:uid="{E295C211-F74A-4E2B-893A-E9FDF18B7EE9}" name="subject4" dataDxfId="2"/>
-    <tableColumn id="31" xr3:uid="{B93E7C74-87A6-4CBE-9E54-1C7E4E717375}" name="subject5" dataDxfId="1"/>
-    <tableColumn id="32" xr3:uid="{AE0F403C-1544-4D9E-929C-27676144B2E2}" name="teachingLevel" dataDxfId="0"/>
-    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="13"/>
-    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="12"/>
-    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="11"/>
-    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="10"/>
-    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="position" dataDxfId="28"/>
+    <tableColumn id="14" xr3:uid="{871D5899-2C99-449D-AE1E-5492B1075D69}" name="designation1" dataDxfId="27"/>
+    <tableColumn id="24" xr3:uid="{9E70E31F-1B17-4E67-A99E-4037A94153C1}" name="advisoryGradeLevel" dataDxfId="26"/>
+    <tableColumn id="25" xr3:uid="{82F63A8C-E0AF-4172-B1EB-CC758DA39858}" name="advisorySection" dataDxfId="25"/>
+    <tableColumn id="15" xr3:uid="{F4F0A446-7DFB-4099-8C3C-39E5D7D48BD0}" name="designation2" dataDxfId="24"/>
+    <tableColumn id="16" xr3:uid="{9D4F6523-1087-480E-82D3-17DF6BB11D95}" name="designation3" dataDxfId="23"/>
+    <tableColumn id="18" xr3:uid="{30162747-79C9-4043-9391-B8B420E4C626}" name="designation4" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{820C0CC6-055B-4F59-A5A5-608142530FDE}" name="otherDesignations" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="category" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="department" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="subjectArea" dataDxfId="18"/>
+    <tableColumn id="26" xr3:uid="{9234D872-27E9-4981-9849-3B92B3D703D7}" name="primarySubjectDepartment" dataDxfId="17"/>
+    <tableColumn id="34" xr3:uid="{168EB6BE-8B21-4305-ABC1-174562CD0A0B}" name="SubjectDepartment2" dataDxfId="3"/>
+    <tableColumn id="35" xr3:uid="{5C2FF8F3-D884-43D6-84E1-D482E29A632A}" name="SubjectDepartment3" dataDxfId="2"/>
+    <tableColumn id="36" xr3:uid="{9BC6D117-EABD-4BEC-9C2D-4F49F4E8F4AF}" name="SubjectDepartment4" dataDxfId="1"/>
+    <tableColumn id="37" xr3:uid="{C21080E4-B7D1-416D-9C89-C64670FF6EAA}" name="SubjectDepartment5" dataDxfId="0"/>
+    <tableColumn id="27" xr3:uid="{BAF0BAF6-D68C-494F-94BF-9DBEAC627028}" name="subject1" dataDxfId="16"/>
+    <tableColumn id="28" xr3:uid="{8B540991-2968-4F70-8AAC-FCFC355A419A}" name="subject2" dataDxfId="15"/>
+    <tableColumn id="29" xr3:uid="{1D6F7D4B-4E56-4246-A153-8FAB0BEB4811}" name="subject3" dataDxfId="14"/>
+    <tableColumn id="30" xr3:uid="{E295C211-F74A-4E2B-893A-E9FDF18B7EE9}" name="subject4" dataDxfId="13"/>
+    <tableColumn id="31" xr3:uid="{B93E7C74-87A6-4CBE-9E54-1C7E4E717375}" name="subject5" dataDxfId="12"/>
+    <tableColumn id="32" xr3:uid="{AE0F403C-1544-4D9E-929C-27676144B2E2}" name="teachingLevel" dataDxfId="11"/>
+    <tableColumn id="23" xr3:uid="{07B5CB0A-FE18-46C6-B1E6-1B1D900FB654}" name="displayGroup" dataDxfId="10"/>
+    <tableColumn id="22" xr3:uid="{65EBFB40-77EE-48B3-8561-311242B8D6D2}" name="subGroup" dataDxfId="9"/>
+    <tableColumn id="21" xr3:uid="{AE424BEB-0E42-47BC-8BF7-A0E6C15B9F30}" name="groupOrder" dataDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{8ED835C9-250F-4A69-B1C0-89AD725EFF0F}" name="subGroupOrder" dataDxfId="7"/>
+    <tableColumn id="19" xr3:uid="{894550D0-2DF4-4E17-A2FB-C537176088F7}" name="personOrder" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="photoUrl" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="status" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2337,17 +2438,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF71"/>
+  <dimension ref="A1:AJ71"/>
   <sheetFormatPr defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="5.59765625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.09765625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.8984375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.59765625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="13.3984375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="10.69921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.69921875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.296875" style="4" customWidth="1"/>
     <col min="6" max="6" width="5.796875" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.3984375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="23.5" style="4" customWidth="1"/>
+    <col min="7" max="7" width="23.59765625" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.69921875" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="40.796875" style="11" customWidth="1"/>
     <col min="10" max="10" width="19.296875" style="11" customWidth="1"/>
     <col min="11" max="11" width="17.296875" style="11" customWidth="1"/>
@@ -2356,14 +2457,14 @@
     <col min="15" max="15" width="32.8984375" style="4" customWidth="1"/>
     <col min="16" max="16" width="26.69921875" style="4" customWidth="1"/>
     <col min="17" max="17" width="20.09765625" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="25" width="45.19921875" style="7" customWidth="1"/>
-    <col min="26" max="30" width="24.19921875" style="7" customWidth="1"/>
-    <col min="31" max="31" width="36.69921875" style="4" customWidth="1"/>
-    <col min="32" max="32" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.796875" style="4"/>
+    <col min="18" max="29" width="45.19921875" style="7" customWidth="1"/>
+    <col min="30" max="34" width="24.19921875" style="7" customWidth="1"/>
+    <col min="35" max="35" width="36.69921875" style="4" customWidth="1"/>
+    <col min="36" max="36" width="6.3984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="37" max="16384" width="8.796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="20.399999999999999" customHeight="1">
+    <row r="1" spans="1:36" ht="39" customHeight="1">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -2392,10 +2493,10 @@
         <v>324</v>
       </c>
       <c r="J1" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="K1" s="8" t="s">
         <v>394</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>395</v>
       </c>
       <c r="L1" s="8" t="s">
         <v>325</v>
@@ -2419,49 +2520,61 @@
         <v>4</v>
       </c>
       <c r="S1" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>478</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>480</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>481</v>
+      </c>
+      <c r="X1" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="Y1" s="8" t="s">
         <v>428</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>429</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="AA1" s="8" t="s">
         <v>430</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="AB1" s="8" t="s">
         <v>431</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="AC1" s="8" t="s">
         <v>432</v>
       </c>
-      <c r="Y1" s="8" t="s">
-        <v>433</v>
-      </c>
-      <c r="Z1" s="8" t="s">
+      <c r="AD1" s="8" t="s">
         <v>360</v>
       </c>
-      <c r="AA1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="AB1" s="8" t="s">
+      <c r="AF1" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="AC1" s="8" t="s">
+      <c r="AG1" s="8" t="s">
         <v>362</v>
       </c>
-      <c r="AD1" s="8" t="s">
+      <c r="AH1" s="8" t="s">
         <v>363</v>
       </c>
-      <c r="AE1" s="8" t="s">
+      <c r="AI1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="AF1" s="8" t="s">
+      <c r="AJ1" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" spans="1:36">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -2507,34 +2620,38 @@
       <c r="S2" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="T2" s="6" t="s">
-        <v>426</v>
-      </c>
+      <c r="T2" s="6"/>
       <c r="U2" s="6"/>
       <c r="V2" s="6"/>
       <c r="W2" s="6"/>
-      <c r="X2" s="6"/>
-      <c r="Y2" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z2" s="6" t="s">
-        <v>366</v>
-      </c>
+      <c r="X2" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="Y2" s="6"/>
+      <c r="Z2" s="6"/>
       <c r="AA2" s="6"/>
       <c r="AB2" s="6"/>
-      <c r="AC2" s="6">
+      <c r="AC2" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD2" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="AE2" s="6"/>
+      <c r="AF2" s="6"/>
+      <c r="AG2" s="6">
         <v>2</v>
       </c>
-      <c r="AD2" s="6"/>
-      <c r="AE2" s="5" t="str">
+      <c r="AH2" s="6"/>
+      <c r="AI2" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C2&amp;" "&amp;B2)," ","-"))&amp;".jpg"</f>
         <v>/personnel/paz-abad.jpg</v>
       </c>
-      <c r="AF2" s="6" t="s">
+      <c r="AJ2" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:32">
+    <row r="3" spans="1:36">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -2566,7 +2683,7 @@
         <v>353</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
@@ -2584,36 +2701,40 @@
       <c r="S3" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="T3" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="U3" s="6" t="s">
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="Y3" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="Z3" s="6" t="s">
         <v>437</v>
-      </c>
-      <c r="V3" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="W3" s="6"/>
-      <c r="X3" s="6"/>
-      <c r="Y3" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="Z3" s="6" t="s">
-        <v>277</v>
       </c>
       <c r="AA3" s="6"/>
       <c r="AB3" s="6"/>
-      <c r="AC3" s="6"/>
-      <c r="AD3" s="6"/>
-      <c r="AE3" s="5" t="str">
-        <f t="shared" ref="AE3:AE66" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C3&amp;" "&amp;B3)," ","-"))&amp;".jpg"</f>
+      <c r="AC3" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD3" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE3" s="6"/>
+      <c r="AF3" s="6"/>
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="5" t="str">
+        <f t="shared" ref="AI3:AI66" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C3&amp;" "&amp;B3)," ","-"))&amp;".jpg"</f>
         <v>/personnel/marissa-abalo.jpg</v>
       </c>
-      <c r="AF3" s="6" t="s">
+      <c r="AJ3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:32">
+    <row r="4" spans="1:36">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -2639,7 +2760,7 @@
         <v>12</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
@@ -2659,32 +2780,36 @@
       <c r="S4" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="T4" s="6" t="s">
-        <v>463</v>
-      </c>
+      <c r="T4" s="6"/>
       <c r="U4" s="6"/>
       <c r="V4" s="6"/>
       <c r="W4" s="6"/>
-      <c r="X4" s="6"/>
-      <c r="Y4" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z4" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="X4" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="Y4" s="6"/>
+      <c r="Z4" s="6"/>
       <c r="AA4" s="6"/>
       <c r="AB4" s="6"/>
-      <c r="AC4" s="6"/>
-      <c r="AD4" s="6"/>
-      <c r="AE4" s="5" t="str">
+      <c r="AC4" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD4" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE4" s="6"/>
+      <c r="AF4" s="6"/>
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
+      <c r="AI4" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joseph-allosada.jpg</v>
       </c>
-      <c r="AF4" s="6" t="s">
+      <c r="AJ4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:32" ht="33.6">
+    <row r="5" spans="1:36" ht="33.6">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -2716,13 +2841,13 @@
         <v>355</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L5" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="M5" s="5" t="s">
         <v>440</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>441</v>
       </c>
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
@@ -2738,34 +2863,38 @@
       <c r="S5" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="T5" s="6" t="s">
-        <v>442</v>
-      </c>
-      <c r="U5" s="6" t="s">
-        <v>436</v>
-      </c>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
       <c r="V5" s="6"/>
       <c r="W5" s="6"/>
-      <c r="X5" s="6"/>
+      <c r="X5" s="6" t="s">
+        <v>441</v>
+      </c>
       <c r="Y5" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z5" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>435</v>
+      </c>
+      <c r="Z5" s="6"/>
       <c r="AA5" s="6"/>
       <c r="AB5" s="6"/>
-      <c r="AC5" s="6"/>
-      <c r="AD5" s="6"/>
-      <c r="AE5" s="5" t="str">
+      <c r="AC5" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD5" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE5" s="6"/>
+      <c r="AF5" s="6"/>
+      <c r="AG5" s="6"/>
+      <c r="AH5" s="6"/>
+      <c r="AI5" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/sharon-gay-alsa.jpg</v>
       </c>
-      <c r="AF5" s="6" t="s">
+      <c r="AJ5" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:32" ht="33.6">
+    <row r="6" spans="1:36" ht="33.6">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -2797,7 +2926,7 @@
         <v>356</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
@@ -2810,39 +2939,43 @@
         <v>14</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>345</v>
-      </c>
-      <c r="T6" s="6" t="s">
-        <v>444</v>
-      </c>
-      <c r="U6" s="6" t="s">
-        <v>445</v>
-      </c>
+        <v>476</v>
+      </c>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
       <c r="V6" s="6"/>
       <c r="W6" s="6"/>
-      <c r="X6" s="6"/>
+      <c r="X6" s="6" t="s">
+        <v>443</v>
+      </c>
       <c r="Y6" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="Z6" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>444</v>
+      </c>
+      <c r="Z6" s="6"/>
       <c r="AA6" s="6"/>
       <c r="AB6" s="6"/>
-      <c r="AC6" s="6"/>
-      <c r="AD6" s="6"/>
-      <c r="AE6" s="5" t="str">
+      <c r="AC6" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="AD6" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE6" s="6"/>
+      <c r="AF6" s="6"/>
+      <c r="AG6" s="6"/>
+      <c r="AH6" s="6"/>
+      <c r="AI6" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lonier-andrade.jpg</v>
       </c>
-      <c r="AF6" s="6" t="s">
+      <c r="AJ6" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:32">
+    <row r="7" spans="1:36">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -2874,13 +3007,13 @@
         <v>354</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="L7" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>446</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>447</v>
       </c>
       <c r="N7" s="5"/>
       <c r="O7" s="5"/>
@@ -2894,34 +3027,38 @@
         <v>344</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>344</v>
-      </c>
-      <c r="T7" s="6" t="s">
-        <v>461</v>
-      </c>
+        <v>477</v>
+      </c>
+      <c r="T7" s="6"/>
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
-      <c r="X7" s="6"/>
-      <c r="Y7" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z7" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="X7" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
       <c r="AA7" s="6"/>
       <c r="AB7" s="6"/>
-      <c r="AC7" s="6"/>
-      <c r="AD7" s="6"/>
-      <c r="AE7" s="5" t="str">
+      <c r="AC7" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD7" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE7" s="6"/>
+      <c r="AF7" s="6"/>
+      <c r="AG7" s="6"/>
+      <c r="AH7" s="6"/>
+      <c r="AI7" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/allan-raul-aparicio.jpg</v>
       </c>
-      <c r="AF7" s="6" t="s">
+      <c r="AJ7" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:32">
+    <row r="8" spans="1:36">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -2969,22 +3106,26 @@
       <c r="W8" s="6"/>
       <c r="X8" s="6"/>
       <c r="Y8" s="6"/>
-      <c r="Z8" s="6" t="s">
-        <v>364</v>
-      </c>
+      <c r="Z8" s="6"/>
       <c r="AA8" s="6"/>
       <c r="AB8" s="6"/>
       <c r="AC8" s="6"/>
-      <c r="AD8" s="6"/>
-      <c r="AE8" s="5" t="str">
+      <c r="AD8" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="AE8" s="6"/>
+      <c r="AF8" s="6"/>
+      <c r="AG8" s="6"/>
+      <c r="AH8" s="6"/>
+      <c r="AI8" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/niña-kristine-ayos.jpg</v>
       </c>
-      <c r="AF8" s="6" t="s">
+      <c r="AJ8" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:32">
+    <row r="9" spans="1:36">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -3010,12 +3151,12 @@
         <v>244</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="J9" s="10"/>
       <c r="K9" s="10"/>
       <c r="L9" s="5" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
@@ -3030,34 +3171,38 @@
         <v>344</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>344</v>
-      </c>
-      <c r="T9" s="6" t="s">
-        <v>462</v>
-      </c>
+        <v>477</v>
+      </c>
+      <c r="T9" s="6"/>
       <c r="U9" s="6"/>
       <c r="V9" s="6"/>
       <c r="W9" s="6"/>
-      <c r="X9" s="6"/>
-      <c r="Y9" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z9" s="6" t="s">
-        <v>368</v>
-      </c>
+      <c r="X9" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="Y9" s="6"/>
+      <c r="Z9" s="6"/>
       <c r="AA9" s="6"/>
       <c r="AB9" s="6"/>
-      <c r="AC9" s="6"/>
-      <c r="AD9" s="6"/>
-      <c r="AE9" s="5" t="str">
+      <c r="AC9" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD9" s="6" t="s">
+        <v>368</v>
+      </c>
+      <c r="AE9" s="6"/>
+      <c r="AF9" s="6"/>
+      <c r="AG9" s="6"/>
+      <c r="AH9" s="6"/>
+      <c r="AI9" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/glenn-barangan.jpg</v>
       </c>
-      <c r="AF9" s="6" t="s">
+      <c r="AJ9" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:32">
+    <row r="10" spans="1:36">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -3089,13 +3234,13 @@
         <v>355</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="L10" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>450</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>451</v>
       </c>
       <c r="N10" s="5"/>
       <c r="O10" s="5"/>
@@ -3111,32 +3256,36 @@
       <c r="S10" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="T10" s="6" t="s">
-        <v>452</v>
-      </c>
+      <c r="T10" s="6"/>
       <c r="U10" s="6"/>
       <c r="V10" s="6"/>
       <c r="W10" s="6"/>
-      <c r="X10" s="6"/>
-      <c r="Y10" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z10" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="X10" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="Y10" s="6"/>
+      <c r="Z10" s="6"/>
       <c r="AA10" s="6"/>
       <c r="AB10" s="6"/>
-      <c r="AC10" s="6"/>
-      <c r="AD10" s="6"/>
-      <c r="AE10" s="5" t="str">
+      <c r="AC10" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD10" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE10" s="6"/>
+      <c r="AF10" s="6"/>
+      <c r="AG10" s="6"/>
+      <c r="AH10" s="6"/>
+      <c r="AI10" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jake-barcenas.jpg</v>
       </c>
-      <c r="AF10" s="6" t="s">
+      <c r="AJ10" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:32">
+    <row r="11" spans="1:36">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -3168,10 +3317,10 @@
         <v>353</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
@@ -3188,32 +3337,36 @@
       <c r="S11" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="T11" s="6" t="s">
-        <v>454</v>
-      </c>
+      <c r="T11" s="6"/>
       <c r="U11" s="6"/>
       <c r="V11" s="6"/>
       <c r="W11" s="6"/>
-      <c r="X11" s="6"/>
-      <c r="Y11" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z11" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="X11" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="Y11" s="6"/>
+      <c r="Z11" s="6"/>
       <c r="AA11" s="6"/>
       <c r="AB11" s="6"/>
-      <c r="AC11" s="6"/>
-      <c r="AD11" s="6"/>
-      <c r="AE11" s="5" t="str">
+      <c r="AC11" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD11" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE11" s="6"/>
+      <c r="AF11" s="6"/>
+      <c r="AG11" s="6"/>
+      <c r="AH11" s="6"/>
+      <c r="AI11" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/eljoy-barroca.jpg</v>
       </c>
-      <c r="AF11" s="6" t="s">
+      <c r="AJ11" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="33.6">
+    <row r="12" spans="1:36" ht="33.6">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -3245,13 +3398,13 @@
         <v>357</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="L12" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>455</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>456</v>
       </c>
       <c r="N12" s="5"/>
       <c r="O12" s="5"/>
@@ -3265,36 +3418,40 @@
         <v>342</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>457</v>
-      </c>
-      <c r="T12" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="U12" s="6" t="s">
-        <v>459</v>
-      </c>
+        <v>456</v>
+      </c>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
       <c r="V12" s="6"/>
       <c r="W12" s="6"/>
-      <c r="X12" s="6"/>
+      <c r="X12" s="6" t="s">
+        <v>457</v>
+      </c>
       <c r="Y12" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="Z12" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>458</v>
+      </c>
+      <c r="Z12" s="6"/>
       <c r="AA12" s="6"/>
       <c r="AB12" s="6"/>
-      <c r="AC12" s="6"/>
-      <c r="AD12" s="6"/>
-      <c r="AE12" s="5" t="str">
+      <c r="AC12" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD12" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE12" s="6"/>
+      <c r="AF12" s="6"/>
+      <c r="AG12" s="6"/>
+      <c r="AH12" s="6"/>
+      <c r="AI12" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/angel-batuigas.jpg</v>
       </c>
-      <c r="AF12" s="6" t="s">
+      <c r="AJ12" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:32">
+    <row r="13" spans="1:36">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -3320,7 +3477,7 @@
         <v>12</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="J13" s="10"/>
       <c r="K13" s="10"/>
@@ -3340,32 +3497,36 @@
       <c r="S13" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="T13" s="6" t="s">
-        <v>464</v>
-      </c>
+      <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
       <c r="W13" s="6"/>
-      <c r="X13" s="6"/>
-      <c r="Y13" s="6" t="s">
-        <v>337</v>
-      </c>
-      <c r="Z13" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="X13" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="Y13" s="6"/>
+      <c r="Z13" s="6"/>
       <c r="AA13" s="6"/>
       <c r="AB13" s="6"/>
-      <c r="AC13" s="6"/>
-      <c r="AD13" s="6"/>
-      <c r="AE13" s="5" t="str">
+      <c r="AC13" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD13" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE13" s="6"/>
+      <c r="AF13" s="6"/>
+      <c r="AG13" s="6"/>
+      <c r="AH13" s="6"/>
+      <c r="AI13" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/mary-josephine-bawiga.jpg</v>
       </c>
-      <c r="AF13" s="6" t="s">
+      <c r="AJ13" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:32">
+    <row r="14" spans="1:36">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -3397,10 +3558,10 @@
         <v>352</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
@@ -3417,34 +3578,38 @@
       <c r="S14" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="T14" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="U14" s="6" t="s">
-        <v>466</v>
-      </c>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
       <c r="V14" s="6"/>
       <c r="W14" s="6"/>
-      <c r="X14" s="6"/>
+      <c r="X14" s="6" t="s">
+        <v>466</v>
+      </c>
       <c r="Y14" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="Z14" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>465</v>
+      </c>
+      <c r="Z14" s="6"/>
       <c r="AA14" s="6"/>
       <c r="AB14" s="6"/>
-      <c r="AC14" s="6"/>
-      <c r="AD14" s="6"/>
-      <c r="AE14" s="5" t="str">
+      <c r="AC14" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD14" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE14" s="6"/>
+      <c r="AF14" s="6"/>
+      <c r="AG14" s="6"/>
+      <c r="AH14" s="6"/>
+      <c r="AI14" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/endrie-bohol.jpg</v>
       </c>
-      <c r="AF14" s="6" t="s">
+      <c r="AJ14" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="33.6">
+    <row r="15" spans="1:36" ht="33.6">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -3475,10 +3640,10 @@
       <c r="J15" s="10"/>
       <c r="K15" s="10"/>
       <c r="L15" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="M15" s="5" t="s">
         <v>468</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>469</v>
       </c>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
@@ -3494,36 +3659,40 @@
       <c r="S15" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="T15" s="6" t="s">
-        <v>470</v>
-      </c>
-      <c r="U15" s="6" t="s">
-        <v>471</v>
-      </c>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
       <c r="V15" s="6"/>
       <c r="W15" s="6"/>
-      <c r="X15" s="6"/>
+      <c r="X15" s="6" t="s">
+        <v>469</v>
+      </c>
       <c r="Y15" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="Z15" s="6" t="s">
-        <v>365</v>
-      </c>
+        <v>470</v>
+      </c>
+      <c r="Z15" s="6"/>
       <c r="AA15" s="6"/>
       <c r="AB15" s="6"/>
-      <c r="AC15" s="6">
+      <c r="AC15" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="AD15" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE15" s="6"/>
+      <c r="AF15" s="6"/>
+      <c r="AG15" s="6">
         <v>1</v>
       </c>
-      <c r="AD15" s="6"/>
-      <c r="AE15" s="5" t="str">
+      <c r="AH15" s="6"/>
+      <c r="AI15" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/maine-bongas.jpg</v>
       </c>
-      <c r="AF15" s="6" t="s">
+      <c r="AJ15" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="33.6">
+    <row r="16" spans="1:36" ht="33.6">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -3553,10 +3722,10 @@
         <v>352</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
@@ -3573,34 +3742,38 @@
       <c r="S16" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="T16" s="6" t="s">
-        <v>473</v>
-      </c>
-      <c r="U16" s="6" t="s">
-        <v>474</v>
-      </c>
+      <c r="T16" s="6"/>
+      <c r="U16" s="6"/>
       <c r="V16" s="6"/>
       <c r="W16" s="6"/>
-      <c r="X16" s="6"/>
+      <c r="X16" s="6" t="s">
+        <v>472</v>
+      </c>
       <c r="Y16" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="Z16" s="6" t="s">
-        <v>277</v>
-      </c>
+        <v>473</v>
+      </c>
+      <c r="Z16" s="6"/>
       <c r="AA16" s="6"/>
       <c r="AB16" s="6"/>
-      <c r="AC16" s="6"/>
-      <c r="AD16" s="6"/>
-      <c r="AE16" s="5" t="str">
+      <c r="AC16" s="6" t="s">
+        <v>433</v>
+      </c>
+      <c r="AD16" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE16" s="6"/>
+      <c r="AF16" s="6"/>
+      <c r="AG16" s="6"/>
+      <c r="AH16" s="6"/>
+      <c r="AI16" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/ruth-briones.jpg</v>
       </c>
-      <c r="AF16" s="6" t="s">
+      <c r="AJ16" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:32">
+    <row r="17" spans="1:36">
       <c r="A17" s="5">
         <v>16</v>
       </c>
@@ -3651,15 +3824,19 @@
       <c r="AB17" s="6"/>
       <c r="AC17" s="6"/>
       <c r="AD17" s="6"/>
-      <c r="AE17" s="5" t="str">
+      <c r="AE17" s="6"/>
+      <c r="AF17" s="6"/>
+      <c r="AG17" s="6"/>
+      <c r="AH17" s="6"/>
+      <c r="AI17" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/sharon-broñola.jpg</v>
       </c>
-      <c r="AF17" s="6" t="s">
+      <c r="AJ17" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:32">
+    <row r="18" spans="1:36">
       <c r="A18" s="5">
         <v>17</v>
       </c>
@@ -3702,7 +3879,9 @@
       <c r="R18" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S18" s="6"/>
+      <c r="S18" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="T18" s="6"/>
       <c r="U18" s="6"/>
       <c r="V18" s="6"/>
@@ -3714,15 +3893,19 @@
       <c r="AB18" s="6"/>
       <c r="AC18" s="6"/>
       <c r="AD18" s="6"/>
-      <c r="AE18" s="5" t="str">
+      <c r="AE18" s="6"/>
+      <c r="AF18" s="6"/>
+      <c r="AG18" s="6"/>
+      <c r="AH18" s="6"/>
+      <c r="AI18" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joan-cabalda.jpg</v>
       </c>
-      <c r="AF18" s="6" t="s">
+      <c r="AJ18" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:32">
+    <row r="19" spans="1:36">
       <c r="A19" s="5">
         <v>18</v>
       </c>
@@ -3765,29 +3948,35 @@
       <c r="R19" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S19" s="6"/>
+      <c r="S19" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="T19" s="6"/>
       <c r="U19" s="6"/>
       <c r="V19" s="6"/>
       <c r="W19" s="6"/>
       <c r="X19" s="6"/>
       <c r="Y19" s="6"/>
-      <c r="Z19" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z19" s="6"/>
       <c r="AA19" s="6"/>
       <c r="AB19" s="6"/>
       <c r="AC19" s="6"/>
-      <c r="AD19" s="6"/>
-      <c r="AE19" s="5" t="str">
+      <c r="AD19" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE19" s="6"/>
+      <c r="AF19" s="6"/>
+      <c r="AG19" s="6"/>
+      <c r="AH19" s="6"/>
+      <c r="AI19" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/gracelyn-cabunag.jpg</v>
       </c>
-      <c r="AF19" s="6" t="s">
+      <c r="AJ19" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:32">
+    <row r="20" spans="1:36">
       <c r="A20" s="5">
         <v>19</v>
       </c>
@@ -3830,7 +4019,9 @@
       <c r="R20" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S20" s="6"/>
+      <c r="S20" s="6" t="s">
+        <v>343</v>
+      </c>
       <c r="T20" s="6"/>
       <c r="U20" s="6"/>
       <c r="V20" s="6"/>
@@ -3840,19 +4031,23 @@
       <c r="Z20" s="6"/>
       <c r="AA20" s="6"/>
       <c r="AB20" s="6"/>
-      <c r="AC20" s="6">
+      <c r="AC20" s="6"/>
+      <c r="AD20" s="6"/>
+      <c r="AE20" s="6"/>
+      <c r="AF20" s="6"/>
+      <c r="AG20" s="6">
         <v>3</v>
       </c>
-      <c r="AD20" s="6"/>
-      <c r="AE20" s="5" t="str">
+      <c r="AH20" s="6"/>
+      <c r="AI20" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/hector-cabanca.jpg</v>
       </c>
-      <c r="AF20" s="6" t="s">
+      <c r="AJ20" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:32">
+    <row r="21" spans="1:36">
       <c r="A21" s="5">
         <v>20</v>
       </c>
@@ -3884,7 +4079,7 @@
         <v>354</v>
       </c>
       <c r="K21" s="10" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
@@ -3899,29 +4094,35 @@
       <c r="R21" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S21" s="6"/>
+      <c r="S21" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="T21" s="6"/>
       <c r="U21" s="6"/>
       <c r="V21" s="6"/>
       <c r="W21" s="6"/>
       <c r="X21" s="6"/>
       <c r="Y21" s="6"/>
-      <c r="Z21" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z21" s="6"/>
       <c r="AA21" s="6"/>
       <c r="AB21" s="6"/>
       <c r="AC21" s="6"/>
-      <c r="AD21" s="6"/>
-      <c r="AE21" s="5" t="str">
+      <c r="AD21" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE21" s="6"/>
+      <c r="AF21" s="6"/>
+      <c r="AG21" s="6"/>
+      <c r="AH21" s="6"/>
+      <c r="AI21" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeffrey-caberte.jpg</v>
       </c>
-      <c r="AF21" s="6" t="s">
+      <c r="AJ21" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:32">
+    <row r="22" spans="1:36">
       <c r="A22" s="5">
         <v>21</v>
       </c>
@@ -3953,7 +4154,7 @@
         <v>355</v>
       </c>
       <c r="K22" s="10" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
@@ -3973,22 +4174,26 @@
       <c r="W22" s="6"/>
       <c r="X22" s="6"/>
       <c r="Y22" s="6"/>
-      <c r="Z22" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z22" s="6"/>
       <c r="AA22" s="6"/>
       <c r="AB22" s="6"/>
       <c r="AC22" s="6"/>
-      <c r="AD22" s="6"/>
-      <c r="AE22" s="5" t="str">
+      <c r="AD22" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE22" s="6"/>
+      <c r="AF22" s="6"/>
+      <c r="AG22" s="6"/>
+      <c r="AH22" s="6"/>
+      <c r="AI22" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marilou-cabriana.jpg</v>
       </c>
-      <c r="AF22" s="6" t="s">
+      <c r="AJ22" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:32">
+    <row r="23" spans="1:36">
       <c r="A23" s="5">
         <v>22</v>
       </c>
@@ -4031,29 +4236,35 @@
       <c r="R23" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S23" s="6"/>
+      <c r="S23" s="6" t="s">
+        <v>474</v>
+      </c>
       <c r="T23" s="6"/>
       <c r="U23" s="6"/>
       <c r="V23" s="6"/>
       <c r="W23" s="6"/>
       <c r="X23" s="6"/>
       <c r="Y23" s="6"/>
-      <c r="Z23" s="6" t="s">
-        <v>364</v>
-      </c>
+      <c r="Z23" s="6"/>
       <c r="AA23" s="6"/>
       <c r="AB23" s="6"/>
       <c r="AC23" s="6"/>
-      <c r="AD23" s="6"/>
-      <c r="AE23" s="5" t="str">
+      <c r="AD23" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="AE23" s="6"/>
+      <c r="AF23" s="6"/>
+      <c r="AG23" s="6"/>
+      <c r="AH23" s="6"/>
+      <c r="AI23" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jasmin-cabuenas.jpg</v>
       </c>
-      <c r="AF23" s="6" t="s">
+      <c r="AJ23" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:32">
+    <row r="24" spans="1:36">
       <c r="A24" s="5">
         <v>23</v>
       </c>
@@ -4079,7 +4290,7 @@
         <v>12</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>
@@ -4096,29 +4307,35 @@
       <c r="R24" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S24" s="6"/>
+      <c r="S24" s="6" t="s">
+        <v>334</v>
+      </c>
       <c r="T24" s="6"/>
       <c r="U24" s="6"/>
       <c r="V24" s="6"/>
       <c r="W24" s="6"/>
       <c r="X24" s="6"/>
       <c r="Y24" s="6"/>
-      <c r="Z24" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z24" s="6"/>
       <c r="AA24" s="6"/>
       <c r="AB24" s="6"/>
       <c r="AC24" s="6"/>
-      <c r="AD24" s="6"/>
-      <c r="AE24" s="5" t="str">
+      <c r="AD24" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE24" s="6"/>
+      <c r="AF24" s="6"/>
+      <c r="AG24" s="6"/>
+      <c r="AH24" s="6"/>
+      <c r="AI24" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/elsa-calunod.jpg</v>
       </c>
-      <c r="AF24" s="6" t="s">
+      <c r="AJ24" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:32">
+    <row r="25" spans="1:36">
       <c r="A25" s="5">
         <v>24</v>
       </c>
@@ -4150,7 +4367,7 @@
         <v>352</v>
       </c>
       <c r="K25" s="10" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
@@ -4165,29 +4382,35 @@
       <c r="R25" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S25" s="6"/>
+      <c r="S25" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="T25" s="6"/>
       <c r="U25" s="6"/>
       <c r="V25" s="6"/>
       <c r="W25" s="6"/>
       <c r="X25" s="6"/>
       <c r="Y25" s="6"/>
-      <c r="Z25" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z25" s="6"/>
       <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>
       <c r="AC25" s="6"/>
-      <c r="AD25" s="6"/>
-      <c r="AE25" s="5" t="str">
+      <c r="AD25" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE25" s="6"/>
+      <c r="AF25" s="6"/>
+      <c r="AG25" s="6"/>
+      <c r="AH25" s="6"/>
+      <c r="AI25" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/leslyn-rose-camero.jpg</v>
       </c>
-      <c r="AF25" s="6" t="s">
+      <c r="AJ25" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:32">
+    <row r="26" spans="1:36">
       <c r="A26" s="5">
         <v>25</v>
       </c>
@@ -4230,29 +4453,35 @@
       <c r="R26" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S26" s="6"/>
+      <c r="S26" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="T26" s="6"/>
       <c r="U26" s="6"/>
       <c r="V26" s="6"/>
       <c r="W26" s="6"/>
       <c r="X26" s="6"/>
       <c r="Y26" s="6"/>
-      <c r="Z26" s="6" t="s">
-        <v>364</v>
-      </c>
+      <c r="Z26" s="6"/>
       <c r="AA26" s="6"/>
       <c r="AB26" s="6"/>
       <c r="AC26" s="6"/>
-      <c r="AD26" s="6"/>
-      <c r="AE26" s="5" t="str">
+      <c r="AD26" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="AE26" s="6"/>
+      <c r="AF26" s="6"/>
+      <c r="AG26" s="6"/>
+      <c r="AH26" s="6"/>
+      <c r="AI26" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/dawn-camille-caparida.jpg</v>
       </c>
-      <c r="AF26" s="6" t="s">
+      <c r="AJ26" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:32">
+    <row r="27" spans="1:36">
       <c r="A27" s="5">
         <v>26</v>
       </c>
@@ -4282,7 +4511,7 @@
         <v>354</v>
       </c>
       <c r="K27" s="10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
@@ -4297,29 +4526,35 @@
       <c r="R27" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="S27" s="6"/>
+      <c r="S27" s="6" t="s">
+        <v>384</v>
+      </c>
       <c r="T27" s="6"/>
       <c r="U27" s="6"/>
       <c r="V27" s="6"/>
       <c r="W27" s="6"/>
       <c r="X27" s="6"/>
       <c r="Y27" s="6"/>
-      <c r="Z27" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z27" s="6"/>
       <c r="AA27" s="6"/>
       <c r="AB27" s="6"/>
       <c r="AC27" s="6"/>
-      <c r="AD27" s="6"/>
-      <c r="AE27" s="5" t="str">
+      <c r="AD27" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE27" s="6"/>
+      <c r="AF27" s="6"/>
+      <c r="AG27" s="6"/>
+      <c r="AH27" s="6"/>
+      <c r="AI27" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lourence-capa.jpg</v>
       </c>
-      <c r="AF27" s="6" t="s">
+      <c r="AJ27" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:32">
+    <row r="28" spans="1:36">
       <c r="A28" s="5">
         <v>27</v>
       </c>
@@ -4351,7 +4586,7 @@
         <v>355</v>
       </c>
       <c r="K28" s="10" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
@@ -4366,29 +4601,35 @@
       <c r="R28" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S28" s="6"/>
+      <c r="S28" s="6" t="s">
+        <v>341</v>
+      </c>
       <c r="T28" s="6"/>
       <c r="U28" s="6"/>
       <c r="V28" s="6"/>
       <c r="W28" s="6"/>
       <c r="X28" s="6"/>
       <c r="Y28" s="6"/>
-      <c r="Z28" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z28" s="6"/>
       <c r="AA28" s="6"/>
       <c r="AB28" s="6"/>
       <c r="AC28" s="6"/>
-      <c r="AD28" s="6"/>
-      <c r="AE28" s="5" t="str">
+      <c r="AD28" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE28" s="6"/>
+      <c r="AF28" s="6"/>
+      <c r="AG28" s="6"/>
+      <c r="AH28" s="6"/>
+      <c r="AI28" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joan-cavite.jpg</v>
       </c>
-      <c r="AF28" s="6" t="s">
+      <c r="AJ28" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:32" ht="33.6">
+    <row r="29" spans="1:36" ht="33.6">
       <c r="A29" s="5">
         <v>28</v>
       </c>
@@ -4422,7 +4663,7 @@
         <v>356</v>
       </c>
       <c r="K29" s="10" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="L29" s="5"/>
       <c r="M29" s="5"/>
@@ -4444,22 +4685,26 @@
       <c r="W29" s="6"/>
       <c r="X29" s="6"/>
       <c r="Y29" s="6"/>
-      <c r="Z29" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z29" s="6"/>
       <c r="AA29" s="6"/>
       <c r="AB29" s="6"/>
       <c r="AC29" s="6"/>
-      <c r="AD29" s="6"/>
-      <c r="AE29" s="5" t="str">
+      <c r="AD29" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE29" s="6"/>
+      <c r="AF29" s="6"/>
+      <c r="AG29" s="6"/>
+      <c r="AH29" s="6"/>
+      <c r="AI29" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joseph-dagaraga.jpg</v>
       </c>
-      <c r="AF29" s="6" t="s">
+      <c r="AJ29" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:32">
+    <row r="30" spans="1:36">
       <c r="A30" s="5">
         <v>29</v>
       </c>
@@ -4503,28 +4748,34 @@
         <v>342</v>
       </c>
       <c r="S30" s="6"/>
-      <c r="T30" s="6"/>
+      <c r="T30" s="6" t="s">
+        <v>474</v>
+      </c>
       <c r="U30" s="6"/>
       <c r="V30" s="6"/>
       <c r="W30" s="6"/>
       <c r="X30" s="6"/>
       <c r="Y30" s="6"/>
-      <c r="Z30" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z30" s="6"/>
       <c r="AA30" s="6"/>
       <c r="AB30" s="6"/>
       <c r="AC30" s="6"/>
-      <c r="AD30" s="6"/>
-      <c r="AE30" s="5" t="str">
+      <c r="AD30" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE30" s="6"/>
+      <c r="AF30" s="6"/>
+      <c r="AG30" s="6"/>
+      <c r="AH30" s="6"/>
+      <c r="AI30" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carolyn-delos-reyes.jpg</v>
       </c>
-      <c r="AF30" s="6" t="s">
+      <c r="AJ30" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:32">
+    <row r="31" spans="1:36">
       <c r="A31" s="5">
         <v>30</v>
       </c>
@@ -4567,29 +4818,37 @@
       <c r="R31" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S31" s="6"/>
+      <c r="S31" s="6" t="s">
+        <v>343</v>
+      </c>
       <c r="T31" s="6"/>
       <c r="U31" s="6"/>
       <c r="V31" s="6"/>
       <c r="W31" s="6"/>
       <c r="X31" s="6"/>
       <c r="Y31" s="6"/>
-      <c r="Z31" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z31" s="6"/>
       <c r="AA31" s="6"/>
       <c r="AB31" s="6"/>
-      <c r="AC31" s="6"/>
-      <c r="AD31" s="6"/>
-      <c r="AE31" s="5" t="str">
+      <c r="AC31" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AD31" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE31" s="6"/>
+      <c r="AF31" s="6"/>
+      <c r="AG31" s="6"/>
+      <c r="AH31" s="6"/>
+      <c r="AI31" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lucille-echavez.jpg</v>
       </c>
-      <c r="AF31" s="6" t="s">
+      <c r="AJ31" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:32">
+    <row r="32" spans="1:36">
       <c r="A32" s="5">
         <v>31</v>
       </c>
@@ -4630,31 +4889,41 @@
         <v>14</v>
       </c>
       <c r="R32" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="S32" s="6"/>
+        <v>345</v>
+      </c>
+      <c r="S32" s="6" t="s">
+        <v>476</v>
+      </c>
       <c r="T32" s="6"/>
       <c r="U32" s="6"/>
       <c r="V32" s="6"/>
       <c r="W32" s="6"/>
-      <c r="X32" s="6"/>
+      <c r="X32" s="6" t="s">
+        <v>475</v>
+      </c>
       <c r="Y32" s="6"/>
-      <c r="Z32" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z32" s="6"/>
       <c r="AA32" s="6"/>
       <c r="AB32" s="6"/>
-      <c r="AC32" s="6"/>
-      <c r="AD32" s="6"/>
-      <c r="AE32" s="5" t="str">
+      <c r="AC32" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="AD32" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE32" s="6"/>
+      <c r="AF32" s="6"/>
+      <c r="AG32" s="6"/>
+      <c r="AH32" s="6"/>
+      <c r="AI32" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/benerando-erediano.jpg</v>
       </c>
-      <c r="AF32" s="6" t="s">
+      <c r="AJ32" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:32">
+    <row r="33" spans="1:36">
       <c r="A33" s="5">
         <v>32</v>
       </c>
@@ -4680,7 +4949,7 @@
         <v>244</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="J33" s="10"/>
       <c r="K33" s="10"/>
@@ -4697,31 +4966,37 @@
       <c r="R33" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S33" s="6"/>
+      <c r="S33" s="6" t="s">
+        <v>341</v>
+      </c>
       <c r="T33" s="6"/>
       <c r="U33" s="6"/>
       <c r="V33" s="6"/>
       <c r="W33" s="6"/>
       <c r="X33" s="6"/>
       <c r="Y33" s="6"/>
-      <c r="Z33" s="6" t="s">
-        <v>367</v>
-      </c>
+      <c r="Z33" s="6"/>
       <c r="AA33" s="6"/>
       <c r="AB33" s="6"/>
-      <c r="AC33" s="6">
+      <c r="AC33" s="6"/>
+      <c r="AD33" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="AE33" s="6"/>
+      <c r="AF33" s="6"/>
+      <c r="AG33" s="6">
         <v>4</v>
       </c>
-      <c r="AD33" s="6"/>
-      <c r="AE33" s="5" t="str">
+      <c r="AH33" s="6"/>
+      <c r="AI33" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/metchie-gay-gastanes.jpg</v>
       </c>
-      <c r="AF33" s="6" t="s">
+      <c r="AJ33" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:32">
+    <row r="34" spans="1:36">
       <c r="A34" s="5">
         <v>33</v>
       </c>
@@ -4764,29 +5039,35 @@
       <c r="R34" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="S34" s="6"/>
+      <c r="S34" s="6" t="s">
+        <v>477</v>
+      </c>
       <c r="T34" s="6"/>
       <c r="U34" s="6"/>
       <c r="V34" s="6"/>
       <c r="W34" s="6"/>
       <c r="X34" s="6"/>
       <c r="Y34" s="6"/>
-      <c r="Z34" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z34" s="6"/>
       <c r="AA34" s="6"/>
       <c r="AB34" s="6"/>
       <c r="AC34" s="6"/>
-      <c r="AD34" s="6"/>
-      <c r="AE34" s="5" t="str">
+      <c r="AD34" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE34" s="6"/>
+      <c r="AF34" s="6"/>
+      <c r="AG34" s="6"/>
+      <c r="AH34" s="6"/>
+      <c r="AI34" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jasmin-gerodias.jpg</v>
       </c>
-      <c r="AF34" s="6" t="s">
+      <c r="AJ34" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:32">
+    <row r="35" spans="1:36">
       <c r="A35" s="5">
         <v>34</v>
       </c>
@@ -4818,7 +5099,7 @@
         <v>353</v>
       </c>
       <c r="K35" s="10" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="L35" s="5"/>
       <c r="M35" s="5"/>
@@ -4840,22 +5121,26 @@
       <c r="W35" s="6"/>
       <c r="X35" s="6"/>
       <c r="Y35" s="6"/>
-      <c r="Z35" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z35" s="6"/>
       <c r="AA35" s="6"/>
       <c r="AB35" s="6"/>
       <c r="AC35" s="6"/>
-      <c r="AD35" s="6"/>
-      <c r="AE35" s="5" t="str">
+      <c r="AD35" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE35" s="6"/>
+      <c r="AF35" s="6"/>
+      <c r="AG35" s="6"/>
+      <c r="AH35" s="6"/>
+      <c r="AI35" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeralyn-gerra.jpg</v>
       </c>
-      <c r="AF35" s="6" t="s">
+      <c r="AJ35" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:32">
+    <row r="36" spans="1:36">
       <c r="A36" s="5">
         <v>35</v>
       </c>
@@ -4887,7 +5172,7 @@
         <v>353</v>
       </c>
       <c r="K36" s="10" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
@@ -4909,22 +5194,26 @@
       <c r="W36" s="6"/>
       <c r="X36" s="6"/>
       <c r="Y36" s="6"/>
-      <c r="Z36" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z36" s="6"/>
       <c r="AA36" s="6"/>
       <c r="AB36" s="6"/>
       <c r="AC36" s="6"/>
-      <c r="AD36" s="6"/>
-      <c r="AE36" s="5" t="str">
+      <c r="AD36" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE36" s="6"/>
+      <c r="AF36" s="6"/>
+      <c r="AG36" s="6"/>
+      <c r="AH36" s="6"/>
+      <c r="AI36" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/genesa-goc-ong.jpg</v>
       </c>
-      <c r="AF36" s="6" t="s">
+      <c r="AJ36" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:32">
+    <row r="37" spans="1:36">
       <c r="A37" s="5">
         <v>36</v>
       </c>
@@ -4974,22 +5263,26 @@
       <c r="W37" s="6"/>
       <c r="X37" s="6"/>
       <c r="Y37" s="6"/>
-      <c r="Z37" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z37" s="6"/>
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
       <c r="AC37" s="6"/>
-      <c r="AD37" s="6"/>
-      <c r="AE37" s="5" t="str">
+      <c r="AD37" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE37" s="6"/>
+      <c r="AF37" s="6"/>
+      <c r="AG37" s="6"/>
+      <c r="AH37" s="6"/>
+      <c r="AI37" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/janelou-gomez.jpg</v>
       </c>
-      <c r="AF37" s="6" t="s">
+      <c r="AJ37" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:32">
+    <row r="38" spans="1:36">
       <c r="A38" s="5">
         <v>37</v>
       </c>
@@ -5021,7 +5314,7 @@
         <v>352</v>
       </c>
       <c r="K38" s="10" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
@@ -5036,29 +5329,35 @@
       <c r="R38" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S38" s="6"/>
+      <c r="S38" s="6" t="s">
+        <v>334</v>
+      </c>
       <c r="T38" s="6"/>
       <c r="U38" s="6"/>
       <c r="V38" s="6"/>
       <c r="W38" s="6"/>
       <c r="X38" s="6"/>
       <c r="Y38" s="6"/>
-      <c r="Z38" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z38" s="6"/>
       <c r="AA38" s="6"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="6"/>
-      <c r="AD38" s="6"/>
-      <c r="AE38" s="5" t="str">
+      <c r="AD38" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE38" s="6"/>
+      <c r="AF38" s="6"/>
+      <c r="AG38" s="6"/>
+      <c r="AH38" s="6"/>
+      <c r="AI38" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/junnelyn-herbito.jpg</v>
       </c>
-      <c r="AF38" s="6" t="s">
+      <c r="AJ38" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:32">
+    <row r="39" spans="1:36">
       <c r="A39" s="5">
         <v>38</v>
       </c>
@@ -5090,7 +5389,7 @@
         <v>355</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="L39" s="5"/>
       <c r="M39" s="5"/>
@@ -5105,29 +5404,35 @@
       <c r="R39" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S39" s="6"/>
+      <c r="S39" s="6" t="s">
+        <v>334</v>
+      </c>
       <c r="T39" s="6"/>
       <c r="U39" s="6"/>
       <c r="V39" s="6"/>
       <c r="W39" s="6"/>
       <c r="X39" s="6"/>
       <c r="Y39" s="6"/>
-      <c r="Z39" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z39" s="6"/>
       <c r="AA39" s="6"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
-      <c r="AD39" s="6"/>
-      <c r="AE39" s="5" t="str">
+      <c r="AD39" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE39" s="6"/>
+      <c r="AF39" s="6"/>
+      <c r="AG39" s="6"/>
+      <c r="AH39" s="6"/>
+      <c r="AI39" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/roxan-mae-jao.jpg</v>
       </c>
-      <c r="AF39" s="6" t="s">
+      <c r="AJ39" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:32">
+    <row r="40" spans="1:36">
       <c r="A40" s="5">
         <v>39</v>
       </c>
@@ -5175,22 +5480,26 @@
       <c r="W40" s="6"/>
       <c r="X40" s="6"/>
       <c r="Y40" s="6"/>
-      <c r="Z40" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z40" s="6"/>
       <c r="AA40" s="6"/>
       <c r="AB40" s="6"/>
       <c r="AC40" s="6"/>
-      <c r="AD40" s="6"/>
-      <c r="AE40" s="5" t="str">
+      <c r="AD40" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE40" s="6"/>
+      <c r="AF40" s="6"/>
+      <c r="AG40" s="6"/>
+      <c r="AH40" s="6"/>
+      <c r="AI40" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/fernando-laspiñas.jpg</v>
       </c>
-      <c r="AF40" s="6" t="s">
+      <c r="AJ40" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:32">
+    <row r="41" spans="1:36">
       <c r="A41" s="5">
         <v>40</v>
       </c>
@@ -5233,29 +5542,35 @@
       <c r="R41" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S41" s="6"/>
+      <c r="S41" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="T41" s="6"/>
       <c r="U41" s="6"/>
       <c r="V41" s="6"/>
       <c r="W41" s="6"/>
       <c r="X41" s="6"/>
       <c r="Y41" s="6"/>
-      <c r="Z41" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z41" s="6"/>
       <c r="AA41" s="6"/>
       <c r="AB41" s="6"/>
       <c r="AC41" s="6"/>
-      <c r="AD41" s="6"/>
-      <c r="AE41" s="5" t="str">
+      <c r="AD41" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE41" s="6"/>
+      <c r="AF41" s="6"/>
+      <c r="AG41" s="6"/>
+      <c r="AH41" s="6"/>
+      <c r="AI41" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/nerisa-lim.jpg</v>
       </c>
-      <c r="AF41" s="6" t="s">
+      <c r="AJ41" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:32">
+    <row r="42" spans="1:36">
       <c r="A42" s="5">
         <v>41</v>
       </c>
@@ -5301,22 +5616,26 @@
       <c r="W42" s="6"/>
       <c r="X42" s="6"/>
       <c r="Y42" s="6"/>
-      <c r="Z42" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z42" s="6"/>
       <c r="AA42" s="6"/>
       <c r="AB42" s="6"/>
       <c r="AC42" s="6"/>
-      <c r="AD42" s="6"/>
-      <c r="AE42" s="5" t="str">
+      <c r="AD42" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE42" s="6"/>
+      <c r="AF42" s="6"/>
+      <c r="AG42" s="6"/>
+      <c r="AH42" s="6"/>
+      <c r="AI42" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carl-loreto.jpg</v>
       </c>
-      <c r="AF42" s="6" t="s">
+      <c r="AJ42" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:32">
+    <row r="43" spans="1:36">
       <c r="A43" s="5">
         <v>42</v>
       </c>
@@ -5364,22 +5683,26 @@
       <c r="W43" s="6"/>
       <c r="X43" s="6"/>
       <c r="Y43" s="6"/>
-      <c r="Z43" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z43" s="6"/>
       <c r="AA43" s="6"/>
       <c r="AB43" s="6"/>
       <c r="AC43" s="6"/>
-      <c r="AD43" s="6"/>
-      <c r="AE43" s="5" t="str">
+      <c r="AD43" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE43" s="6"/>
+      <c r="AF43" s="6"/>
+      <c r="AG43" s="6"/>
+      <c r="AH43" s="6"/>
+      <c r="AI43" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/lyka-mabanag.jpg</v>
       </c>
-      <c r="AF43" s="6" t="s">
+      <c r="AJ43" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:32">
+    <row r="44" spans="1:36">
       <c r="A44" s="5">
         <v>43</v>
       </c>
@@ -5426,29 +5749,35 @@
       <c r="R44" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="S44" s="6"/>
+      <c r="S44" s="6" t="s">
+        <v>476</v>
+      </c>
       <c r="T44" s="6"/>
       <c r="U44" s="6"/>
       <c r="V44" s="6"/>
       <c r="W44" s="6"/>
       <c r="X44" s="6"/>
       <c r="Y44" s="6"/>
-      <c r="Z44" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z44" s="6"/>
       <c r="AA44" s="6"/>
       <c r="AB44" s="6"/>
       <c r="AC44" s="6"/>
-      <c r="AD44" s="6"/>
-      <c r="AE44" s="5" t="str">
+      <c r="AD44" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE44" s="6"/>
+      <c r="AF44" s="6"/>
+      <c r="AG44" s="6"/>
+      <c r="AH44" s="6"/>
+      <c r="AI44" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/richie-ryan-mabunay.jpg</v>
       </c>
-      <c r="AF44" s="6" t="s">
+      <c r="AJ44" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:32">
+    <row r="45" spans="1:36">
       <c r="A45" s="5">
         <v>44</v>
       </c>
@@ -5498,22 +5827,26 @@
       <c r="W45" s="6"/>
       <c r="X45" s="6"/>
       <c r="Y45" s="6"/>
-      <c r="Z45" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z45" s="6"/>
       <c r="AA45" s="6"/>
       <c r="AB45" s="6"/>
       <c r="AC45" s="6"/>
-      <c r="AD45" s="6"/>
-      <c r="AE45" s="5" t="str">
+      <c r="AD45" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE45" s="6"/>
+      <c r="AF45" s="6"/>
+      <c r="AG45" s="6"/>
+      <c r="AH45" s="6"/>
+      <c r="AI45" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/maria-jeziel-macanin.jpg</v>
       </c>
-      <c r="AF45" s="6" t="s">
+      <c r="AJ45" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:32">
+    <row r="46" spans="1:36">
       <c r="A46" s="5">
         <v>45</v>
       </c>
@@ -5545,7 +5878,7 @@
         <v>354</v>
       </c>
       <c r="K46" s="10" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
@@ -5560,29 +5893,35 @@
       <c r="R46" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S46" s="6"/>
+      <c r="S46" s="6" t="s">
+        <v>341</v>
+      </c>
       <c r="T46" s="6"/>
       <c r="U46" s="6"/>
       <c r="V46" s="6"/>
       <c r="W46" s="6"/>
       <c r="X46" s="6"/>
       <c r="Y46" s="6"/>
-      <c r="Z46" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z46" s="6"/>
       <c r="AA46" s="6"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="6"/>
-      <c r="AD46" s="6"/>
-      <c r="AE46" s="5" t="str">
+      <c r="AD46" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE46" s="6"/>
+      <c r="AF46" s="6"/>
+      <c r="AG46" s="6"/>
+      <c r="AH46" s="6"/>
+      <c r="AI46" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jeralen-maloloy-on.jpg</v>
       </c>
-      <c r="AF46" s="6" t="s">
+      <c r="AJ46" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:32">
+    <row r="47" spans="1:36">
       <c r="A47" s="5">
         <v>46</v>
       </c>
@@ -5614,7 +5953,7 @@
         <v>352</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
@@ -5629,29 +5968,35 @@
       <c r="R47" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="S47" s="6"/>
+      <c r="S47" s="6" t="s">
+        <v>343</v>
+      </c>
       <c r="T47" s="6"/>
       <c r="U47" s="6"/>
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
       <c r="X47" s="6"/>
       <c r="Y47" s="6"/>
-      <c r="Z47" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z47" s="6"/>
       <c r="AA47" s="6"/>
       <c r="AB47" s="6"/>
       <c r="AC47" s="6"/>
-      <c r="AD47" s="6"/>
-      <c r="AE47" s="5" t="str">
+      <c r="AD47" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE47" s="6"/>
+      <c r="AF47" s="6"/>
+      <c r="AG47" s="6"/>
+      <c r="AH47" s="6"/>
+      <c r="AI47" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/elbert-misterio.jpg</v>
       </c>
-      <c r="AF47" s="6" t="s">
+      <c r="AJ47" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:32">
+    <row r="48" spans="1:36">
       <c r="A48" s="5">
         <v>47</v>
       </c>
@@ -5683,7 +6028,7 @@
         <v>353</v>
       </c>
       <c r="K48" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
@@ -5703,22 +6048,26 @@
       <c r="W48" s="6"/>
       <c r="X48" s="6"/>
       <c r="Y48" s="6"/>
-      <c r="Z48" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z48" s="6"/>
       <c r="AA48" s="6"/>
       <c r="AB48" s="6"/>
       <c r="AC48" s="6"/>
-      <c r="AD48" s="6"/>
-      <c r="AE48" s="5" t="str">
+      <c r="AD48" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE48" s="6"/>
+      <c r="AF48" s="6"/>
+      <c r="AG48" s="6"/>
+      <c r="AH48" s="6"/>
+      <c r="AI48" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joy-mortal.jpg</v>
       </c>
-      <c r="AF48" s="6" t="s">
+      <c r="AJ48" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:32">
+    <row r="49" spans="1:36">
       <c r="A49" s="5">
         <v>48</v>
       </c>
@@ -5766,22 +6115,26 @@
       <c r="W49" s="6"/>
       <c r="X49" s="6"/>
       <c r="Y49" s="6"/>
-      <c r="Z49" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z49" s="6"/>
       <c r="AA49" s="6"/>
       <c r="AB49" s="6"/>
       <c r="AC49" s="6"/>
-      <c r="AD49" s="6"/>
-      <c r="AE49" s="5" t="str">
+      <c r="AD49" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE49" s="6"/>
+      <c r="AF49" s="6"/>
+      <c r="AG49" s="6"/>
+      <c r="AH49" s="6"/>
+      <c r="AI49" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/claire-medillo.jpg</v>
       </c>
-      <c r="AF49" s="6" t="s">
+      <c r="AJ49" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:32">
+    <row r="50" spans="1:36">
       <c r="A50" s="5">
         <v>49</v>
       </c>
@@ -5813,7 +6166,7 @@
         <v>352</v>
       </c>
       <c r="K50" s="10" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
@@ -5828,29 +6181,35 @@
       <c r="R50" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="S50" s="6"/>
+      <c r="S50" s="6" t="s">
+        <v>341</v>
+      </c>
       <c r="T50" s="6"/>
       <c r="U50" s="6"/>
       <c r="V50" s="6"/>
       <c r="W50" s="6"/>
       <c r="X50" s="6"/>
       <c r="Y50" s="6"/>
-      <c r="Z50" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z50" s="6"/>
       <c r="AA50" s="6"/>
       <c r="AB50" s="6"/>
       <c r="AC50" s="6"/>
-      <c r="AD50" s="6"/>
-      <c r="AE50" s="5" t="str">
+      <c r="AD50" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE50" s="6"/>
+      <c r="AF50" s="6"/>
+      <c r="AG50" s="6"/>
+      <c r="AH50" s="6"/>
+      <c r="AI50" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/gwendolyn-olo.jpg</v>
       </c>
-      <c r="AF50" s="6" t="s">
+      <c r="AJ50" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:32">
+    <row r="51" spans="1:36">
       <c r="A51" s="5">
         <v>50</v>
       </c>
@@ -5882,7 +6241,7 @@
         <v>355</v>
       </c>
       <c r="K51" s="10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
@@ -5902,22 +6261,26 @@
       <c r="W51" s="6"/>
       <c r="X51" s="6"/>
       <c r="Y51" s="6"/>
-      <c r="Z51" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z51" s="6"/>
       <c r="AA51" s="6"/>
       <c r="AB51" s="6"/>
       <c r="AC51" s="6"/>
-      <c r="AD51" s="6"/>
-      <c r="AE51" s="5" t="str">
+      <c r="AD51" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE51" s="6"/>
+      <c r="AF51" s="6"/>
+      <c r="AG51" s="6"/>
+      <c r="AH51" s="6"/>
+      <c r="AI51" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jay-neil-oro.jpg</v>
       </c>
-      <c r="AF51" s="6" t="s">
+      <c r="AJ51" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:32">
+    <row r="52" spans="1:36">
       <c r="A52" s="5">
         <v>51</v>
       </c>
@@ -5949,7 +6312,7 @@
         <v>357</v>
       </c>
       <c r="K52" s="10" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
@@ -5962,31 +6325,37 @@
         <v>14</v>
       </c>
       <c r="R52" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="S52" s="6"/>
+        <v>387</v>
+      </c>
+      <c r="S52" s="6" t="s">
+        <v>476</v>
+      </c>
       <c r="T52" s="6"/>
       <c r="U52" s="6"/>
       <c r="V52" s="6"/>
       <c r="W52" s="6"/>
       <c r="X52" s="6"/>
       <c r="Y52" s="6"/>
-      <c r="Z52" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z52" s="6"/>
       <c r="AA52" s="6"/>
       <c r="AB52" s="6"/>
       <c r="AC52" s="6"/>
-      <c r="AD52" s="6"/>
-      <c r="AE52" s="5" t="str">
+      <c r="AD52" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE52" s="6"/>
+      <c r="AF52" s="6"/>
+      <c r="AG52" s="6"/>
+      <c r="AH52" s="6"/>
+      <c r="AI52" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/glendale-orocay.jpg</v>
       </c>
-      <c r="AF52" s="6" t="s">
+      <c r="AJ52" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:32" ht="33.6">
+    <row r="53" spans="1:36" ht="33.6">
       <c r="A53" s="5">
         <v>52</v>
       </c>
@@ -6018,7 +6387,7 @@
         <v>356</v>
       </c>
       <c r="K53" s="10" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="L53" s="5"/>
       <c r="M53" s="5"/>
@@ -6033,29 +6402,35 @@
       <c r="R53" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="S53" s="6"/>
+      <c r="S53" s="6" t="s">
+        <v>384</v>
+      </c>
       <c r="T53" s="6"/>
       <c r="U53" s="6"/>
       <c r="V53" s="6"/>
       <c r="W53" s="6"/>
       <c r="X53" s="6"/>
       <c r="Y53" s="6"/>
-      <c r="Z53" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z53" s="6"/>
       <c r="AA53" s="6"/>
       <c r="AB53" s="6"/>
       <c r="AC53" s="6"/>
-      <c r="AD53" s="6"/>
-      <c r="AE53" s="5" t="str">
+      <c r="AD53" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE53" s="6"/>
+      <c r="AF53" s="6"/>
+      <c r="AG53" s="6"/>
+      <c r="AH53" s="6"/>
+      <c r="AI53" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marissa-pintuan.jpg</v>
       </c>
-      <c r="AF53" s="6" t="s">
+      <c r="AJ53" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:32">
+    <row r="54" spans="1:36">
       <c r="A54" s="5">
         <v>53</v>
       </c>
@@ -6105,22 +6480,26 @@
       <c r="W54" s="6"/>
       <c r="X54" s="6"/>
       <c r="Y54" s="6"/>
-      <c r="Z54" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z54" s="6"/>
       <c r="AA54" s="6"/>
       <c r="AB54" s="6"/>
       <c r="AC54" s="6"/>
-      <c r="AD54" s="6"/>
-      <c r="AE54" s="5" t="str">
+      <c r="AD54" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE54" s="6"/>
+      <c r="AF54" s="6"/>
+      <c r="AG54" s="6"/>
+      <c r="AH54" s="6"/>
+      <c r="AI54" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/ma.-lourdes-prajes.jpg</v>
       </c>
-      <c r="AF54" s="6" t="s">
+      <c r="AJ54" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:32">
+    <row r="55" spans="1:36">
       <c r="A55" s="5">
         <v>54</v>
       </c>
@@ -6152,7 +6531,7 @@
         <v>353</v>
       </c>
       <c r="K55" s="10" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
@@ -6172,22 +6551,26 @@
       <c r="W55" s="6"/>
       <c r="X55" s="6"/>
       <c r="Y55" s="6"/>
-      <c r="Z55" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z55" s="6"/>
       <c r="AA55" s="6"/>
       <c r="AB55" s="6"/>
       <c r="AC55" s="6"/>
-      <c r="AD55" s="6"/>
-      <c r="AE55" s="5" t="str">
+      <c r="AD55" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE55" s="6"/>
+      <c r="AF55" s="6"/>
+      <c r="AG55" s="6"/>
+      <c r="AH55" s="6"/>
+      <c r="AI55" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/bret-kalvin-primacio.jpg</v>
       </c>
-      <c r="AF55" s="6" t="s">
+      <c r="AJ55" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:32">
+    <row r="56" spans="1:36">
       <c r="A56" s="5">
         <v>55</v>
       </c>
@@ -6230,29 +6613,35 @@
       <c r="R56" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S56" s="6"/>
+      <c r="S56" s="6" t="s">
+        <v>334</v>
+      </c>
       <c r="T56" s="6"/>
       <c r="U56" s="6"/>
       <c r="V56" s="6"/>
       <c r="W56" s="6"/>
       <c r="X56" s="6"/>
       <c r="Y56" s="6"/>
-      <c r="Z56" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z56" s="6"/>
       <c r="AA56" s="6"/>
       <c r="AB56" s="6"/>
       <c r="AC56" s="6"/>
-      <c r="AD56" s="6"/>
-      <c r="AE56" s="5" t="str">
+      <c r="AD56" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE56" s="6"/>
+      <c r="AF56" s="6"/>
+      <c r="AG56" s="6"/>
+      <c r="AH56" s="6"/>
+      <c r="AI56" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jhea-quiling.jpg</v>
       </c>
-      <c r="AF56" s="6" t="s">
+      <c r="AJ56" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:32">
+    <row r="57" spans="1:36">
       <c r="A57" s="5">
         <v>56</v>
       </c>
@@ -6295,29 +6684,35 @@
       <c r="R57" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S57" s="6"/>
+      <c r="S57" s="6" t="s">
+        <v>342</v>
+      </c>
       <c r="T57" s="6"/>
       <c r="U57" s="6"/>
       <c r="V57" s="6"/>
       <c r="W57" s="6"/>
       <c r="X57" s="6"/>
       <c r="Y57" s="6"/>
-      <c r="Z57" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z57" s="6"/>
       <c r="AA57" s="6"/>
       <c r="AB57" s="6"/>
       <c r="AC57" s="6"/>
-      <c r="AD57" s="6"/>
-      <c r="AE57" s="5" t="str">
+      <c r="AD57" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE57" s="6"/>
+      <c r="AF57" s="6"/>
+      <c r="AG57" s="6"/>
+      <c r="AH57" s="6"/>
+      <c r="AI57" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/joyce-racaza.jpg</v>
       </c>
-      <c r="AF57" s="6" t="s">
+      <c r="AJ57" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:32">
+    <row r="58" spans="1:36">
       <c r="A58" s="5">
         <v>57</v>
       </c>
@@ -6360,29 +6755,35 @@
       <c r="R58" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="S58" s="6"/>
+      <c r="S58" s="6" t="s">
+        <v>477</v>
+      </c>
       <c r="T58" s="6"/>
       <c r="U58" s="6"/>
       <c r="V58" s="6"/>
       <c r="W58" s="6"/>
       <c r="X58" s="6"/>
       <c r="Y58" s="6"/>
-      <c r="Z58" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z58" s="6"/>
       <c r="AA58" s="6"/>
       <c r="AB58" s="6"/>
       <c r="AC58" s="6"/>
-      <c r="AD58" s="6"/>
-      <c r="AE58" s="5" t="str">
+      <c r="AD58" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE58" s="6"/>
+      <c r="AF58" s="6"/>
+      <c r="AG58" s="6"/>
+      <c r="AH58" s="6"/>
+      <c r="AI58" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/cromwell-retuya.jpg</v>
       </c>
-      <c r="AF58" s="6" t="s">
+      <c r="AJ58" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:32">
+    <row r="59" spans="1:36">
       <c r="A59" s="5">
         <v>58</v>
       </c>
@@ -6408,7 +6809,7 @@
         <v>12</v>
       </c>
       <c r="I59" s="10" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="J59" s="10"/>
       <c r="K59" s="10"/>
@@ -6425,31 +6826,37 @@
       <c r="R59" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="S59" s="6"/>
+      <c r="S59" s="6" t="s">
+        <v>384</v>
+      </c>
       <c r="T59" s="6"/>
       <c r="U59" s="6"/>
       <c r="V59" s="6"/>
       <c r="W59" s="6"/>
       <c r="X59" s="6"/>
       <c r="Y59" s="6"/>
-      <c r="Z59" s="6" t="s">
-        <v>367</v>
-      </c>
+      <c r="Z59" s="6"/>
       <c r="AA59" s="6"/>
       <c r="AB59" s="6"/>
-      <c r="AC59" s="6">
+      <c r="AC59" s="6"/>
+      <c r="AD59" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="AE59" s="6"/>
+      <c r="AF59" s="6"/>
+      <c r="AG59" s="6">
         <v>5</v>
       </c>
-      <c r="AD59" s="6"/>
-      <c r="AE59" s="5" t="str">
+      <c r="AH59" s="6"/>
+      <c r="AI59" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/nancy-reyes.jpg</v>
       </c>
-      <c r="AF59" s="6" t="s">
+      <c r="AJ59" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:32">
+    <row r="60" spans="1:36">
       <c r="A60" s="5">
         <v>59</v>
       </c>
@@ -6481,7 +6888,7 @@
         <v>354</v>
       </c>
       <c r="K60" s="10" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="L60" s="5"/>
       <c r="M60" s="5"/>
@@ -6501,22 +6908,26 @@
       <c r="W60" s="6"/>
       <c r="X60" s="6"/>
       <c r="Y60" s="6"/>
-      <c r="Z60" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z60" s="6"/>
       <c r="AA60" s="6"/>
       <c r="AB60" s="6"/>
       <c r="AC60" s="6"/>
-      <c r="AD60" s="6"/>
-      <c r="AE60" s="5" t="str">
+      <c r="AD60" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE60" s="6"/>
+      <c r="AF60" s="6"/>
+      <c r="AG60" s="6"/>
+      <c r="AH60" s="6"/>
+      <c r="AI60" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/angelo-saavedra.jpg</v>
       </c>
-      <c r="AF60" s="6" t="s">
+      <c r="AJ60" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:32">
+    <row r="61" spans="1:36">
       <c r="A61" s="5">
         <v>60</v>
       </c>
@@ -6542,7 +6953,7 @@
         <v>244</v>
       </c>
       <c r="I61" s="10" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="J61" s="10"/>
       <c r="K61" s="10"/>
@@ -6557,31 +6968,37 @@
         <v>17</v>
       </c>
       <c r="R61" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="S61" s="6"/>
+        <v>388</v>
+      </c>
+      <c r="S61" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="T61" s="6"/>
       <c r="U61" s="6"/>
       <c r="V61" s="6"/>
       <c r="W61" s="6"/>
       <c r="X61" s="6"/>
       <c r="Y61" s="6"/>
-      <c r="Z61" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z61" s="6"/>
       <c r="AA61" s="6"/>
       <c r="AB61" s="6"/>
       <c r="AC61" s="6"/>
-      <c r="AD61" s="6"/>
-      <c r="AE61" s="5" t="str">
+      <c r="AD61" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE61" s="6"/>
+      <c r="AF61" s="6"/>
+      <c r="AG61" s="6"/>
+      <c r="AH61" s="6"/>
+      <c r="AI61" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/brendel-sacaris.jpg</v>
       </c>
-      <c r="AF61" s="6" t="s">
+      <c r="AJ61" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:32">
+    <row r="62" spans="1:36">
       <c r="A62" s="5">
         <v>61</v>
       </c>
@@ -6613,7 +7030,7 @@
         <v>354</v>
       </c>
       <c r="K62" s="10" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="L62" s="5"/>
       <c r="M62" s="5"/>
@@ -6626,29 +7043,35 @@
         <v>17</v>
       </c>
       <c r="R62" s="6"/>
-      <c r="S62" s="6"/>
+      <c r="S62" s="6" t="s">
+        <v>477</v>
+      </c>
       <c r="T62" s="6"/>
       <c r="U62" s="6"/>
       <c r="V62" s="6"/>
       <c r="W62" s="6"/>
       <c r="X62" s="6"/>
       <c r="Y62" s="6"/>
-      <c r="Z62" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z62" s="6"/>
       <c r="AA62" s="6"/>
       <c r="AB62" s="6"/>
       <c r="AC62" s="6"/>
-      <c r="AD62" s="6"/>
-      <c r="AE62" s="5" t="str">
+      <c r="AD62" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE62" s="6"/>
+      <c r="AF62" s="6"/>
+      <c r="AG62" s="6"/>
+      <c r="AH62" s="6"/>
+      <c r="AI62" s="5" t="str">
         <f>"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C62&amp;" "&amp;B62)," ","-"))&amp;".jpg"</f>
         <v>/personnel/bella-arquine-samontañez.jpg</v>
       </c>
-      <c r="AF62" s="6" t="s">
+      <c r="AJ62" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:32">
+    <row r="63" spans="1:36">
       <c r="A63" s="5">
         <v>62</v>
       </c>
@@ -6680,7 +7103,7 @@
         <v>357</v>
       </c>
       <c r="K63" s="10" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="L63" s="5"/>
       <c r="M63" s="5"/>
@@ -6695,29 +7118,35 @@
       <c r="R63" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="S63" s="6"/>
+      <c r="S63" s="6" t="s">
+        <v>334</v>
+      </c>
       <c r="T63" s="6"/>
       <c r="U63" s="6"/>
       <c r="V63" s="6"/>
       <c r="W63" s="6"/>
       <c r="X63" s="6"/>
       <c r="Y63" s="6"/>
-      <c r="Z63" s="6" t="s">
-        <v>277</v>
-      </c>
+      <c r="Z63" s="6"/>
       <c r="AA63" s="6"/>
       <c r="AB63" s="6"/>
       <c r="AC63" s="6"/>
-      <c r="AD63" s="6"/>
-      <c r="AE63" s="5" t="str">
+      <c r="AD63" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="AE63" s="6"/>
+      <c r="AF63" s="6"/>
+      <c r="AG63" s="6"/>
+      <c r="AH63" s="6"/>
+      <c r="AI63" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/jevy-ann-uy.jpg</v>
       </c>
-      <c r="AF63" s="6" t="s">
+      <c r="AJ63" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:32">
+    <row r="64" spans="1:36">
       <c r="A64" s="5">
         <v>63</v>
       </c>
@@ -6760,29 +7189,35 @@
       <c r="R64" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="S64" s="6"/>
+      <c r="S64" s="6" t="s">
+        <v>342</v>
+      </c>
       <c r="T64" s="6"/>
       <c r="U64" s="6"/>
       <c r="V64" s="6"/>
       <c r="W64" s="6"/>
       <c r="X64" s="6"/>
       <c r="Y64" s="6"/>
-      <c r="Z64" s="6" t="s">
-        <v>365</v>
-      </c>
+      <c r="Z64" s="6"/>
       <c r="AA64" s="6"/>
       <c r="AB64" s="6"/>
       <c r="AC64" s="6"/>
-      <c r="AD64" s="6"/>
-      <c r="AE64" s="5" t="str">
+      <c r="AD64" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE64" s="6"/>
+      <c r="AF64" s="6"/>
+      <c r="AG64" s="6"/>
+      <c r="AH64" s="6"/>
+      <c r="AI64" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/grace-vergara.jpg</v>
       </c>
-      <c r="AF64" s="6" t="s">
+      <c r="AJ64" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:32">
+    <row r="65" spans="1:36">
       <c r="A65" s="5">
         <v>64</v>
       </c>
@@ -6825,29 +7260,35 @@
       <c r="R65" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S65" s="6"/>
+      <c r="S65" s="6" t="s">
+        <v>7</v>
+      </c>
       <c r="T65" s="6"/>
       <c r="U65" s="6"/>
       <c r="V65" s="6"/>
       <c r="W65" s="6"/>
       <c r="X65" s="6"/>
       <c r="Y65" s="6"/>
-      <c r="Z65" s="6" t="s">
-        <v>271</v>
-      </c>
+      <c r="Z65" s="6"/>
       <c r="AA65" s="6"/>
       <c r="AB65" s="6"/>
       <c r="AC65" s="6"/>
-      <c r="AD65" s="6"/>
-      <c r="AE65" s="5" t="str">
+      <c r="AD65" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="AE65" s="6"/>
+      <c r="AF65" s="6"/>
+      <c r="AG65" s="6"/>
+      <c r="AH65" s="6"/>
+      <c r="AI65" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/guillermo-villavelez.jpg</v>
       </c>
-      <c r="AF65" s="6" t="s">
+      <c r="AJ65" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:32">
+    <row r="66" spans="1:36">
       <c r="A66" s="5">
         <v>65</v>
       </c>
@@ -6890,29 +7331,35 @@
       <c r="R66" s="6" t="s">
         <v>339</v>
       </c>
-      <c r="S66" s="6"/>
+      <c r="S66" s="6" t="s">
+        <v>339</v>
+      </c>
       <c r="T66" s="6"/>
       <c r="U66" s="6"/>
       <c r="V66" s="6"/>
       <c r="W66" s="6"/>
       <c r="X66" s="6"/>
       <c r="Y66" s="6"/>
-      <c r="Z66" s="6" t="s">
-        <v>369</v>
-      </c>
+      <c r="Z66" s="6"/>
       <c r="AA66" s="6"/>
       <c r="AB66" s="6"/>
       <c r="AC66" s="6"/>
-      <c r="AD66" s="6"/>
-      <c r="AE66" s="5" t="str">
+      <c r="AD66" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="AE66" s="6"/>
+      <c r="AF66" s="6"/>
+      <c r="AG66" s="6"/>
+      <c r="AH66" s="6"/>
+      <c r="AI66" s="5" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/marilou-villaver.jpg</v>
       </c>
-      <c r="AF66" s="6" t="s">
+      <c r="AJ66" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:32">
+    <row r="67" spans="1:36">
       <c r="A67" s="5">
         <v>66</v>
       </c>
@@ -6955,29 +7402,35 @@
       <c r="R67" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S67" s="6"/>
+      <c r="S67" s="6" t="s">
+        <v>385</v>
+      </c>
       <c r="T67" s="6"/>
       <c r="U67" s="6"/>
       <c r="V67" s="6"/>
       <c r="W67" s="6"/>
       <c r="X67" s="6"/>
       <c r="Y67" s="6"/>
-      <c r="Z67" s="6" t="s">
-        <v>370</v>
-      </c>
+      <c r="Z67" s="6"/>
       <c r="AA67" s="6"/>
       <c r="AB67" s="6"/>
       <c r="AC67" s="6"/>
-      <c r="AD67" s="6"/>
-      <c r="AE67" s="5" t="str">
-        <f t="shared" ref="AE67:AE68" si="8">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C67&amp;" "&amp;B67)," ","-"))&amp;".jpg"</f>
+      <c r="AD67" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AE67" s="6"/>
+      <c r="AF67" s="6"/>
+      <c r="AG67" s="6"/>
+      <c r="AH67" s="6"/>
+      <c r="AI67" s="5" t="str">
+        <f t="shared" ref="AI67:AI68" si="8">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C67&amp;" "&amp;B67)," ","-"))&amp;".jpg"</f>
         <v>/personnel/markjil-bacaltos.jpg</v>
       </c>
-      <c r="AF67" s="6" t="s">
+      <c r="AJ67" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:32">
+    <row r="68" spans="1:36">
       <c r="A68" s="5">
         <v>67</v>
       </c>
@@ -7020,29 +7473,35 @@
       <c r="R68" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S68" s="6"/>
+      <c r="S68" s="6" t="s">
+        <v>385</v>
+      </c>
       <c r="T68" s="6"/>
       <c r="U68" s="6"/>
       <c r="V68" s="6"/>
       <c r="W68" s="6"/>
       <c r="X68" s="6"/>
       <c r="Y68" s="6"/>
-      <c r="Z68" s="6" t="s">
-        <v>370</v>
-      </c>
+      <c r="Z68" s="6"/>
       <c r="AA68" s="6"/>
       <c r="AB68" s="6"/>
       <c r="AC68" s="6"/>
-      <c r="AD68" s="6"/>
-      <c r="AE68" s="5" t="str">
+      <c r="AD68" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AE68" s="6"/>
+      <c r="AF68" s="6"/>
+      <c r="AG68" s="6"/>
+      <c r="AH68" s="6"/>
+      <c r="AI68" s="5" t="str">
         <f t="shared" si="8"/>
         <v>/personnel/diocel-celocia.jpg</v>
       </c>
-      <c r="AF68" s="6" t="s">
+      <c r="AJ68" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:32">
+    <row r="69" spans="1:36">
       <c r="A69" s="5">
         <v>68</v>
       </c>
@@ -7085,29 +7544,35 @@
       <c r="R69" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S69" s="6"/>
+      <c r="S69" s="6" t="s">
+        <v>385</v>
+      </c>
       <c r="T69" s="6"/>
       <c r="U69" s="6"/>
       <c r="V69" s="6"/>
       <c r="W69" s="6"/>
       <c r="X69" s="6"/>
       <c r="Y69" s="6"/>
-      <c r="Z69" s="6" t="s">
-        <v>370</v>
-      </c>
+      <c r="Z69" s="6"/>
       <c r="AA69" s="6"/>
       <c r="AB69" s="6"/>
       <c r="AC69" s="6"/>
-      <c r="AD69" s="6"/>
-      <c r="AE69" s="5" t="str">
-        <f t="shared" ref="AE69:AE70" si="11">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C69&amp;" "&amp;B69)," ","-"))&amp;".jpg"</f>
+      <c r="AD69" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AE69" s="6"/>
+      <c r="AF69" s="6"/>
+      <c r="AG69" s="6"/>
+      <c r="AH69" s="6"/>
+      <c r="AI69" s="5" t="str">
+        <f t="shared" ref="AI69:AI70" si="11">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C69&amp;" "&amp;B69)," ","-"))&amp;".jpg"</f>
         <v>/personnel/luie-cabs.jpg</v>
       </c>
-      <c r="AF69" s="6" t="s">
+      <c r="AJ69" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:32">
+    <row r="70" spans="1:36">
       <c r="A70" s="5">
         <v>69</v>
       </c>
@@ -7150,29 +7615,35 @@
       <c r="R70" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="S70" s="6"/>
+      <c r="S70" s="6" t="s">
+        <v>385</v>
+      </c>
       <c r="T70" s="6"/>
       <c r="U70" s="6"/>
       <c r="V70" s="6"/>
       <c r="W70" s="6"/>
       <c r="X70" s="6"/>
       <c r="Y70" s="6"/>
-      <c r="Z70" s="6" t="s">
-        <v>370</v>
-      </c>
+      <c r="Z70" s="6"/>
       <c r="AA70" s="6"/>
       <c r="AB70" s="6"/>
       <c r="AC70" s="6"/>
-      <c r="AD70" s="6"/>
-      <c r="AE70" s="5" t="str">
+      <c r="AD70" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="AE70" s="6"/>
+      <c r="AF70" s="6"/>
+      <c r="AG70" s="6"/>
+      <c r="AH70" s="6"/>
+      <c r="AI70" s="5" t="str">
         <f t="shared" si="11"/>
         <v>/personnel/luis-mans.jpg</v>
       </c>
-      <c r="AF70" s="6" t="s">
+      <c r="AJ70" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:32">
+    <row r="71" spans="1:36">
       <c r="A71" s="5">
         <v>70</v>
       </c>
@@ -7208,8 +7679,12 @@
       <c r="AB71" s="6"/>
       <c r="AC71" s="6"/>
       <c r="AD71" s="6"/>
-      <c r="AE71" s="5"/>
+      <c r="AE71" s="6"/>
       <c r="AF71" s="6"/>
+      <c r="AG71" s="6"/>
+      <c r="AH71" s="6"/>
+      <c r="AI71" s="5"/>
+      <c r="AJ71" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -7242,19 +7717,19 @@
           <x14:formula1>
             <xm:f>Dropdown_Lists!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>AF2:AF71</xm:sqref>
+          <xm:sqref>AJ2:AJ71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{70D54F6E-2A67-40F0-92CA-B6E53F44843D}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$D$2:$D$61</xm:f>
           </x14:formula1>
-          <xm:sqref>Z2:Z71</xm:sqref>
+          <xm:sqref>AD2:AD71</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7834D497-9733-4178-89DF-4B7895726F53}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$E$2:$E$60</xm:f>
           </x14:formula1>
-          <xm:sqref>AA2:AA71</xm:sqref>
+          <xm:sqref>AE2:AE71</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Update organization personnel cards and profile modal
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A4156A-61C5-4F35-A02A-3EF891CEF649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF7F748-A227-49A9-A125-900F3BE35132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="511">
   <si>
     <t>order</t>
   </si>
@@ -1378,9 +1378,6 @@
     <t>Araling Panlipunan Coordinator (SHS)</t>
   </si>
   <si>
-    <t>AP</t>
-  </si>
-  <si>
     <t>Araling Panlipunan 9</t>
   </si>
   <si>
@@ -1561,16 +1558,16 @@
     <t>"Everything is a process, don't skip, don't jump to the next level without the experience needed."</t>
   </si>
   <si>
-    <t>Grade Leader (Grade 10)</t>
-  </si>
-  <si>
-    <t>Grade Leader (Grade 9)</t>
-  </si>
-  <si>
-    <t>Grade Leader (Grade 8)</t>
-  </si>
-  <si>
-    <t>Grade Leader (Grade 7)</t>
+    <t>10th Grade - Grade Leader</t>
+  </si>
+  <si>
+    <t>9th Grade - Grade Leader</t>
+  </si>
+  <si>
+    <t>8th Grade - Grade Leader</t>
+  </si>
+  <si>
+    <t>7th Grade - Grade Leader</t>
   </si>
 </sst>
 </file>
@@ -2665,16 +2662,16 @@
         <v>419</v>
       </c>
       <c r="T1" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="U1" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="U1" s="5" t="s">
+      <c r="V1" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="V1" s="5" t="s">
+      <c r="W1" s="5" t="s">
         <v>470</v>
-      </c>
-      <c r="W1" s="5" t="s">
-        <v>471</v>
       </c>
       <c r="X1" s="5" t="s">
         <v>420</v>
@@ -2710,10 +2707,10 @@
         <v>362</v>
       </c>
       <c r="AI1" s="5" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="AJ1" s="5" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="AK1" s="5" t="s">
         <v>5</v>
@@ -2748,12 +2745,12 @@
         <v>10</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="7" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
@@ -2795,7 +2792,7 @@
       <c r="AH2" s="8"/>
       <c r="AI2" s="8"/>
       <c r="AJ2" s="6" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="AK2" s="7" t="str">
         <f t="shared" ref="AK2:AK33" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C2&amp;" "&amp;B2)," ","-"))&amp;".jpg"</f>
@@ -2871,7 +2868,7 @@
       <c r="AA3" s="8"/>
       <c r="AB3" s="8"/>
       <c r="AC3" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AD3" s="8" t="s">
         <v>276</v>
@@ -2921,7 +2918,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="7" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
@@ -2943,7 +2940,7 @@
       <c r="V4" s="8"/>
       <c r="W4" s="8"/>
       <c r="X4" s="8" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="Y4" s="8"/>
       <c r="Z4" s="8"/>
@@ -2961,7 +2958,7 @@
       <c r="AH4" s="8"/>
       <c r="AI4" s="8"/>
       <c r="AJ4" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="AK4" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3106,14 +3103,14 @@
         <v>434</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
       <c r="V6" s="8"/>
       <c r="W6" s="8"/>
       <c r="X6" s="8" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="Y6" s="8" t="s">
         <v>435</v>
@@ -3190,17 +3187,17 @@
         <v>14</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S7" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
       <c r="V7" s="8"/>
       <c r="W7" s="8"/>
       <c r="X7" s="8" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="Y7" s="8"/>
       <c r="Z7" s="8"/>
@@ -3218,7 +3215,7 @@
       <c r="AH7" s="8"/>
       <c r="AI7" s="8"/>
       <c r="AJ7" s="6" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="AK7" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3323,7 +3320,7 @@
         <v>268</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
@@ -3413,17 +3410,17 @@
         <v>16</v>
       </c>
       <c r="R10" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S10" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="T10" s="8"/>
       <c r="U10" s="8"/>
       <c r="V10" s="8"/>
       <c r="W10" s="8"/>
       <c r="X10" s="8" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="Y10" s="8"/>
       <c r="Z10" s="8"/>
@@ -3609,7 +3606,7 @@
       <c r="AH12" s="8"/>
       <c r="AI12" s="8"/>
       <c r="AJ12" s="6" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="AK12" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3660,7 +3657,7 @@
         <v>445</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="O13" s="7"/>
       <c r="P13" s="8" t="s">
@@ -3673,23 +3670,23 @@
         <v>341</v>
       </c>
       <c r="S13" s="8" t="s">
-        <v>447</v>
+        <v>341</v>
       </c>
       <c r="T13" s="8"/>
       <c r="U13" s="8"/>
       <c r="V13" s="8"/>
       <c r="W13" s="8"/>
       <c r="X13" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="Y13" s="8" t="s">
         <v>448</v>
-      </c>
-      <c r="Y13" s="8" t="s">
-        <v>449</v>
       </c>
       <c r="Z13" s="8"/>
       <c r="AA13" s="8"/>
       <c r="AB13" s="8"/>
       <c r="AC13" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AD13" s="8" t="s">
         <v>276</v>
@@ -3700,7 +3697,7 @@
       <c r="AH13" s="8"/>
       <c r="AI13" s="8"/>
       <c r="AJ13" s="6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="AK13" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3736,7 +3733,7 @@
         <v>12</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
@@ -3761,7 +3758,7 @@
       <c r="V14" s="8"/>
       <c r="W14" s="8"/>
       <c r="X14" s="8" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="Y14" s="8"/>
       <c r="Z14" s="8"/>
@@ -3822,7 +3819,7 @@
         <v>393</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
@@ -3844,16 +3841,16 @@
       <c r="V15" s="8"/>
       <c r="W15" s="8"/>
       <c r="X15" s="8" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="Y15" s="8" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="Z15" s="8"/>
       <c r="AA15" s="8"/>
       <c r="AB15" s="8"/>
       <c r="AC15" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AD15" s="8" t="s">
         <v>276</v>
@@ -3864,7 +3861,7 @@
       <c r="AH15" s="8"/>
       <c r="AI15" s="8"/>
       <c r="AJ15" s="6" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="AK15" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3905,13 +3902,13 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
       <c r="L16" s="7" t="s">
+        <v>457</v>
+      </c>
+      <c r="M16" s="7" t="s">
         <v>458</v>
       </c>
-      <c r="M16" s="7" t="s">
-        <v>459</v>
-      </c>
       <c r="N16" s="7" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="O16" s="7"/>
       <c r="P16" s="8" t="s">
@@ -3931,10 +3928,10 @@
       <c r="V16" s="8"/>
       <c r="W16" s="8"/>
       <c r="X16" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="Y16" s="8" t="s">
         <v>460</v>
-      </c>
-      <c r="Y16" s="8" t="s">
-        <v>461</v>
       </c>
       <c r="Z16" s="8"/>
       <c r="AA16" s="8"/>
@@ -3953,7 +3950,7 @@
       <c r="AH16" s="8"/>
       <c r="AI16" s="8"/>
       <c r="AJ16" s="6" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="AK16" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3996,7 +3993,7 @@
         <v>411</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
@@ -4018,16 +4015,16 @@
       <c r="V17" s="8"/>
       <c r="W17" s="8"/>
       <c r="X17" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="Y17" s="8" t="s">
         <v>463</v>
-      </c>
-      <c r="Y17" s="8" t="s">
-        <v>464</v>
       </c>
       <c r="Z17" s="8"/>
       <c r="AA17" s="8"/>
       <c r="AB17" s="8"/>
       <c r="AC17" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="AD17" s="8" t="s">
         <v>276</v>
@@ -4103,7 +4100,7 @@
       <c r="AH18" s="8"/>
       <c r="AI18" s="8"/>
       <c r="AJ18" s="6" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="AK18" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4210,7 +4207,7 @@
         <v>10</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
@@ -4433,7 +4430,7 @@
         <v>266</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
@@ -4524,7 +4521,7 @@
         <v>382</v>
       </c>
       <c r="S24" s="8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="T24" s="8"/>
       <c r="U24" s="8"/>
@@ -4691,7 +4688,7 @@
       <c r="AH26" s="8"/>
       <c r="AI26" s="8"/>
       <c r="AJ26" s="6" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="AK26" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4770,7 +4767,7 @@
       <c r="AH27" s="8"/>
       <c r="AI27" s="8"/>
       <c r="AJ27" s="6" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="AK27" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4847,7 +4844,7 @@
       <c r="AH28" s="8"/>
       <c r="AI28" s="8"/>
       <c r="AJ28" s="6" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AK28" s="7" t="str">
         <f t="shared" si="2"/>
@@ -5033,7 +5030,7 @@
         <v>268</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
@@ -5204,7 +5201,7 @@
       </c>
       <c r="S33" s="8"/>
       <c r="T33" s="8" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="U33" s="8"/>
       <c r="V33" s="8"/>
@@ -5299,7 +5296,7 @@
       <c r="AH34" s="8"/>
       <c r="AI34" s="8"/>
       <c r="AJ34" s="6" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="AK34" s="7" t="str">
         <f t="shared" ref="AK34:AK70" si="5">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C34&amp;" "&amp;B34)," ","-"))&amp;".jpg"</f>
@@ -5350,17 +5347,17 @@
         <v>14</v>
       </c>
       <c r="R35" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="S35" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="T35" s="8"/>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
       <c r="W35" s="8"/>
       <c r="X35" s="8" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="Y35" s="8"/>
       <c r="Z35" s="8"/>
@@ -5412,7 +5409,7 @@
         <v>243</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
@@ -5502,10 +5499,10 @@
         <v>16</v>
       </c>
       <c r="R37" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S37" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="T37" s="8"/>
       <c r="U37" s="8"/>
@@ -5901,7 +5898,7 @@
       <c r="AH42" s="8"/>
       <c r="AI42" s="8"/>
       <c r="AJ42" s="6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="AK42" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6112,7 +6109,7 @@
       <c r="AH45" s="8"/>
       <c r="AI45" s="8"/>
       <c r="AJ45" s="6" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="AK45" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6148,7 +6145,7 @@
         <v>269</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
@@ -6239,14 +6236,14 @@
         <v>434</v>
       </c>
       <c r="S47" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="T47" s="8"/>
       <c r="U47" s="8"/>
       <c r="V47" s="8"/>
       <c r="W47" s="8"/>
       <c r="X47" s="8" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="Y47" s="8"/>
       <c r="Z47" s="8"/>
@@ -6262,7 +6259,7 @@
       <c r="AH47" s="8"/>
       <c r="AI47" s="8"/>
       <c r="AJ47" s="6" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="AK47" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6446,7 +6443,7 @@
         <v>266</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="6"/>
@@ -6694,7 +6691,7 @@
       <c r="V53" s="8"/>
       <c r="W53" s="8"/>
       <c r="X53" s="8" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="Y53" s="8"/>
       <c r="Z53" s="8"/>
@@ -6711,10 +6708,10 @@
       <c r="AG53" s="8"/>
       <c r="AH53" s="8"/>
       <c r="AI53" s="8" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="AJ53" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="AK53" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6866,7 +6863,7 @@
       <c r="AH55" s="8"/>
       <c r="AI55" s="8"/>
       <c r="AJ55" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="AK55" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6924,7 +6921,7 @@
         <v>434</v>
       </c>
       <c r="S56" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="T56" s="8"/>
       <c r="U56" s="8"/>
@@ -7361,10 +7358,10 @@
         <v>16</v>
       </c>
       <c r="R62" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S62" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="T62" s="8"/>
       <c r="U62" s="8"/>
@@ -7419,7 +7416,7 @@
         <v>243</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="J63" s="6"/>
       <c r="K63" s="6"/>
@@ -7460,7 +7457,7 @@
       <c r="AH63" s="8"/>
       <c r="AI63" s="8"/>
       <c r="AJ63" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="AK63" s="7" t="str">
         <f t="shared" si="5"/>
@@ -7535,7 +7532,7 @@
       <c r="AH64" s="8"/>
       <c r="AI64" s="8"/>
       <c r="AJ64" s="6" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="AK64" s="7" t="str">
         <f t="shared" si="5"/>
@@ -7598,7 +7595,7 @@
       <c r="V65" s="8"/>
       <c r="W65" s="8"/>
       <c r="X65" s="8" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="Y65" s="8"/>
       <c r="Z65" s="8"/>
@@ -7636,12 +7633,12 @@
         <v>222</v>
       </c>
       <c r="E66" s="7" t="str">
-        <f t="shared" ref="E66:E97" si="6">IF(D66="","",LEFT(TRIM(D66),1)&amp;".")</f>
+        <f t="shared" ref="E66:E71" si="6">IF(D66="","",LEFT(TRIM(D66),1)&amp;".")</f>
         <v>T.</v>
       </c>
       <c r="F66" s="7"/>
       <c r="G66" s="7" t="str">
-        <f t="shared" ref="G66:G97" si="7">TRIM(_xlfn.TEXTJOIN(" ",TRUE,C66,IF(E66&lt;&gt;"",IF(RIGHT(E66,1)=".",E66,E66&amp;"."),D66),B66,F66))</f>
+        <f t="shared" ref="G66:G70" si="7">TRIM(_xlfn.TEXTJOIN(" ",TRUE,C66,IF(E66&lt;&gt;"",IF(RIGHT(E66,1)=".",E66,E66&amp;"."),D66),B66,F66))</f>
         <v>Bella Arquine T. Samontañez</v>
       </c>
       <c r="H66" s="7" t="s">
@@ -7667,10 +7664,10 @@
         <v>16</v>
       </c>
       <c r="R66" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="S66" s="8" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="T66" s="8"/>
       <c r="U66" s="8"/>
@@ -7841,7 +7838,7 @@
       <c r="AH68" s="8"/>
       <c r="AI68" s="8"/>
       <c r="AJ68" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="AK68" s="7" t="str">
         <f t="shared" si="5"/>

</xml_diff>

<commit_message>
Update organization page group layout
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF7F748-A227-49A9-A125-900F3BE35132}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41A45A3-9911-49B0-87C1-CCDF7DF5E568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="517">
   <si>
     <t>order</t>
   </si>
@@ -1568,6 +1568,24 @@
   </si>
   <si>
     <t>7th Grade - Grade Leader</t>
+  </si>
+  <si>
+    <t>Hairdressing NCII</t>
+  </si>
+  <si>
+    <t>glendale.orocay@deped.gov.ph</t>
+  </si>
+  <si>
+    <t>"I believe every learner can succeed with proper guidance, encouragement, and opportunities to grow. As a Hairdressing Teacher, I help students build skills, confidence, and creativity for lifelong success."</t>
+  </si>
+  <si>
+    <t>Guidance Designate for Junior High School</t>
+  </si>
+  <si>
+    <t>carolyn.delosreyes002@deped.gov.ph</t>
+  </si>
+  <si>
+    <t>"My teaching philosophy us that every learner is capable of growth when given support, respect, and meaningful learning experiences. I believe teaching should be student-centered, where learners actively construct understanding through engagement, critical thinking, and real-life connections. My role is to guide, motivate, and create an inclusive environment where students feel safe to ask questions, make mistakes, and improve continuously."</t>
   </si>
 </sst>
 </file>
@@ -5156,7 +5174,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:38">
+    <row r="33" spans="1:38" ht="218.4">
       <c r="A33" s="7">
         <v>29</v>
       </c>
@@ -5179,10 +5197,10 @@
         <v>Carolyn L. Delos Reyes</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>368</v>
+        <v>514</v>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
@@ -5219,8 +5237,12 @@
       <c r="AF33" s="8"/>
       <c r="AG33" s="8"/>
       <c r="AH33" s="8"/>
-      <c r="AI33" s="8"/>
-      <c r="AJ33" s="6"/>
+      <c r="AI33" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="AJ33" s="6" t="s">
+        <v>516</v>
+      </c>
       <c r="AK33" s="7" t="str">
         <f t="shared" si="2"/>
         <v>/personnel/carolyn-delos-reyes.jpg</v>
@@ -6873,7 +6895,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:38">
+    <row r="56" spans="1:38" ht="100.8">
       <c r="A56" s="7">
         <v>51</v>
       </c>
@@ -6927,7 +6949,9 @@
       <c r="U56" s="8"/>
       <c r="V56" s="8"/>
       <c r="W56" s="8"/>
-      <c r="X56" s="8"/>
+      <c r="X56" s="8" t="s">
+        <v>511</v>
+      </c>
       <c r="Y56" s="8"/>
       <c r="Z56" s="8"/>
       <c r="AA56" s="8"/>
@@ -6940,8 +6964,12 @@
       <c r="AF56" s="8"/>
       <c r="AG56" s="8"/>
       <c r="AH56" s="8"/>
-      <c r="AI56" s="8"/>
-      <c r="AJ56" s="6"/>
+      <c r="AI56" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="AJ56" s="6" t="s">
+        <v>513</v>
+      </c>
       <c r="AK56" s="7" t="str">
         <f t="shared" si="5"/>
         <v>/personnel/glendale-orocay.jpg</v>
@@ -8058,31 +8086,31 @@
           <x14:formula1>
             <xm:f>Dropdown_Lists!$A$2:$A$6</xm:f>
           </x14:formula1>
-          <xm:sqref>P2:P70</xm:sqref>
+          <xm:sqref>P57:P70 P2:P32 P34:P55</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{909FCDCA-C40C-4807-A52A-02A68E381F21}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$B$2:$B$35</xm:f>
           </x14:formula1>
-          <xm:sqref>H2:H70</xm:sqref>
+          <xm:sqref>H57:H70 H2:H32 H34:H55</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$G$2:$G$5</xm:f>
           </x14:formula1>
-          <xm:sqref>AL2:AL71</xm:sqref>
+          <xm:sqref>AL57:AL71 AL2:AL32 AL34:AL55</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{70D54F6E-2A67-40F0-92CA-B6E53F44843D}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$D$2:$D$61</xm:f>
           </x14:formula1>
-          <xm:sqref>AD2:AD71</xm:sqref>
+          <xm:sqref>AD57:AD71 AD2:AD32 AD34:AD55</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7834D497-9733-4178-89DF-4B7895726F53}">
           <x14:formula1>
             <xm:f>Dropdown_Lists!$E$2:$E$60</xm:f>
           </x14:formula1>
-          <xm:sqref>AE2:AE71</xm:sqref>
+          <xm:sqref>AE57:AE71 AE2:AE32 AE34:AE55</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Update enrollment guide layout and contact icons
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41A45A3-9911-49B0-87C1-CCDF7DF5E568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E923B6-4374-43B9-99D9-399F4BF7BA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="517">
   <si>
     <t>order</t>
   </si>
@@ -1153,18 +1153,6 @@
     <t>Job Order/Support Personnel</t>
   </si>
   <si>
-    <t>Cabs</t>
-  </si>
-  <si>
-    <t>Mans</t>
-  </si>
-  <si>
-    <t>Luis</t>
-  </si>
-  <si>
-    <t>Luie</t>
-  </si>
-  <si>
     <t>Senior High School In-Charge</t>
   </si>
   <si>
@@ -1586,6 +1574,18 @@
   </si>
   <si>
     <t>"My teaching philosophy us that every learner is capable of growth when given support, respect, and meaningful learning experiences. I believe teaching should be student-centered, where learners actively construct understanding through engagement, critical thinking, and real-life connections. My role is to guide, motivate, and create an inclusive environment where students feel safe to ask questions, make mistakes, and improve continuously."</t>
+  </si>
+  <si>
+    <t>Caballero</t>
+  </si>
+  <si>
+    <t>Rocer</t>
+  </si>
+  <si>
+    <t>Rellon</t>
+  </si>
+  <si>
+    <t>Severino</t>
   </si>
 </sst>
 </file>
@@ -2650,10 +2650,10 @@
         <v>323</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>324</v>
@@ -2677,37 +2677,37 @@
         <v>4</v>
       </c>
       <c r="S1" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="T1" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="U1" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="V1" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="W1" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="X1" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="Y1" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="Z1" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="AA1" s="5" t="s">
         <v>419</v>
       </c>
-      <c r="T1" s="5" t="s">
-        <v>467</v>
-      </c>
-      <c r="U1" s="5" t="s">
-        <v>468</v>
-      </c>
-      <c r="V1" s="5" t="s">
-        <v>469</v>
-      </c>
-      <c r="W1" s="5" t="s">
-        <v>470</v>
-      </c>
-      <c r="X1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>420</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>421</v>
-      </c>
-      <c r="Z1" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="AA1" s="5" t="s">
-        <v>423</v>
-      </c>
-      <c r="AB1" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="AC1" s="5" t="s">
-        <v>425</v>
       </c>
       <c r="AD1" s="5" t="s">
         <v>359</v>
@@ -2725,10 +2725,10 @@
         <v>362</v>
       </c>
       <c r="AI1" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
         <v>473</v>
-      </c>
-      <c r="AJ1" s="5" t="s">
-        <v>477</v>
       </c>
       <c r="AK1" s="5" t="s">
         <v>5</v>
@@ -2763,12 +2763,12 @@
         <v>10</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="7" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
       <c r="M2" s="7"/>
       <c r="N2" s="7"/>
@@ -2790,7 +2790,7 @@
       <c r="V2" s="8"/>
       <c r="W2" s="8"/>
       <c r="X2" s="8" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="Y2" s="8"/>
       <c r="Z2" s="8"/>
@@ -2810,7 +2810,7 @@
       <c r="AH2" s="8"/>
       <c r="AI2" s="8"/>
       <c r="AJ2" s="6" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="AK2" s="7" t="str">
         <f t="shared" ref="AK2:AK33" si="2">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C2&amp;" "&amp;B2)," ","-"))&amp;".jpg"</f>
@@ -2852,7 +2852,7 @@
         <v>352</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
@@ -2875,18 +2875,18 @@
       <c r="V3" s="8"/>
       <c r="W3" s="8"/>
       <c r="X3" s="8" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="Y3" s="8" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="Z3" s="8" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
       <c r="AA3" s="8"/>
       <c r="AB3" s="8"/>
       <c r="AC3" s="8" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="AD3" s="8" t="s">
         <v>276</v>
@@ -2931,12 +2931,12 @@
         <v>240</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="7" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="M4" s="7"/>
       <c r="N4" s="7"/>
@@ -2958,7 +2958,7 @@
       <c r="V4" s="8"/>
       <c r="W4" s="8"/>
       <c r="X4" s="8" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
       <c r="Y4" s="8"/>
       <c r="Z4" s="8"/>
@@ -2976,7 +2976,7 @@
       <c r="AH4" s="8"/>
       <c r="AI4" s="8"/>
       <c r="AJ4" s="6" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="AK4" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3018,13 +3018,13 @@
         <v>354</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
@@ -3045,10 +3045,10 @@
       <c r="V5" s="8"/>
       <c r="W5" s="8"/>
       <c r="X5" s="8" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="Y5" s="8" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="Z5" s="8"/>
       <c r="AA5" s="8"/>
@@ -3105,7 +3105,7 @@
         <v>355</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
@@ -3118,20 +3118,20 @@
         <v>14</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="S6" s="8" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="T6" s="8"/>
       <c r="U6" s="8"/>
       <c r="V6" s="8"/>
       <c r="W6" s="8"/>
       <c r="X6" s="8" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="Y6" s="8" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="Z6" s="8"/>
       <c r="AA6" s="8"/>
@@ -3188,13 +3188,13 @@
         <v>353</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
@@ -3205,17 +3205,17 @@
         <v>14</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="S7" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
       <c r="V7" s="8"/>
       <c r="W7" s="8"/>
       <c r="X7" s="8" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
       <c r="Y7" s="8"/>
       <c r="Z7" s="8"/>
@@ -3233,7 +3233,7 @@
       <c r="AH7" s="8"/>
       <c r="AI7" s="8"/>
       <c r="AJ7" s="6" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="AK7" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3282,7 +3282,7 @@
         <v>7</v>
       </c>
       <c r="R8" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S8" s="8"/>
       <c r="T8" s="8"/>
@@ -3338,7 +3338,7 @@
         <v>268</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6"/>
@@ -3353,10 +3353,10 @@
         <v>370</v>
       </c>
       <c r="R9" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S9" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="T9" s="8"/>
       <c r="U9" s="8"/>
@@ -3411,12 +3411,12 @@
         <v>243</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
       <c r="L10" s="7" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
@@ -3428,17 +3428,17 @@
         <v>16</v>
       </c>
       <c r="R10" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="S10" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="T10" s="8"/>
       <c r="U10" s="8"/>
       <c r="V10" s="8"/>
       <c r="W10" s="8"/>
       <c r="X10" s="8" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
       <c r="Y10" s="8"/>
       <c r="Z10" s="8"/>
@@ -3496,13 +3496,13 @@
         <v>354</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
@@ -3513,17 +3513,17 @@
         <v>14</v>
       </c>
       <c r="R11" s="8" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="S11" s="8" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="T11" s="8"/>
       <c r="U11" s="8"/>
       <c r="V11" s="8"/>
       <c r="W11" s="8"/>
       <c r="X11" s="8" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
       <c r="Y11" s="8"/>
       <c r="Z11" s="8"/>
@@ -3581,10 +3581,10 @@
         <v>352</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
@@ -3606,7 +3606,7 @@
       <c r="V12" s="8"/>
       <c r="W12" s="8"/>
       <c r="X12" s="8" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
       <c r="Y12" s="8"/>
       <c r="Z12" s="8"/>
@@ -3624,7 +3624,7 @@
       <c r="AH12" s="8"/>
       <c r="AI12" s="8"/>
       <c r="AJ12" s="6" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="AK12" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3666,16 +3666,16 @@
         <v>356</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="O13" s="7"/>
       <c r="P13" s="8" t="s">
@@ -3695,16 +3695,16 @@
       <c r="V13" s="8"/>
       <c r="W13" s="8"/>
       <c r="X13" s="8" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
       <c r="Y13" s="8" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="Z13" s="8"/>
       <c r="AA13" s="8"/>
       <c r="AB13" s="8"/>
       <c r="AC13" s="8" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="AD13" s="8" t="s">
         <v>276</v>
@@ -3715,7 +3715,7 @@
       <c r="AH13" s="8"/>
       <c r="AI13" s="8"/>
       <c r="AJ13" s="6" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="AK13" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3751,7 +3751,7 @@
         <v>12</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
@@ -3776,7 +3776,7 @@
       <c r="V14" s="8"/>
       <c r="W14" s="8"/>
       <c r="X14" s="8" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="Y14" s="8"/>
       <c r="Z14" s="8"/>
@@ -3834,10 +3834,10 @@
         <v>351</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="M15" s="7"/>
       <c r="N15" s="7"/>
@@ -3859,16 +3859,16 @@
       <c r="V15" s="8"/>
       <c r="W15" s="8"/>
       <c r="X15" s="8" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
       <c r="Y15" s="8" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
       <c r="Z15" s="8"/>
       <c r="AA15" s="8"/>
       <c r="AB15" s="8"/>
       <c r="AC15" s="8" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="AD15" s="8" t="s">
         <v>276</v>
@@ -3879,7 +3879,7 @@
       <c r="AH15" s="8"/>
       <c r="AI15" s="8"/>
       <c r="AJ15" s="6" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="AK15" s="7" t="str">
         <f t="shared" si="2"/>
@@ -3920,13 +3920,13 @@
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
       <c r="L16" s="7" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
       <c r="M16" s="7" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="N16" s="7" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="O16" s="7"/>
       <c r="P16" s="8" t="s">
@@ -3946,10 +3946,10 @@
       <c r="V16" s="8"/>
       <c r="W16" s="8"/>
       <c r="X16" s="8" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="Y16" s="8" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="Z16" s="8"/>
       <c r="AA16" s="8"/>
@@ -3968,7 +3968,7 @@
       <c r="AH16" s="8"/>
       <c r="AI16" s="8"/>
       <c r="AJ16" s="6" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="AK16" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4008,10 +4008,10 @@
         <v>351</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
@@ -4033,16 +4033,16 @@
       <c r="V17" s="8"/>
       <c r="W17" s="8"/>
       <c r="X17" s="8" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="Y17" s="8" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="Z17" s="8"/>
       <c r="AA17" s="8"/>
       <c r="AB17" s="8"/>
       <c r="AC17" s="8" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="AD17" s="8" t="s">
         <v>276</v>
@@ -4118,7 +4118,7 @@
       <c r="AH18" s="8"/>
       <c r="AI18" s="8"/>
       <c r="AJ18" s="6" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="AK18" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4154,7 +4154,7 @@
         <v>259</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
@@ -4169,7 +4169,7 @@
         <v>14</v>
       </c>
       <c r="R19" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S19" s="8" t="s">
         <v>7</v>
@@ -4225,7 +4225,7 @@
         <v>10</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
@@ -4304,7 +4304,7 @@
         <v>353</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="L21" s="7"/>
       <c r="M21" s="7"/>
@@ -4381,7 +4381,7 @@
         <v>354</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="L22" s="7"/>
       <c r="M22" s="7"/>
@@ -4427,28 +4427,26 @@
         <v>68</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>372</v>
+        <v>513</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>375</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>197</v>
-      </c>
+        <v>514</v>
+      </c>
+      <c r="D23" s="7"/>
       <c r="E23" s="7" t="str">
         <f t="shared" si="0"/>
-        <v>B.</v>
+        <v/>
       </c>
       <c r="F23" s="7"/>
       <c r="G23" s="7" t="str">
         <f t="shared" si="1"/>
-        <v>Luie B. Cabs</v>
+        <v>Rocer Caballero</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>266</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
@@ -4463,10 +4461,10 @@
         <v>370</v>
       </c>
       <c r="R23" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S23" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="T23" s="8"/>
       <c r="U23" s="8"/>
@@ -4489,7 +4487,7 @@
       <c r="AJ23" s="6"/>
       <c r="AK23" s="7" t="str">
         <f t="shared" si="2"/>
-        <v>/personnel/luie-cabs.jpg</v>
+        <v>/personnel/rocer-caballero.jpg</v>
       </c>
       <c r="AL23" s="8" t="s">
         <v>9</v>
@@ -4536,10 +4534,10 @@
         <v>7</v>
       </c>
       <c r="R24" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S24" s="8" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="T24" s="8"/>
       <c r="U24" s="8"/>
@@ -4594,7 +4592,7 @@
         <v>248</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
@@ -4667,7 +4665,7 @@
         <v>15</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
       <c r="J26" s="6"/>
       <c r="K26" s="6"/>
@@ -4706,7 +4704,7 @@
       <c r="AH26" s="8"/>
       <c r="AI26" s="8"/>
       <c r="AJ26" s="6" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="AK26" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4748,7 +4746,7 @@
         <v>351</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="L27" s="7"/>
       <c r="M27" s="7"/>
@@ -4785,7 +4783,7 @@
       <c r="AH27" s="8"/>
       <c r="AI27" s="8"/>
       <c r="AJ27" s="6" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="AK27" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4825,7 +4823,7 @@
         <v>353</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="L28" s="7"/>
       <c r="M28" s="7"/>
@@ -4862,7 +4860,7 @@
       <c r="AH28" s="8"/>
       <c r="AI28" s="8"/>
       <c r="AJ28" s="6" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="AK28" s="7" t="str">
         <f t="shared" si="2"/>
@@ -4898,7 +4896,7 @@
         <v>259</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
@@ -4913,7 +4911,7 @@
         <v>16</v>
       </c>
       <c r="R29" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S29" s="8" t="s">
         <v>7</v>
@@ -4977,7 +4975,7 @@
         <v>354</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
       <c r="L30" s="7"/>
       <c r="M30" s="7"/>
@@ -5048,7 +5046,7 @@
         <v>268</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6"/>
@@ -5063,10 +5061,10 @@
         <v>370</v>
       </c>
       <c r="R31" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S31" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="T31" s="8"/>
       <c r="U31" s="8"/>
@@ -5129,7 +5127,7 @@
         <v>355</v>
       </c>
       <c r="K32" s="6" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="L32" s="7"/>
       <c r="M32" s="7"/>
@@ -5200,7 +5198,7 @@
         <v>15</v>
       </c>
       <c r="I33" s="6" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6"/>
@@ -5219,7 +5217,7 @@
       </c>
       <c r="S33" s="8"/>
       <c r="T33" s="8" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="U33" s="8"/>
       <c r="V33" s="8"/>
@@ -5238,10 +5236,10 @@
       <c r="AG33" s="8"/>
       <c r="AH33" s="8"/>
       <c r="AI33" s="8" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="AJ33" s="6" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="AK33" s="7" t="str">
         <f t="shared" si="2"/>
@@ -5318,7 +5316,7 @@
       <c r="AH34" s="8"/>
       <c r="AI34" s="8"/>
       <c r="AJ34" s="6" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="AK34" s="7" t="str">
         <f t="shared" ref="AK34:AK70" si="5">"/personnel/"&amp;LOWER(SUBSTITUTE(TRIM(C34&amp;" "&amp;B34)," ","-"))&amp;".jpg"</f>
@@ -5369,17 +5367,17 @@
         <v>14</v>
       </c>
       <c r="R35" s="8" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="S35" s="8" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="T35" s="8"/>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
       <c r="W35" s="8"/>
       <c r="X35" s="8" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
       <c r="Y35" s="8"/>
       <c r="Z35" s="8"/>
@@ -5431,7 +5429,7 @@
         <v>243</v>
       </c>
       <c r="I36" s="6" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="J36" s="6"/>
       <c r="K36" s="6"/>
@@ -5506,7 +5504,7 @@
         <v>12</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
       <c r="J37" s="6"/>
       <c r="K37" s="6"/>
@@ -5521,10 +5519,10 @@
         <v>16</v>
       </c>
       <c r="R37" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="S37" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="T37" s="8"/>
       <c r="U37" s="8"/>
@@ -5585,7 +5583,7 @@
         <v>352</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
@@ -5660,7 +5658,7 @@
         <v>352</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
       <c r="L39" s="7"/>
       <c r="M39" s="7"/>
@@ -5806,7 +5804,7 @@
         <v>351</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
       <c r="L41" s="7"/>
       <c r="M41" s="7"/>
@@ -5883,7 +5881,7 @@
         <v>354</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
@@ -5920,7 +5918,7 @@
       <c r="AH42" s="8"/>
       <c r="AI42" s="8"/>
       <c r="AJ42" s="6" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="AK42" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6131,7 +6129,7 @@
       <c r="AH45" s="8"/>
       <c r="AI45" s="8"/>
       <c r="AJ45" s="6" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="AK45" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6167,7 +6165,7 @@
         <v>269</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
@@ -6236,7 +6234,7 @@
         <v>249</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
       <c r="J47" s="6"/>
       <c r="K47" s="6"/>
@@ -6255,17 +6253,17 @@
         <v>14</v>
       </c>
       <c r="R47" s="8" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="S47" s="8" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="T47" s="8"/>
       <c r="U47" s="8"/>
       <c r="V47" s="8"/>
       <c r="W47" s="8"/>
       <c r="X47" s="8" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
       <c r="Y47" s="8"/>
       <c r="Z47" s="8"/>
@@ -6281,7 +6279,7 @@
       <c r="AH47" s="8"/>
       <c r="AI47" s="8"/>
       <c r="AJ47" s="6" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="AK47" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6394,7 +6392,7 @@
         <v>353</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
@@ -6444,28 +6442,26 @@
         <v>69</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>373</v>
+        <v>515</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>374</v>
-      </c>
-      <c r="D50" s="7" t="s">
-        <v>197</v>
-      </c>
+        <v>516</v>
+      </c>
+      <c r="D50" s="7"/>
       <c r="E50" s="7" t="str">
         <f t="shared" si="3"/>
-        <v>B.</v>
+        <v/>
       </c>
       <c r="F50" s="7"/>
       <c r="G50" s="7" t="str">
         <f t="shared" si="4"/>
-        <v>Luis B. Mans</v>
+        <v>Severino Rellon</v>
       </c>
       <c r="H50" s="7" t="s">
         <v>266</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="6"/>
@@ -6480,10 +6476,10 @@
         <v>370</v>
       </c>
       <c r="R50" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S50" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="T50" s="8"/>
       <c r="U50" s="8"/>
@@ -6506,7 +6502,7 @@
       <c r="AJ50" s="6"/>
       <c r="AK50" s="7" t="str">
         <f t="shared" si="5"/>
-        <v>/personnel/luis-mans.jpg</v>
+        <v>/personnel/severino-rellon.jpg</v>
       </c>
       <c r="AL50" s="8" t="s">
         <v>9</v>
@@ -6613,7 +6609,7 @@
         <v>351</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
@@ -6690,7 +6686,7 @@
         <v>352</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
@@ -6713,7 +6709,7 @@
       <c r="V53" s="8"/>
       <c r="W53" s="8"/>
       <c r="X53" s="8" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
       <c r="Y53" s="8"/>
       <c r="Z53" s="8"/>
@@ -6730,10 +6726,10 @@
       <c r="AG53" s="8"/>
       <c r="AH53" s="8"/>
       <c r="AI53" s="8" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="AJ53" s="6" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="AK53" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6775,7 +6771,7 @@
         <v>351</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
@@ -6852,7 +6848,7 @@
         <v>354</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
@@ -6885,7 +6881,7 @@
       <c r="AH55" s="8"/>
       <c r="AI55" s="8"/>
       <c r="AJ55" s="6" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="AK55" s="7" t="str">
         <f t="shared" si="5"/>
@@ -6927,7 +6923,7 @@
         <v>356</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="L56" s="7"/>
       <c r="M56" s="7"/>
@@ -6940,17 +6936,17 @@
         <v>14</v>
       </c>
       <c r="R56" s="8" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="S56" s="8" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
       <c r="T56" s="8"/>
       <c r="U56" s="8"/>
       <c r="V56" s="8"/>
       <c r="W56" s="8"/>
       <c r="X56" s="8" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="Y56" s="8"/>
       <c r="Z56" s="8"/>
@@ -6965,10 +6961,10 @@
       <c r="AG56" s="8"/>
       <c r="AH56" s="8"/>
       <c r="AI56" s="8" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="AJ56" s="6" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="AK56" s="7" t="str">
         <f t="shared" si="5"/>
@@ -7010,7 +7006,7 @@
         <v>355</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
       <c r="L57" s="7"/>
       <c r="M57" s="7"/>
@@ -7096,7 +7092,7 @@
         <v>16</v>
       </c>
       <c r="R58" s="8" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="S58" s="8"/>
       <c r="T58" s="8"/>
@@ -7158,7 +7154,7 @@
         <v>352</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
       <c r="L59" s="7"/>
       <c r="M59" s="7"/>
@@ -7386,10 +7382,10 @@
         <v>16</v>
       </c>
       <c r="R62" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="S62" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="T62" s="8"/>
       <c r="U62" s="8"/>
@@ -7444,7 +7440,7 @@
         <v>243</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="J63" s="6"/>
       <c r="K63" s="6"/>
@@ -7485,7 +7481,7 @@
       <c r="AH63" s="8"/>
       <c r="AI63" s="8"/>
       <c r="AJ63" s="6" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="AK63" s="7" t="str">
         <f t="shared" si="5"/>
@@ -7527,7 +7523,7 @@
         <v>353</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
       <c r="L64" s="7"/>
       <c r="M64" s="7"/>
@@ -7560,7 +7556,7 @@
       <c r="AH64" s="8"/>
       <c r="AI64" s="8"/>
       <c r="AJ64" s="6" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="AK64" s="7" t="str">
         <f t="shared" si="5"/>
@@ -7596,7 +7592,7 @@
         <v>243</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="J65" s="6"/>
       <c r="K65" s="6"/>
@@ -7617,13 +7613,13 @@
         <v>338</v>
       </c>
       <c r="T65" s="8" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="U65" s="8"/>
       <c r="V65" s="8"/>
       <c r="W65" s="8"/>
       <c r="X65" s="8" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
       <c r="Y65" s="8"/>
       <c r="Z65" s="8"/>
@@ -7679,7 +7675,7 @@
         <v>353</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
       <c r="L66" s="7"/>
       <c r="M66" s="7"/>
@@ -7692,10 +7688,10 @@
         <v>16</v>
       </c>
       <c r="R66" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="S66" s="8" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="T66" s="8"/>
       <c r="U66" s="8"/>
@@ -7756,7 +7752,7 @@
         <v>356</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="L67" s="7"/>
       <c r="M67" s="7"/>
@@ -7827,7 +7823,7 @@
         <v>243</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
       <c r="J68" s="6"/>
       <c r="K68" s="6"/>
@@ -7866,7 +7862,7 @@
       <c r="AH68" s="8"/>
       <c r="AI68" s="8"/>
       <c r="AJ68" s="6" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="AK68" s="7" t="str">
         <f t="shared" si="5"/>
@@ -7917,7 +7913,7 @@
         <v>7</v>
       </c>
       <c r="R69" s="8" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
       <c r="S69" s="8" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Update organization personnel card preview
</commit_message>
<xml_diff>
--- a/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
+++ b/public/data/Tabunoc_NHS_Personnel_Roster_Master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\tabunoc-nhs-website\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E923B6-4374-43B9-99D9-399F4BF7BA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88DA8D6D-E7D2-4E4D-9574-C8A55B642AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1077" uniqueCount="518">
   <si>
     <t>order</t>
   </si>
@@ -1586,6 +1586,9 @@
   </si>
   <si>
     <t>Severino</t>
+  </si>
+  <si>
+    <t>Guildance Counselor</t>
   </si>
 </sst>
 </file>
@@ -4519,7 +4522,7 @@
         <v>261</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>363</v>
+        <v>517</v>
       </c>
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>

</xml_diff>